<commit_message>
[看板] 加 V0 重启验收 ✅ / D20e 相位锁定 / D24 开机立方体动画 / D23 V1 内容通路; 达成率 V0 93.0% V1 75.5% V2 66.7%
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/progress/显性目的进度_2026-10-16.xlsx
+++ b/docs/progress/显性目的进度_2026-10-16.xlsx
@@ -8593,16 +8593,16 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>0.975</v>
+        <v>0.9302325581395349</v>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>39/40</t>
+          <t>40/43</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>KR 24/25 + 交付 15/15 — 统一口径：达成率_P = (P 目标已达标的 KR 数 + P 需要的交付里已完成数) ÷ (有 P 目标的 KR 数 + P 需要的交付总数)，P = V0 / V1 / V2。</t>
+          <t>KR 24/25 + 交付 16/18 — 统一口径：达成率_P = (P 目标已达标的 KR 数 + P 需要的交付里已完成数) ÷ (有 P 目标的 KR 数 + P 需要的交付总数)，P = V0 / V1 / V2。</t>
         </is>
       </c>
       <c r="G4" s="8" t="n">
@@ -8625,16 +8625,16 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>0.7959183673469388</v>
+        <v>0.7547169811320755</v>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>39/49</t>
+          <t>40/53</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>KR 16/24 + 交付 23/25 — 只按「必须」项计：KR 全算必须；交付看 deliverables.csv 的「级别」列 (必须/加分)，加分项不进分子分母。</t>
+          <t>KR 16/24 + 交付 24/29 — 只按「必须」项计：KR 全算必须；交付看 deliverables.csv 的「级别」列 (必须/加分)，加分项不进分子分母。</t>
         </is>
       </c>
       <c r="G5" s="8" t="n">
@@ -8657,16 +8657,16 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.6981132075471698</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>37/53</t>
+          <t>38/57</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>KR 14/24 + 交付 23/29 — 交付的"需要"是嵌套的：V0 需要 = 阶段 V0；V1 需要 = V0 + V1准备；V2 需要 = V1 需要 + V2 (阶段列见 deliverables.csv，没填阶段的交付不计)。</t>
+          <t>KR 14/24 + 交付 24/33 — 交付的"需要"是嵌套的：V0 需要 = 阶段 V0；V1 需要 = V0 + V1准备；V2 需要 = V1 需要 + V2 (阶段列见 deliverables.csv，没填阶段的交付不计)。</t>
         </is>
       </c>
       <c r="G6" s="8" t="n">
@@ -8706,13 +8706,13 @@
         <v>46311</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>0.975</v>
+        <v>0.9302</v>
       </c>
       <c r="I8" s="9" t="n">
-        <v>0.7959000000000001</v>
+        <v>0.7547</v>
       </c>
       <c r="J8" s="9" t="n">
-        <v>0.6981000000000001</v>
+        <v>0.6667</v>
       </c>
     </row>
     <row r="9">
@@ -16894,7 +16894,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H56"/>
+  <dimension ref="A1:H60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -16938,7 +16938,7 @@
         <v>46307</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C4" s="6" t="n">
         <v>5</v>
@@ -16952,7 +16952,7 @@
         <v>46308</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C5" s="6" t="n">
         <v>7</v>
@@ -16966,7 +16966,7 @@
         <v>46309</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C6" s="6" t="n">
         <v>8</v>
@@ -16980,7 +16980,7 @@
         <v>46310</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>12</v>
@@ -16994,13 +16994,13 @@
         <v>46311</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9">
@@ -17008,10 +17008,10 @@
         <v>46312</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D9" s="6" t="n"/>
     </row>
@@ -17020,10 +17020,10 @@
         <v>46313</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D10" s="6" t="n"/>
     </row>
@@ -17032,10 +17032,10 @@
         <v>46314</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D11" s="6" t="n"/>
     </row>
@@ -17044,10 +17044,10 @@
         <v>46315</v>
       </c>
       <c r="B12" s="6" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D12" s="6" t="n"/>
     </row>
@@ -17056,10 +17056,10 @@
         <v>46316</v>
       </c>
       <c r="B13" s="6" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C13" s="6" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D13" s="6" t="n"/>
     </row>
@@ -17068,10 +17068,10 @@
         <v>46317</v>
       </c>
       <c r="B14" s="6" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C14" s="6" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D14" s="6" t="n"/>
     </row>
@@ -17080,10 +17080,10 @@
         <v>46318</v>
       </c>
       <c r="B15" s="6" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D15" s="6" t="n"/>
     </row>
@@ -17092,10 +17092,10 @@
         <v>46319</v>
       </c>
       <c r="B16" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="C16" s="6" t="n">
         <v>32</v>
-      </c>
-      <c r="C16" s="6" t="n">
-        <v>28</v>
       </c>
       <c r="D16" s="6" t="n"/>
     </row>
@@ -18339,6 +18339,152 @@
       <c r="H56" s="7" t="inlineStr">
         <is>
           <t>合主线 (task/merge-d21); 上板换档 PASS; 含 voxslice sub01 修复 (主线隐患); 全回归 12 套</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t>V0A</t>
+        </is>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>V0 重启验收 (不插串口: 找回/守护/开机默认/WiFi/推流/稳定 6 项)</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D57" s="6" t="inlineStr">
+        <is>
+          <t>公共</t>
+        </is>
+      </c>
+      <c r="E57" s="17" t="n">
+        <v>46311</v>
+      </c>
+      <c r="F57" s="17" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G57" s="11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H57" s="7" t="inlineStr">
+        <is>
+          <t>dr1v90 v0_accept/accept.sh 88b6eba; 6/6 PASS (progress/v0_accept/)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>D20e</t>
+        </is>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>推流相位锁定 (消 auto 推流 5% 滑格)</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D58" s="6" t="inlineStr">
+        <is>
+          <t>公共</t>
+        </is>
+      </c>
+      <c r="E58" s="17" t="n">
+        <v>46312</v>
+      </c>
+      <c r="F58" s="17" t="n"/>
+      <c r="G58" s="15" t="inlineStr">
+        <is>
+          <t>🔄</t>
+        </is>
+      </c>
+      <c r="H58" s="7" t="inlineStr">
+        <is>
+          <t>task/d20e-phaselock (agent 进行中)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>D24</t>
+        </is>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>开机默认动画 = 立方体动图 (用户 10-16 提)</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D59" s="6" t="inlineStr">
+        <is>
+          <t>公共</t>
+        </is>
+      </c>
+      <c r="E59" s="17" t="n">
+        <v>46312</v>
+      </c>
+      <c r="F59" s="17" t="n"/>
+      <c r="G59" s="24" t="inlineStr">
+        <is>
+          <t>⏸</t>
+        </is>
+      </c>
+      <c r="H59" s="7" t="inlineStr">
+        <is>
+          <t>待用户确认是哪版立方体动画</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>D23</t>
+        </is>
+      </c>
+      <c r="B60" s="7" t="inlineStr">
+        <is>
+          <t>V1 真内容板端通路 (voxslice 加 2260 后端)</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D60" s="6" t="inlineStr">
+        <is>
+          <t>公共</t>
+        </is>
+      </c>
+      <c r="E60" s="17" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F60" s="17" t="n"/>
+      <c r="G60" s="15" t="inlineStr">
+        <is>
+          <t>🔄</t>
+        </is>
+      </c>
+      <c r="H60" s="7" t="inlineStr">
+        <is>
+          <t>task/d23-v1content (agent 进行中)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[看板] D20e/D23 完成, 02 部署 D20e 验收 6/6, KR7.3/D24 合并, DR1M90-03 写卡
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/progress/显性目的进度_2026-10-16.xlsx
+++ b/docs/progress/显性目的进度_2026-10-16.xlsx
@@ -8522,7 +8522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J152"/>
+  <dimension ref="A1:J158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -8593,16 +8593,16 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>0.9302325581395349</v>
+        <v>0.9767441860465116</v>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>40/43</t>
+          <t>42/43</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>KR 24/25 + 交付 16/18 — 统一口径：达成率_P = (P 目标已达标的 KR 数 + P 需要的交付里已完成数) ÷ (有 P 目标的 KR 数 + P 需要的交付总数)，P = V0 / V1 / V2。</t>
+          <t>KR 24/25 + 交付 18/18 — 统一口径：达成率_P = (P 目标已达标的 KR 数 + P 需要的交付里已完成数) ÷ (有 P 目标的 KR 数 + P 需要的交付总数)，P = V0 / V1 / V2。</t>
         </is>
       </c>
       <c r="G4" s="8" t="n">
@@ -8625,16 +8625,16 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>0.7547169811320755</v>
+        <v>0.8113207547169812</v>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>40/53</t>
+          <t>43/53</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>KR 16/24 + 交付 24/29 — 只按「必须」项计：KR 全算必须；交付看 deliverables.csv 的「级别」列 (必须/加分)，加分项不进分子分母。</t>
+          <t>KR 16/24 + 交付 27/29 — 只按「必须」项计：KR 全算必须；交付看 deliverables.csv 的「级别」列 (必须/加分)，加分项不进分子分母。</t>
         </is>
       </c>
       <c r="G5" s="8" t="n">
@@ -8657,16 +8657,16 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.7192982456140351</v>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>38/57</t>
+          <t>41/57</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>KR 14/24 + 交付 24/33 — 交付的"需要"是嵌套的：V0 需要 = 阶段 V0；V1 需要 = V0 + V1准备；V2 需要 = V1 需要 + V2 (阶段列见 deliverables.csv，没填阶段的交付不计)。</t>
+          <t>KR 14/24 + 交付 27/33 — 交付的"需要"是嵌套的：V0 需要 = 阶段 V0；V1 需要 = V0 + V1准备；V2 需要 = V1 需要 + V2 (阶段列见 deliverables.csv，没填阶段的交付不计)。</t>
         </is>
       </c>
       <c r="G6" s="8" t="n">
@@ -8706,13 +8706,13 @@
         <v>46311</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>0.9302</v>
+        <v>0.9767</v>
       </c>
       <c r="I8" s="9" t="n">
-        <v>0.7547</v>
+        <v>0.8113</v>
       </c>
       <c r="J8" s="9" t="n">
-        <v>0.6667</v>
+        <v>0.7193000000000001</v>
       </c>
     </row>
     <row r="9">
@@ -10055,151 +10055,151 @@
     </row>
     <row r="67">
       <c r="A67" s="17" t="n">
-        <v>46310</v>
-      </c>
-      <c r="B67" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46311</v>
+      </c>
+      <c r="B67" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C67" s="7" t="inlineStr">
         <is>
-          <t>KR7.2</t>
+          <t>D24</t>
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>8 h 无人值守长跑 9/9 通过 (重开轮 23:45-07:45; 判读 S1 行数口径误判已改为覆盖时长 fe53bde); V0 出口 ⑥ 达成 → V0 出口 8/8</t>
+          <t>用户: 开机动画就用现在这个 (geo_loop, 含线框立方体), 不换; D26 V2 位流构建放行, 主会话后台跑; 新板定名 DR1M90-03, 拷卡包 card_kit_dr1m90-03 待用户管理员运行 make_card.ps1</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>progress/soak_v0/report.md</t>
+          <t>用户</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="17" t="n">
-        <v>46310</v>
-      </c>
-      <c r="B68" s="6" t="inlineStr">
-        <is>
-          <t>测量</t>
+        <v>46311</v>
+      </c>
+      <c r="B68" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>QoS</t>
+          <t>D23</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>QoS (XMON DDR_S2 QOS_CONFIG=0x0F) 带载对照 (纯切片 30 Hz): 体素流+TCP 迟到 4.12% → 0.000%, CPU memcpy 300 MB/s 91.5% → 0.000%; 2047 32 bit@16.15 rps 完成率无改善 (86/71% vs 无 QoS 91/82%, 带宽上限); 测后寄存器已写回 0</t>
+          <t>V1 显示后端 voxslice --disp 2260 合主线 a41d63b (独立复验 24/0, 合并后回归 d21/d23 过)</t>
         </is>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>~/qos_runs</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="17" t="n">
-        <v>46310</v>
-      </c>
-      <c r="B69" s="6" t="inlineStr">
-        <is>
-          <t>测量</t>
+        <v>46311</v>
+      </c>
+      <c r="B69" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>D16b</t>
+          <t>D20e</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>4x4 分块上板 A/B: 体素流+TCP 迟到 现布局 5.34%/4.45% (漂移 0.89 pp) vs 分块 4.79%, 收益在漂移内 = 无效; 迟到角度随相位漂移, 非几何换行主导。按约定不合主线, 分支 task/d16b-tile 保留</t>
+          <t>推流相位锁定合主线 c80f5fb: 583 rpm 滑格 5.2%→0.19%, 900 rpm 22%→0.12% (p95 = 理想间隔); 代价 延迟 120→170-250 ms (--phaselock off 可回老行为)</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d16b-tile 7936b7e</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="17" t="n">
-        <v>46310</v>
-      </c>
-      <c r="B70" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+        <v>46311</v>
+      </c>
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>部署</t>
         </is>
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>用户定 V0/V1/V2 兼容 300-1200 rpm; 实转 583 rpm PL 只 8 fps (等整圈换帧) → D19 半圈换帧开做 (RTL+voxslice+假转扫速验收)</t>
+          <t>02 卡上 voxslice 换 D20e 版 (ba243d71, 旧版留 .bak-d20e), 重启后 V0 验收 6/6 PASS (推流 1326 帧/90 s, WiFi -44 dBm 丢 0)</t>
         </is>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>用户 10-15</t>
+          <t>progress/v0_accept/accept_1016_d20e.log</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="17" t="n">
-        <v>46310</v>
-      </c>
-      <c r="B71" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+        <v>46311</v>
+      </c>
+      <c r="B71" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C71" s="7" t="inlineStr">
         <is>
-          <t>D20</t>
+          <t>KR7.3/D24</t>
         </is>
       </c>
       <c r="D71" s="7" t="inlineStr">
         <is>
-          <t>用户定流畅显示为一等要求 (V0/V1/V2); D20 阶段 1 流畅度指标+门槛+基线开做 (与 D19 并行)</t>
+          <t>KR7.3 16 位计数回绕修正合主线 (存档无原始计数, 99.84% 无法重算; 38/57 转动行待核); D24 立方体候选合主线, 用户定开机保持 geo_loop</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>用户 10-15</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="17" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>分析</t>
+          <t>硬件</t>
         </is>
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>V1/V2</t>
+          <t>DR1M90-03</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
         <is>
-          <t>转速 300-1200 rpm 纸面预算: 300 rpm 体刷新仅 10 Hz (物理闪烁); V1 358 片只到 ~718 rpm, 1200 需降到 215 片; V2 605 片到 ~1060 rpm; 公共切片核需支持运行时换每圈片数 (见 budget/rpm_range_2026-10-15.md)</t>
+          <t>第二块板: 公司 DLP 拦 TF 卡文件写入 → WSL 做 512 MB 镜像 + host/flash_card_raw.ps1 块级写, 读回 PASS; 等上电按名字找</t>
         </is>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
-          <t>budget/rpm_range_2026-10-15.md</t>
+          <t>D:\card03</t>
         </is>
       </c>
     </row>
@@ -10214,17 +10214,17 @@
       </c>
       <c r="C73" s="7" t="inlineStr">
         <is>
-          <t>KR7.3</t>
+          <t>KR7.2</t>
         </is>
       </c>
       <c r="D73" s="7" t="inlineStr">
         <is>
-          <t>实转 1 h 无故障通过 (583 rpm, QoS 开机默认已上卡 7d301a6); V0 必须项全部达成</t>
+          <t>8 h 无人值守长跑 9/9 通过 (重开轮 23:45-07:45; 判读 S1 行数口径误判已改为覆盖时长 fe53bde); V0 出口 ⑥ 达成 → V0 出口 8/8</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
-          <t>progress/realspin_v0/</t>
+          <t>progress/soak_v0/report.md</t>
         </is>
       </c>
     </row>
@@ -10232,24 +10232,24 @@
       <c r="A74" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B74" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B74" s="6" t="inlineStr">
+        <is>
+          <t>测量</t>
         </is>
       </c>
       <c r="C74" s="7" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>QoS</t>
         </is>
       </c>
       <c r="D74" s="7" t="inlineStr">
         <is>
-          <t>实转换帧仅 10.45/s (583 rpm 整圈换帧限制), 用户感觉卡; D19 半圈换帧 + D20 流畅度门槛处理</t>
+          <t>QoS (XMON DDR_S2 QOS_CONFIG=0x0F) 带载对照 (纯切片 30 Hz): 体素流+TCP 迟到 4.12% → 0.000%, CPU memcpy 300 MB/s 91.5% → 0.000%; 2047 32 bit@16.15 rps 完成率无改善 (86/71% vs 无 QoS 91/82%, 带宽上限); 测后寄存器已写回 0</t>
         </is>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>progress/realspin_v0/</t>
+          <t>~/qos_runs</t>
         </is>
       </c>
     </row>
@@ -10259,22 +10259,22 @@
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>交付</t>
+          <t>测量</t>
         </is>
       </c>
       <c r="C75" s="7" t="inlineStr">
         <is>
-          <t>D20</t>
+          <t>D16b</t>
         </is>
       </c>
       <c r="D75" s="7" t="inlineStr">
         <is>
-          <t>流畅度阶段 1: host/smooth_report.py + 门槛 (软件损失≤3%, 间隔 p99≤2T0, 长停顿≤5‰, 撕裂 0 等, SPEC §12) + voxslice --flip-log; 基线: 8 h 假转软件损失 2.3% 但约每 2 min 一次 2-3 s 无新帧 (主机/链路侧, 板端 PL 无缺口) 判 FAIL; 实转 648 rpm 软件损失 3.5%, 每分钟至少一顿 0.3-1.1 s 判 FAIL。主会话复验中</t>
+          <t>4x4 分块上板 A/B: 体素流+TCP 迟到 现布局 5.34%/4.45% (漂移 0.89 pp) vs 分块 4.79%, 收益在漂移内 = 无效; 迟到角度随相位漂移, 非几何换行主导。按约定不合主线, 分支 task/d16b-tile 保留</t>
         </is>
       </c>
       <c r="E75" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20-smooth 83a5fd7</t>
+          <t>dr1v90 task/d16b-tile 7936b7e</t>
         </is>
       </c>
     </row>
@@ -10282,24 +10282,24 @@
       <c r="A76" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B76" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B76" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C76" s="7" t="inlineStr">
         <is>
-          <t>D14</t>
+          <t>D19</t>
         </is>
       </c>
       <c r="D76" s="7" t="inlineStr">
         <is>
-          <t>更多内容 + 手机网页控制合主线 (用户实转看过); 新克隆回归全过</t>
+          <t>用户定 V0/V1/V2 兼容 300-1200 rpm; 实转 583 rpm PL 只 8 fps (等整圈换帧) → D19 半圈换帧开做 (RTL+voxslice+假转扫速验收)</t>
         </is>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 e215176</t>
+          <t>用户 10-15</t>
         </is>
       </c>
     </row>
@@ -10307,24 +10307,24 @@
       <c r="A77" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B77" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+      <c r="B77" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C77" s="7" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>D20</t>
         </is>
       </c>
       <c r="D77" s="7" t="inlineStr">
         <is>
-          <t>半圈换帧: 换网格上限 1×→2×转速 (583 rpm 9.7→~19/s), 慢转均匀丢帧; 16/32 档位流时序收住 (REV 0x20471019/1A); 转速窗口 300-1200; 离线 16/16 + 仿真 21+5 + pls2047 32/32。主会话复验+上板假转扫点中</t>
+          <t>用户定流畅显示为一等要求 (V0/V1/V2); D20 阶段 1 流畅度指标+门槛+基线开做 (与 D19 并行)</t>
         </is>
       </c>
       <c r="E77" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d19-halfrev 1beafa6</t>
+          <t>用户 10-15</t>
         </is>
       </c>
     </row>
@@ -10334,22 +10334,22 @@
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>交付</t>
+          <t>分析</t>
         </is>
       </c>
       <c r="C78" s="7" t="inlineStr">
         <is>
-          <t>D20b</t>
+          <t>V1/V2</t>
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr">
         <is>
-          <t>画面模拟器 host/pov_view.py (按视觉暂留合成人眼所见, 并排对比): 整圈换帧 9.8/s 跳 51 帧; 半圈 15/s 但 51/103 ms 交替 (内容 15 fps 与半圈节拍不齐 → D20 阶段 3 内容帧率跟转速); 300 rpm 闪烁; 停推冻结后跳帧。示例 gif 在 dr1v90/_work/d20b/d20_smooth/sim_out/; 复验 PASS</t>
+          <t>转速 300-1200 rpm 纸面预算: 300 rpm 体刷新仅 10 Hz (物理闪烁); V1 358 片只到 ~718 rpm, 1200 需降到 215 片; V2 605 片到 ~1060 rpm; 公共切片核需支持运行时换每圈片数 (见 budget/rpm_range_2026-10-15.md)</t>
         </is>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20b-sim 9081f62</t>
+          <t>budget/rpm_range_2026-10-15.md</t>
         </is>
       </c>
     </row>
@@ -10357,24 +10357,24 @@
       <c r="A79" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B79" s="6" t="inlineStr">
-        <is>
-          <t>验证</t>
+      <c r="B79" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C79" s="7" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>KR7.3</t>
         </is>
       </c>
       <c r="D79" s="7" t="inlineStr">
         <is>
-          <t>半圈换帧上板假转扫点 PASS: 5/7.5/10/15/20 rps 换网格 9.00/13.56/15.09/15.09/15.08 每秒 (老行为 10 rps 仅 9.00), 完成率 100%, 撕裂 0, 对拍全一致, 超时 0; 卡上开机默认已是 D19 位流 0x20471019。D19+D20+D20b 合并分支全回归中</t>
+          <t>实转 1 h 无故障通过 (583 rpm, QoS 开机默认已上卡 7d301a6); V0 必须项全部达成</t>
         </is>
       </c>
       <c r="E79" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/merge-d19-d20 106364e</t>
+          <t>progress/realspin_v0/</t>
         </is>
       </c>
     </row>
@@ -10382,24 +10382,24 @@
       <c r="A80" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B80" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B80" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C80" s="7" t="inlineStr">
         <is>
-          <t>D19/D20</t>
+          <t>D19</t>
         </is>
       </c>
       <c r="D80" s="7" t="inlineStr">
         <is>
-          <t>半圈换帧 + 流畅度检测 + 画面模拟器合主线; 全回归 10 套 (D18/D13/D19/D20/D20b/color/pls2047/rotor_ops/live_push/重连) 通过; 下一步 D20 阶段 3 (内容帧率跟转速、主机侧停顿诊断) + 实转复核</t>
+          <t>实转换帧仅 10.45/s (583 rpm 整圈换帧限制), 用户感觉卡; D19 半圈换帧 + D20 流畅度门槛处理</t>
         </is>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>progress/realspin_v0/</t>
         </is>
       </c>
     </row>
@@ -10414,17 +10414,17 @@
       </c>
       <c r="C81" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D20</t>
         </is>
       </c>
       <c r="D81" s="7" t="inlineStr">
         <is>
-          <t>每圈片数随转速换档 (V1/V2 到 1200 rpm 的前提): N/PB/LUT 圈边界同步锁存, 回差 5%; V0 2047 人为 142/128 两档仿真逐字节一致、撕裂 0, 假转斜坡升降各 1 次不抖; 16/32 档位流时序收住 (REV 0x20471021/22)。风险: 软件写序时间窗 (可加影子寄存器)。主会话复验中, 诊断跑完后上板</t>
+          <t>流畅度阶段 1: host/smooth_report.py + 门槛 (软件损失≤3%, 间隔 p99≤2T0, 长停顿≤5‰, 撕裂 0 等, SPEC §12) + voxslice --flip-log; 基线: 8 h 假转软件损失 2.3% 但约每 2 min 一次 2-3 s 无新帧 (主机/链路侧, 板端 PL 无缺口) 判 FAIL; 实转 648 rpm 软件损失 3.5%, 每分钟至少一顿 0.3-1.1 s 判 FAIL。主会话复验中</t>
         </is>
       </c>
       <c r="E81" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d21-nband adeba44</t>
+          <t>dr1v90 task/d20-smooth 83a5fd7</t>
         </is>
       </c>
     </row>
@@ -10432,24 +10432,24 @@
       <c r="A82" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B82" s="6" t="inlineStr">
-        <is>
-          <t>根因</t>
+      <c r="B82" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C82" s="7" t="inlineStr">
         <is>
-          <t>D20/D22</t>
+          <t>D14</t>
         </is>
       </c>
       <c r="D82" s="7" t="inlineStr">
         <is>
-          <t>推流每 124.5 s 卡 3 s 的根因 = 长跑脚本的板上对拍 (--pl-verify 1800 ≈ 每 120 s, 每次停 ~3 s), 测试工具自身, 产品默认不开; WiFi 链路同刻 ping 0 丢。WSL/Windows 各 6 min 回放对照: 无周期卡顿, 但有偶发 1-1.7 s ACK 停顿 (每 6 min 1-2 次) = 真实 WiFi 抖动 → D22 WiFi 稳定 (用户 10-15: V0 必须搞定, 不能靠串口)</t>
+          <t>更多内容 + 手机网页控制合主线 (用户实转看过); 新克隆回归全过</t>
         </is>
       </c>
       <c r="E82" s="7" t="inlineStr">
         <is>
-          <t>~/realspin/tcp</t>
+          <t>dr1v90 e215176</t>
         </is>
       </c>
     </row>
@@ -10457,24 +10457,24 @@
       <c r="A83" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B83" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B83" s="6" t="inlineStr">
+        <is>
+          <t>交付</t>
         </is>
       </c>
       <c r="C83" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D19</t>
         </is>
       </c>
       <c r="D83" s="7" t="inlineStr">
         <is>
-          <t>用户: 不插串口也必须永远连得上, 彻底解决 (V0 必须) → D22 四层兜底开做: 服务监护 + 硬件看门狗 + 兜底热点 + 故障注入验收</t>
+          <t>半圈换帧: 换网格上限 1×→2×转速 (583 rpm 9.7→~19/s), 慢转均匀丢帧; 16/32 档位流时序收住 (REV 0x20471019/1A); 转速窗口 300-1200; 离线 16/16 + 仿真 21+5 + pls2047 32/32。主会话复验+上板假转扫点中</t>
         </is>
       </c>
       <c r="E83" s="7" t="inlineStr">
         <is>
-          <t>用户 10-15</t>
+          <t>dr1v90 task/d19-halfrev 1beafa6</t>
         </is>
       </c>
     </row>
@@ -10489,17 +10489,17 @@
       </c>
       <c r="C84" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D20b</t>
         </is>
       </c>
       <c r="D84" s="7" t="inlineStr">
         <is>
-          <t>不插串口永远连得上: povreach 服务监护 + 硬件看门狗 (60 s, 防风暴) + 兜底热点 POV-&lt;板名&gt; (hostapd 静编, 192.168.77.1, 状态页可填 WiFi) + 30 min 无网重启; 失效模式表 16 行; 离线 9/9。排队上板故障演练 (8 项, 含 2 次看门狗复位)</t>
+          <t>画面模拟器 host/pov_view.py (按视觉暂留合成人眼所见, 并排对比): 整圈换帧 9.8/s 跳 51 帧; 半圈 15/s 但 51/103 ms 交替 (内容 15 fps 与半圈节拍不齐 → D20 阶段 3 内容帧率跟转速); 300 rpm 闪烁; 停推冻结后跳帧。示例 gif 在 dr1v90/_work/d20b/d20_smooth/sim_out/; 复验 PASS</t>
         </is>
       </c>
       <c r="E84" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach ee4a55c</t>
+          <t>dr1v90 task/d20b-sim 9081f62</t>
         </is>
       </c>
     </row>
@@ -10509,22 +10509,22 @@
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>交付</t>
+          <t>验证</t>
         </is>
       </c>
       <c r="C85" s="7" t="inlineStr">
         <is>
-          <t>D20c</t>
+          <t>D19</t>
         </is>
       </c>
       <c r="D85" s="7" t="inlineStr">
         <is>
-          <t>内容帧率跟转速 voxlive --fps auto: 583 rpm 换帧间隔 std 23.4→0.1-0.9 ms (离线假转)。取舍: 板端默认 (max-fps 15, margin 0.9) 下 583 rpm 均匀但仅 9.7 fps; 板端 max-fps 20 + margin 1.0 → 19.4 fps 均匀。计划 D22 后上板验证 20/1.0 后改开机默认</t>
+          <t>半圈换帧上板假转扫点 PASS: 5/7.5/10/15/20 rps 换网格 9.00/13.56/15.09/15.09/15.08 每秒 (老行为 10 rps 仅 9.00), 完成率 100%, 撕裂 0, 对拍全一致, 超时 0; 卡上开机默认已是 D19 位流 0x20471019。D19+D20+D20b 合并分支全回归中</t>
         </is>
       </c>
       <c r="E85" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20c-fps 338eaaf</t>
+          <t>dr1v90 task/merge-d19-d20 106364e</t>
         </is>
       </c>
     </row>
@@ -10532,24 +10532,24 @@
       <c r="A86" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B86" s="6" t="inlineStr">
-        <is>
-          <t>复验</t>
+      <c r="B86" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C86" s="7" t="inlineStr">
         <is>
-          <t>D20c</t>
+          <t>D19/D20</t>
         </is>
       </c>
       <c r="D86" s="7" t="inlineStr">
         <is>
-          <t>复验 F3 端到端节拍均匀度在主机忙 (D8 大仿真并行) 时不达标: 583 auto std 9.0/5.2 ms (门槛 3/4), 帧率正确; 主机计时抖动敏感, 先不合主线, 待空闲复验 + 上板实测定</t>
+          <t>半圈换帧 + 流畅度检测 + 画面模拟器合主线; 全回归 10 套 (D18/D13/D19/D20/D20b/color/pls2047/rotor_ops/live_push/重连) 通过; 下一步 D20 阶段 3 (内容帧率跟转速、主机侧停顿诊断) + 实转复核</t>
         </is>
       </c>
       <c r="E86" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d20c.v.log</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10564,17 +10564,17 @@
       </c>
       <c r="C87" s="7" t="inlineStr">
         <is>
-          <t>D8</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D87" s="7" t="inlineStr">
         <is>
-          <t>V1 主控↔桥↔2260 联合仿真 0 错 (12/8 bit, 6 链×16 片, 训练锁定, 半圈换帧); 抓出并修 2 个回板必错 bug: 12-bit 字槽格式主控两 beat vs 桥紧排不一致 (改主控 PK12, 上行 195→110 µs/片) + 1 期切片器 NXG 未传 (160 宽按 192 算); 待: 1 期 12-bit 位流重综合 (hclk 余量原 +0.001 ns)</t>
+          <t>每圈片数随转速换档 (V1/V2 到 1200 rpm 的前提): N/PB/LUT 圈边界同步锁存, 回差 5%; V0 2047 人为 142/128 两档仿真逐字节一致、撕裂 0, 假转斜坡升降各 1 次不抖; 16/32 档位流时序收住 (REV 0x20471021/22)。风险: 软件写序时间窗 (可加影子寄存器)。主会话复验中, 诊断跑完后上板</t>
         </is>
       </c>
       <c r="E87" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d8-cosim 85dfe51</t>
+          <t>dr1v90 task/d21-nband adeba44</t>
         </is>
       </c>
     </row>
@@ -10582,24 +10582,24 @@
       <c r="A88" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B88" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B88" s="6" t="inlineStr">
+        <is>
+          <t>根因</t>
         </is>
       </c>
       <c r="C88" s="7" t="inlineStr">
         <is>
-          <t>D8</t>
+          <t>D20/D22</t>
         </is>
       </c>
       <c r="D88" s="7" t="inlineStr">
         <is>
-          <t>V1 联合仿真合主线 (新克隆复验 5/5; 合并回归 sim_v1/pls2047/D18/D19 通过, D19 O4 一次主机忙计时抖动重跑过); V1 回板就绪清单 ⑤ 达成</t>
+          <t>推流每 124.5 s 卡 3 s 的根因 = 长跑脚本的板上对拍 (--pl-verify 1800 ≈ 每 120 s, 每次停 ~3 s), 测试工具自身, 产品默认不开; WiFi 链路同刻 ping 0 丢。WSL/Windows 各 6 min 回放对照: 无周期卡顿, 但有偶发 1-1.7 s ACK 停顿 (每 6 min 1-2 次) = 真实 WiFi 抖动 → D22 WiFi 稳定 (用户 10-15: V0 必须搞定, 不能靠串口)</t>
         </is>
       </c>
       <c r="E88" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>~/realspin/tcp</t>
         </is>
       </c>
     </row>
@@ -10607,24 +10607,24 @@
       <c r="A89" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B89" s="6" t="inlineStr">
-        <is>
-          <t>测量</t>
+      <c r="B89" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C89" s="7" t="inlineStr">
         <is>
-          <t>D22/D20</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D89" s="7" t="inlineStr">
         <is>
-          <t>1 h 产品配置 (无对拍) 推流诊断: 换帧 14.64/s 软件损失 2.4% ✅, 间隔 p99 124 ms ✅, 长停顿 3.7‰ ✅, 最长 495 ms ❌ (门槛 267); PC→板 ping 16781/0 丢; &gt;0.5 s ACK 停顿 46 min 内 4 次 (最长 0.78 s), 同刻 PC→网关 RTT 165-275 ms = PC 侧 WiFi 抖动。周期 3 s 卡顿消失 (确认系对拍)。余项: 0.5-0.8 s 偶发抖动 (播放缓冲 vs 延迟取舍 / PC 有线或专用路由)</t>
+          <t>用户: 不插串口也必须永远连得上, 彻底解决 (V0 必须) → D22 四层兜底开做: 服务监护 + 硬件看门狗 + 兜底热点 + 故障注入验收</t>
         </is>
       </c>
       <c r="E89" s="7" t="inlineStr">
         <is>
-          <t>soak_runs/netdiag_1015_1814</t>
+          <t>用户 10-15</t>
         </is>
       </c>
     </row>
@@ -10632,24 +10632,24 @@
       <c r="A90" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B90" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B90" s="6" t="inlineStr">
+        <is>
+          <t>交付</t>
         </is>
       </c>
       <c r="C90" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D90" s="7" t="inlineStr">
         <is>
-          <t>换档位流 (REV 0x20471021) 上板起步即停摆 (档 0 未换档时写完 47 片后停, 换网格全超时), 仿真全过 → 硅上与仿真不同; D21b 开查根因。另: D21 上板收尾用 m90/up.sh 会让板子没 PL, 已重启回开机默认 (0x20471019 + QoS)</t>
+          <t>不插串口永远连得上: povreach 服务监护 + 硬件看门狗 (60 s, 防风暴) + 兜底热点 POV-&lt;板名&gt; (hostapd 静编, 192.168.77.1, 状态页可填 WiFi) + 30 min 无网重启; 失效模式表 16 行; 离线 9/9。排队上板故障演练 (8 项, 含 2 次看门狗复位)</t>
         </is>
       </c>
       <c r="E90" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d21.board.log</t>
+          <t>dr1v90 task/d22-reach ee4a55c</t>
         </is>
       </c>
     </row>
@@ -10657,24 +10657,24 @@
       <c r="A91" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B91" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B91" s="6" t="inlineStr">
+        <is>
+          <t>交付</t>
         </is>
       </c>
       <c r="C91" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D20c</t>
         </is>
       </c>
       <c r="D91" s="7" t="inlineStr">
         <is>
-          <t>新克隆离线 O6 误 FAIL: hostapd/povreach 二进制 git 模式 644, WSL 本地盘克隆不可执行, qemu 静默拒绝 (板上 autorun 有 chmod, 不受影响); 已修 (git +x, verify chmod), 重跑后自动上板演练</t>
+          <t>内容帧率跟转速 voxlive --fps auto: 583 rpm 换帧间隔 std 23.4→0.1-0.9 ms (离线假转)。取舍: 板端默认 (max-fps 15, margin 0.9) 下 583 rpm 均匀但仅 9.7 fps; 板端 max-fps 20 + margin 1.0 → 19.4 fps 均匀。计划 D22 后上板验证 20/1.0 后改开机默认</t>
         </is>
       </c>
       <c r="E91" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach</t>
+          <t>dr1v90 task/d20c-fps 338eaaf</t>
         </is>
       </c>
     </row>
@@ -10682,24 +10682,24 @@
       <c r="A92" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B92" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B92" s="6" t="inlineStr">
+        <is>
+          <t>复验</t>
         </is>
       </c>
       <c r="C92" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D20c</t>
         </is>
       </c>
       <c r="D92" s="7" t="inlineStr">
         <is>
-          <t>首轮上板演练 9 项误 FAIL = 验收脚本 info() 把板上 board_d22.sh info 的非 0 退出码当失败 (内容正常), settle/wait_healthy 恒失败; 板子本身正常 (装好开机 healthy, povreach managed, 看门狗 armed)。已修, 单独重跑全套演练 (~80 min); 期间 D21 取证因同时上板被干扰, 待 D22 后单独跑</t>
+          <t>复验 F3 端到端节拍均匀度在主机忙 (D8 大仿真并行) 时不达标: 583 auto std 9.0/5.2 ms (门槛 3/4), 帧率正确; 主机计时抖动敏感, 先不合主线, 待空闲复验 + 上板实测定</t>
         </is>
       </c>
       <c r="E92" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach</t>
+          <t>~/rv_d20c.v.log</t>
         </is>
       </c>
     </row>
@@ -10709,22 +10709,22 @@
       </c>
       <c r="B93" s="6" t="inlineStr">
         <is>
-          <t>验证</t>
+          <t>交付</t>
         </is>
       </c>
       <c r="C93" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D8</t>
         </is>
       </c>
       <c r="D93" s="7" t="inlineStr">
         <is>
-          <t>第二轮上板演练 (单独): 杀 sshd/mdns/povnetd 27-72 s 自愈找回 ✅; 错 SSID → 兜底热点 → 自己回公司网 ✅ (但 23.5 min, 目标 ≤10); 杀 wpa/关网卡、装后重启: 板子恢复了但 mDNS 按名字 240 s 内找不回 ❌ (缓存 IP 可连); 看门狗复位发生但晚于测试判定、卡上未记非正常结束 ❌。交回 D22 agent 修 (mDNS 找回为主)</t>
+          <t>V1 主控↔桥↔2260 联合仿真 0 错 (12/8 bit, 6 链×16 片, 训练锁定, 半圈换帧); 抓出并修 2 个回板必错 bug: 12-bit 字槽格式主控两 beat vs 桥紧排不一致 (改主控 PK12, 上行 195→110 µs/片) + 1 期切片器 NXG 未传 (160 宽按 192 算); 待: 1 期 12-bit 位流重综合 (hclk 余量原 +0.001 ns)</t>
         </is>
       </c>
       <c r="E93" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d22.board2.log</t>
+          <t>dr1v90 task/d8-cosim 85dfe51</t>
         </is>
       </c>
     </row>
@@ -10732,24 +10732,24 @@
       <c r="A94" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B94" s="6" t="inlineStr">
-        <is>
-          <t>根因</t>
+      <c r="B94" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C94" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D8</t>
         </is>
       </c>
       <c r="D94" s="7" t="inlineStr">
         <is>
-          <t>板上取证: 显示每圈取满 142 片, 但 s3rt_sys 旁听只认片号 0..47 → PL 每圈 48 触发后停摆; 不带档位 / 补 sub10 都一样 → RTL 旁听上限 (D21 改为按 FBO) 问题。交回 D21b 修 RTL; 板子已重启回默认 0x20471019</t>
+          <t>V1 联合仿真合主线 (新克隆复验 5/5; 合并回归 sim_v1/pls2047/D18/D19 通过, D19 O4 一次主机忙计时抖动重跑过); V1 回板就绪清单 ⑤ 达成</t>
         </is>
       </c>
       <c r="E94" s="7" t="inlineStr">
         <is>
-          <t>~/d21b_forensic.log</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10759,22 +10759,22 @@
       </c>
       <c r="B95" s="6" t="inlineStr">
         <is>
-          <t>根因</t>
+          <t>测量</t>
         </is>
       </c>
       <c r="C95" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D22/D20</t>
         </is>
       </c>
       <c r="D95" s="7" t="inlineStr">
         <is>
-          <t>按名字找不回的根因: povmdns 在地址回来/重关联时不重新发 IGMP 报告 (重复入组 EADDRINUSE 无报告), 企业 AP 只把组播转给报告过的站点 → mDNS 查询数分钟到不了板。修: 重关联/地址变化时退组再入组 + 宣告 (0/1/3/7/15/30 s) + 每 60 s 刷新; 看门狗读回实际超时并减半到 ≤60 s; 卡上记非正常结束。离线 10/10, 上板复验中</t>
+          <t>1 h 产品配置 (无对拍) 推流诊断: 换帧 14.64/s 软件损失 2.4% ✅, 间隔 p99 124 ms ✅, 长停顿 3.7‰ ✅, 最长 495 ms ❌ (门槛 267); PC→板 ping 16781/0 丢; &gt;0.5 s ACK 停顿 46 min 内 4 次 (最长 0.78 s), 同刻 PC→网关 RTT 165-275 ms = PC 侧 WiFi 抖动。周期 3 s 卡顿消失 (确认系对拍)。余项: 0.5-0.8 s 偶发抖动 (播放缓冲 vs 延迟取舍 / PC 有线或专用路由)</t>
         </is>
       </c>
       <c r="E95" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach 0d1da09</t>
+          <t>soak_runs/netdiag_1015_1814</t>
         </is>
       </c>
     </row>
@@ -10782,24 +10782,24 @@
       <c r="A96" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B96" s="6" t="inlineStr">
-        <is>
-          <t>验证</t>
+      <c r="B96" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C96" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D96" s="7" t="inlineStr">
         <is>
-          <t>第三轮上板演练 9/10: 装后重启 24 s 按名字找回 ✅ (上轮找不回); sshd/mdns/povnetd 杀掉 38-72 s ✅; 关网卡 191 s ✅; 错 SSID→热点→自动回 543 s ✅ (上轮 1411); 看门狗复位 reachkill 54 s / netdstop 213 s 且记非正常结束 ✅ (实际超时 32 s); 仅 kill wpa_supplicant 240 s 内未找回 ❌ (随后恢复), 单独重跑定位中</t>
+          <t>换档位流 (REV 0x20471021) 上板起步即停摆 (档 0 未换档时写完 47 片后停, 换网格全超时), 仿真全过 → 硅上与仿真不同; D21b 开查根因。另: D21 上板收尾用 m90/up.sh 会让板子没 PL, 已重启回开机默认 (0x20471019 + QoS)</t>
         </is>
       </c>
       <c r="E96" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d22b.board.log</t>
+          <t>~/rv_d21.board.log</t>
         </is>
       </c>
     </row>
@@ -10807,9 +10807,9 @@
       <c r="A97" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B97" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+      <c r="B97" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C97" s="7" t="inlineStr">
@@ -10819,12 +10819,12 @@
       </c>
       <c r="D97" s="7" t="inlineStr">
         <is>
-          <t>povnetd 1.2: wpa 进程没了/卡死/接口 down 立即重连 (原来一律等 60 s, 且 60 s 后的重连反把已自愈的连接打断 → 73-240+ s 且不稳); 只丢包仍按 60 s 防误重连; 关键事件写卡 (复位后可查); verify wpakill/ifdown 各连跑 3 次、120 s 内按名字找回。离线 11/11, 上板全套复验中</t>
+          <t>新克隆离线 O6 误 FAIL: hostapd/povreach 二进制 git 模式 644, WSL 本地盘克隆不可执行, qemu 静默拒绝 (板上 autorun 有 chmod, 不受影响); 已修 (git +x, verify chmod), 重跑后自动上板演练</t>
         </is>
       </c>
       <c r="E97" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach e438a12</t>
+          <t>dr1v90 task/d22-reach</t>
         </is>
       </c>
     </row>
@@ -10832,174 +10832,174 @@
       <c r="A98" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B98" s="6" t="inlineStr">
-        <is>
-          <t>根因</t>
+      <c r="B98" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C98" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D98" s="7" t="inlineStr">
         <is>
-          <t>停摆根因不在 RTL: voxslice --pl 从不写显示 0x0C sub01 (bpp3), 重新加载位流后显示按 1-bit 片距 0x3000 取片, 旁听按 0x9000 片首只认 1/3 → 每圈 48 触发卡死。主线同有此隐患 (默认开机靠别的程序先写对)。修: pl_setup 先写 sub01; 仿真 +NOBPP3 复现与板上一致; 位流不变。离线 12/12, 排在 D22 后上板</t>
+          <t>首轮上板演练 9 项误 FAIL = 验收脚本 info() 把板上 board_d22.sh info 的非 0 退出码当失败 (内容正常), settle/wait_healthy 恒失败; 板子本身正常 (装好开机 healthy, povreach managed, 看门狗 armed)。已修, 单独重跑全套演练 (~80 min); 期间 D21 取证因同时上板被干扰, 待 D22 后单独跑</t>
         </is>
       </c>
       <c r="E98" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d21-nband 084bba3</t>
+          <t>dr1v90 task/d22-reach</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="17" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B99" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+        <v>46310</v>
+      </c>
+      <c r="B99" s="6" t="inlineStr">
+        <is>
+          <t>验证</t>
         </is>
       </c>
       <c r="C99" s="7" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D99" s="7" t="inlineStr">
         <is>
-          <t>上行出口全量复验 45/0, 合主线</t>
+          <t>第二轮上板演练 (单独): 杀 sshd/mdns/povnetd 27-72 s 自愈找回 ✅; 错 SSID → 兜底热点 → 自己回公司网 ✅ (但 23.5 min, 目标 ≤10); 杀 wpa/关网卡、装后重启: 板子恢复了但 mDNS 按名字 240 s 内找不回 ❌ (缓存 IP 可连); 看门狗复位发生但晚于测试判定、卡上未记非正常结束 ❌。交回 D22 agent 修 (mDNS 找回为主)</t>
         </is>
       </c>
       <c r="E99" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 fdb4de6</t>
+          <t>~/rv_d22.board2.log</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="17" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B100" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+        <v>46310</v>
+      </c>
+      <c r="B100" s="6" t="inlineStr">
+        <is>
+          <t>根因</t>
         </is>
       </c>
       <c r="C100" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D100" s="7" t="inlineStr">
         <is>
-          <t>PL 切片上板: 与 CPU 逐字节一致、30 min 无停摆, 但内容帧率 4.2&lt;15, 退回</t>
+          <t>板上取证: 显示每圈取满 142 片, 但 s3rt_sys 旁听只认片号 0..47 → PL 每圈 48 触发后停摆; 不带档位 / 补 sub10 都一样 → RTL 旁听上限 (D21 改为按 FBO) 问题。交回 D21b 修 RTL; 板子已重启回默认 0x20471019</t>
         </is>
       </c>
       <c r="E100" s="7" t="inlineStr">
         <is>
-          <t>scratchpad/v_pls4_board.log</t>
+          <t>~/d21b_forensic.log</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="17" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B101" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+        <v>46310</v>
+      </c>
+      <c r="B101" s="6" t="inlineStr">
+        <is>
+          <t>根因</t>
         </is>
       </c>
       <c r="C101" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D101" s="7" t="inlineStr">
         <is>
-          <t>30 Hz 带载迟到+掉片 3.7% (空载 0.2% 来自旧 netguard), 归因测试中</t>
+          <t>按名字找不回的根因: povmdns 在地址回来/重关联时不重新发 IGMP 报告 (重复入组 EADDRINUSE 无报告), 企业 AP 只把组播转给报告过的站点 → mDNS 查询数分钟到不了板。修: 重关联/地址变化时退组再入组 + 宣告 (0/1/3/7/15/30 s) + 每 60 s 刷新; 看门狗读回实际超时并减半到 ≤60 s; 卡上记非正常结束。离线 10/10, 上板复验中</t>
         </is>
       </c>
       <c r="E101" s="7" t="inlineStr">
         <is>
-          <t>project_ddr_budget_by_phase_1013</t>
+          <t>dr1v90 task/d22-reach 0d1da09</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="17" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B102" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+        <v>46310</v>
+      </c>
+      <c r="B102" s="6" t="inlineStr">
+        <is>
+          <t>验证</t>
         </is>
       </c>
       <c r="C102" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D102" s="7" t="inlineStr">
         <is>
-          <t>纯切片带载约 21 min 停摆; 无负载浸泡 2×30 min 不停摆</t>
+          <t>第三轮上板演练 9/10: 装后重启 24 s 按名字找回 ✅ (上轮找不回); sshd/mdns/povnetd 杀掉 38-72 s ✅; 关网卡 191 s ✅; 错 SSID→热点→自动回 543 s ✅ (上轮 1411); 看门狗复位 reachkill 54 s / netdstop 213 s 且记非正常结束 ✅ (实际超时 32 s); 仅 kill wpa_supplicant 240 s 内未找回 ❌ (随后恢复), 单独重跑定位中</t>
         </is>
       </c>
       <c r="E102" s="7" t="inlineStr">
         <is>
-          <t>project_ddr_budget_by_phase_1013</t>
+          <t>~/rv_d22b.board.log</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="17" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B103" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+        <v>46310</v>
+      </c>
+      <c r="B103" s="6" t="inlineStr">
+        <is>
+          <t>交付</t>
         </is>
       </c>
       <c r="C103" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D103" s="7" t="inlineStr">
         <is>
-          <t>用户定目标: 复位到亮起 ≤12 s, 找板 ≤20 s</t>
+          <t>povnetd 1.2: wpa 进程没了/卡死/接口 down 立即重连 (原来一律等 60 s, 且 60 s 后的重连反把已自愈的连接打断 → 73-240+ s 且不稳); 只丢包仍按 60 s 防误重连; 关键事件写卡 (复位后可查); verify wpakill/ifdown 各连跑 3 次、120 s 内按名字找回。离线 11/11, 上板全套复验中</t>
         </is>
       </c>
       <c r="E103" s="7" t="inlineStr">
         <is>
-          <t>project_short_term_delivery_1013</t>
+          <t>dr1v90 task/d22-reach e438a12</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="17" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B104" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+        <v>46310</v>
+      </c>
+      <c r="B104" s="6" t="inlineStr">
+        <is>
+          <t>根因</t>
         </is>
       </c>
       <c r="C104" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D104" s="7" t="inlineStr">
         <is>
-          <t>找到 PL 切片器带载停摆根因: 零列描述符丢失 (公共核, 2260 也有) + pop 握手串片, 已修</t>
+          <t>停摆根因不在 RTL: voxslice --pl 从不写显示 0x0C sub01 (bpp3), 重新加载位流后显示按 1-bit 片距 0x3000 取片, 旁听按 0x9000 片首只认 1/3 → 每圈 48 触发卡死。主线同有此隐患 (默认开机靠别的程序先写对)。修: pl_setup 先写 sub01; 仿真 +NOBPP3 复现与板上一致; 位流不变。离线 12/12, 排在 D22 后上板</t>
         </is>
       </c>
       <c r="E104" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 debd3cd</t>
+          <t>dr1v90 task/d21-nband 084bba3</t>
         </is>
       </c>
     </row>
@@ -11007,24 +11007,24 @@
       <c r="A105" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B105" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B105" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C105" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="D105" s="7" t="inlineStr">
         <is>
-          <t>上板 60 min 带载 0 停摆、逐字节一致、late 0; 帧率 13.8 差 0.5 退回</t>
+          <t>上行出口全量复验 45/0, 合主线</t>
         </is>
       </c>
       <c r="E105" s="7" t="inlineStr">
         <is>
-          <t>scratchpad v_pls6_board.log</t>
+          <t>dr1v90 fdb4de6</t>
         </is>
       </c>
     </row>
@@ -11032,9 +11032,9 @@
       <c r="A106" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B106" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B106" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C106" s="7" t="inlineStr">
@@ -11044,12 +11044,12 @@
       </c>
       <c r="D106" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 实时切片上板全过: 60 min 带载 0 停摆, 帧率 15.0, 与 CPU 逐字节一致</t>
+          <t>PL 切片上板: 与 CPU 逐字节一致、30 min 无停摆, 但内容帧率 4.2&lt;15, 退回</t>
         </is>
       </c>
       <c r="E106" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 782e9e3</t>
+          <t>scratchpad/v_pls4_board.log</t>
         </is>
       </c>
     </row>
@@ -11069,12 +11069,12 @@
       </c>
       <c r="D107" s="7" t="inlineStr">
         <is>
-          <t>DDR 慢读根因: 每圈约 1/3 角度每取一列都换行, 两类 CPU 负载叠加越阈值 (0.002%→3%); 建议网格 4×4 分块</t>
+          <t>30 Hz 带载迟到+掉片 3.7% (空载 0.2% 来自旧 netguard), 归因测试中</t>
         </is>
       </c>
       <c r="E107" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d16-ddr 539d303</t>
+          <t>project_ddr_budget_by_phase_1013</t>
         </is>
       </c>
     </row>
@@ -11082,24 +11082,24 @@
       <c r="A108" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B108" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B108" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C108" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D108" s="7" t="inlineStr">
         <is>
-          <t>用户定: 子 agent 并行 ≤5 (周额度); 跑完的 agent 关掉</t>
+          <t>纯切片带载约 21 min 停摆; 无负载浸泡 2×30 min 不停摆</t>
         </is>
       </c>
       <c r="E108" s="7" t="inlineStr">
         <is>
-          <t>feedback_save_weekly_quota</t>
+          <t>project_ddr_budget_by_phase_1013</t>
         </is>
       </c>
     </row>
@@ -11107,24 +11107,24 @@
       <c r="A109" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B109" s="19" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+      <c r="B109" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C109" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D109" s="7" t="inlineStr">
         <is>
-          <t>V0 出口清单: PL 切片上板通过 (D2) 可打勾</t>
+          <t>用户定目标: 复位到亮起 ≤12 s, 找板 ≤20 s</t>
         </is>
       </c>
       <c r="E109" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 782e9e3</t>
+          <t>project_short_term_delivery_1013</t>
         </is>
       </c>
     </row>
@@ -11132,9 +11132,9 @@
       <c r="A110" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B110" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B110" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C110" s="7" t="inlineStr">
@@ -11144,12 +11144,12 @@
       </c>
       <c r="D110" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 实时切片合进主线 (含公共核两处 bug 修复); D3 上行档位流需按新核重综合</t>
+          <t>找到 PL 切片器带载停摆根因: 零列描述符丢失 (公共核, 2260 也有) + pop 握手串片, 已修</t>
         </is>
       </c>
       <c r="E110" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 2364e5c</t>
+          <t>dr1v90 task/pls-2047 debd3cd</t>
         </is>
       </c>
     </row>
@@ -11157,9 +11157,9 @@
       <c r="A111" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B111" s="19" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+      <c r="B111" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C111" s="7" t="inlineStr">
@@ -11169,12 +11169,12 @@
       </c>
       <c r="D111" s="7" t="inlineStr">
         <is>
-          <t>PL 硬件切片首次实转上屏 (650 rpm, 完成率 100%, CPU 82% 空闲), 用户确认与 CPU 切片无区别</t>
+          <t>上板 60 min 带载 0 停摆、逐字节一致、late 0; 帧率 13.8 差 0.5 退回</t>
         </is>
       </c>
       <c r="E111" s="7" t="inlineStr">
         <is>
-          <t>用户在场实转</t>
+          <t>scratchpad v_pls6_board.log</t>
         </is>
       </c>
     </row>
@@ -11182,24 +11182,24 @@
       <c r="A112" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B112" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B112" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C112" s="7" t="inlineStr">
         <is>
-          <t>D18</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D112" s="7" t="inlineStr">
         <is>
-          <t>用户定: 只保留 PL 切片, 固化开机流程, CPU 切片只留应急退路</t>
+          <t>2047 PL 实时切片上板全过: 60 min 带载 0 停摆, 帧率 15.0, 与 CPU 逐字节一致</t>
         </is>
       </c>
       <c r="E112" s="7" t="inlineStr">
         <is>
-          <t>用户 10-14</t>
+          <t>dr1v90 task/pls-2047 782e9e3</t>
         </is>
       </c>
     </row>
@@ -11207,24 +11207,24 @@
       <c r="A113" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B113" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B113" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C113" s="7" t="inlineStr">
         <is>
-          <t>D18</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D113" s="7" t="inlineStr">
         <is>
-          <t>开机默认 PL 切片合主线: 上电基础显示 → 推流显示推流 → 停推 5 min 回基础演示; CPU 只留应急退路</t>
+          <t>DDR 慢读根因: 每圈约 1/3 角度每取一列都换行, 两类 CPU 负载叠加越阈值 (0.002%→3%); 建议网格 4×4 分块</t>
         </is>
       </c>
       <c r="E113" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d18-pl-default d35c6d4</t>
+          <t>dr1v90 task/d16-ddr 539d303</t>
         </is>
       </c>
     </row>
@@ -11239,17 +11239,17 @@
       </c>
       <c r="C114" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D114" s="7" t="inlineStr">
         <is>
-          <t>用户定目标放宽: 亮起 ≤12.5 s / 找板 ≤21 s; V0 出口 ④ 达成</t>
+          <t>用户定: 子 agent 并行 ≤5 (周额度); 跑完的 agent 关掉</t>
         </is>
       </c>
       <c r="E114" s="7" t="inlineStr">
         <is>
-          <t>用户 10-14</t>
+          <t>feedback_save_weekly_quota</t>
         </is>
       </c>
     </row>
@@ -11257,24 +11257,24 @@
       <c r="A115" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B115" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B115" s="19" t="inlineStr">
+        <is>
+          <t>里程碑</t>
         </is>
       </c>
       <c r="C115" s="7" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D115" s="7" t="inlineStr">
         <is>
-          <t>无串口远程运维合主线: 升级坏包 (含断网包) 自动回滚后板子能按名字找回; 网络守护不再造成切片迟到 (旧版每分钟 2061 次 → 0); V0 出口 ⑤ 达成</t>
+          <t>V0 出口清单: PL 切片上板通过 (D2) 可打勾</t>
         </is>
       </c>
       <c r="E115" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 dee9be6</t>
+          <t>dr1v90 task/pls-2047 782e9e3</t>
         </is>
       </c>
     </row>
@@ -11282,24 +11282,24 @@
       <c r="A116" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B116" s="6" t="inlineStr">
-        <is>
-          <t>根因</t>
+      <c r="B116" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C116" s="7" t="inlineStr">
         <is>
-          <t>D15b</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D116" s="7" t="inlineStr">
         <is>
-          <t>32 bit PL 全黑: 板端写 LUT 基址仍用 16 bit 布局偏移, PL 把网格当角度表读; 已修 308d1bb, 待上板</t>
+          <t>2047 PL 实时切片合进主线 (含公共核两处 bug 修复); D3 上行档位流需按新核重综合</t>
         </is>
       </c>
       <c r="E116" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d15b-color-p2</t>
+          <t>dr1v90 2364e5c</t>
         </is>
       </c>
     </row>
@@ -11307,24 +11307,24 @@
       <c r="A117" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B117" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B117" s="19" t="inlineStr">
+        <is>
+          <t>里程碑</t>
         </is>
       </c>
       <c r="C117" s="7" t="inlineStr">
         <is>
-          <t>D15</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D117" s="7" t="inlineStr">
         <is>
-          <t>WiFi 端 12-bit 通路合主线: 32 bit 像素 PL/CPU 与 CPU 逐字节一致, 2047 上跑通; V0 出口 ⑦ 达成 (7/8)。已知限制: 32 bit 只到 10.83 rps (16.15 rps 时完成率 82-91%)</t>
+          <t>PL 硬件切片首次实转上屏 (650 rpm, 完成率 100%, CPU 82% 空闲), 用户确认与 CPU 切片无区别</t>
         </is>
       </c>
       <c r="E117" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 3a41eb7</t>
+          <t>用户在场实转</t>
         </is>
       </c>
     </row>
@@ -11332,24 +11332,24 @@
       <c r="A118" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B118" s="6" t="inlineStr">
-        <is>
-          <t>开始</t>
+      <c r="B118" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C118" s="7" t="inlineStr">
         <is>
-          <t>KR7.2</t>
+          <t>D18</t>
         </is>
       </c>
       <c r="D118" s="7" t="inlineStr">
         <is>
-          <t>8 h 无人值守长跑开跑 19:20 (假转黑屏, 主线 voxslice 0.6 + 卡上 PL 默认; 推 40 min/停 7 min 循环; 判据 S1-S9; 15 min 试跑 9/9)</t>
+          <t>用户定: 只保留 PL 切片, 固化开机流程, CPU 切片只留应急退路</t>
         </is>
       </c>
       <c r="E118" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 26e69ec soak8h</t>
+          <t>用户 10-14</t>
         </is>
       </c>
     </row>
@@ -11357,24 +11357,24 @@
       <c r="A119" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B119" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B119" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C119" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D18</t>
         </is>
       </c>
       <c r="D119" s="7" t="inlineStr">
         <is>
-          <t>用户批准 QoS 寄存器写入 + 网格 4×4 分块 (D16b 开做, 离线); 长跑后在 2047 做对照</t>
+          <t>开机默认 PL 切片合主线: 上电基础显示 → 推流显示推流 → 停推 5 min 回基础演示; CPU 只留应急退路</t>
         </is>
       </c>
       <c r="E119" s="7" t="inlineStr">
         <is>
-          <t>用户 10-14</t>
+          <t>dr1v90 task/d18-pl-default d35c6d4</t>
         </is>
       </c>
     </row>
@@ -11382,30 +11382,30 @@
       <c r="A120" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B120" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B120" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C120" s="7" t="inlineStr">
         <is>
-          <t>KR7.2</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D120" s="7" t="inlineStr">
         <is>
-          <t>长跑第 6 段企业 WiFi 踢线 ~5 s, 推流端 voxlive 不重连直接退出 (板端处理正确); 修: voxlive 断线自动重连 5cbe79f; 23:45 重开 8 h</t>
+          <t>用户定目标放宽: 亮起 ≤12.5 s / 找板 ≤21 s; V0 出口 ④ 达成</t>
         </is>
       </c>
       <c r="E120" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 5cbe79f</t>
+          <t>用户 10-14</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="17" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B121" s="11" t="inlineStr">
         <is>
@@ -11414,48 +11414,48 @@
       </c>
       <c r="C121" s="7" t="inlineStr">
         <is>
-          <t>E6</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="D121" s="7" t="inlineStr">
         <is>
-          <t>按名字找板 (mDNS) 完成：无串口自重启后 34 s 按名字找到并 ssh 上</t>
+          <t>无串口远程运维合主线: 升级坏包 (含断网包) 自动回滚后板子能按名字找回; 网络守护不再造成切片迟到 (旧版每分钟 2061 次 → 0); V0 出口 ⑤ 达成</t>
         </is>
       </c>
       <c r="E121" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 b0f6b5d</t>
+          <t>dr1v90 dee9be6</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="17" t="n">
-        <v>46308</v>
-      </c>
-      <c r="B122" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46309</v>
+      </c>
+      <c r="B122" s="6" t="inlineStr">
+        <is>
+          <t>根因</t>
         </is>
       </c>
       <c r="C122" s="7" t="inlineStr">
         <is>
-          <t>E7</t>
+          <t>D15b</t>
         </is>
       </c>
       <c r="D122" s="7" t="inlineStr">
         <is>
-          <t>纯切片 30 Hz 位流第一次上硅 D'0–D'3，尾部 late 0.2%，暂停 netguard 后 late/miss 为 0</t>
+          <t>32 bit PL 全黑: 板端写 LUT 基址仍用 16 bit 布局偏移, PL 把网格当角度表读; 已修 308d1bb, 待上板</t>
         </is>
       </c>
       <c r="E122" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 71d006f / 473abcf</t>
+          <t>dr1v90 task/d15b-color-p2</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="17" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B123" s="11" t="inlineStr">
         <is>
@@ -11464,92 +11464,92 @@
       </c>
       <c r="C123" s="7" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>D15</t>
         </is>
       </c>
       <c r="D123" s="7" t="inlineStr">
         <is>
-          <t>主机实时推流完成：10 分钟 15.0 fps，NAK 0 / forced 0</t>
+          <t>WiFi 端 12-bit 通路合主线: 32 bit 像素 PL/CPU 与 CPU 逐字节一致, 2047 上跑通; V0 出口 ⑦ 达成 (7/8)。已知限制: 32 bit 只到 10.83 rps (16.15 rps 时完成率 82-91%)</t>
         </is>
       </c>
       <c r="E123" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 596b191</t>
+          <t>dr1v90 3a41eb7</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="17" t="n">
-        <v>46308</v>
-      </c>
-      <c r="B124" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+        <v>46309</v>
+      </c>
+      <c r="B124" s="6" t="inlineStr">
+        <is>
+          <t>开始</t>
         </is>
       </c>
       <c r="C124" s="7" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>KR7.2</t>
         </is>
       </c>
       <c r="D124" s="7" t="inlineStr">
         <is>
-          <t>第一次上板端到端延迟 p50 114 ms 未过（停等发送），改发送流水线后降到 84.7 ms</t>
+          <t>8 h 无人值守长跑开跑 19:20 (假转黑屏, 主线 voxslice 0.6 + 卡上 PL 默认; 推 40 min/停 7 min 循环; 判据 S1-S9; 15 min 试跑 9/9)</t>
         </is>
       </c>
       <c r="E124" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 60c619a / 596b191</t>
+          <t>dr1v90 26e69ec soak8h</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="17" t="n">
-        <v>46308</v>
-      </c>
-      <c r="B125" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+        <v>46309</v>
+      </c>
+      <c r="B125" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C125" s="7" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D125" s="7" t="inlineStr">
         <is>
-          <t>主会话新克隆独立复验离线+上板全过，合主线（延迟 p50 95 ms / p99 236.6 ms）</t>
+          <t>用户批准 QoS 寄存器写入 + 网格 4×4 分块 (D16b 开做, 离线); 长跑后在 2047 做对照</t>
         </is>
       </c>
       <c r="E125" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 9bf16ad</t>
+          <t>用户 10-14</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="17" t="n">
-        <v>46308</v>
-      </c>
-      <c r="B126" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+        <v>46309</v>
+      </c>
+      <c r="B126" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C126" s="7" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>KR7.2</t>
         </is>
       </c>
       <c r="D126" s="7" t="inlineStr">
         <is>
-          <t>桥接收核对 12-bit 第一次复验 FAIL（新克隆无可执行位），退回</t>
+          <t>长跑第 6 段企业 WiFi 踢线 ~5 s, 推流端 voxlive 不重连直接退出 (板端处理正确); 修: voxlive 断线自动重连 5cbe79f; 23:45 重开 8 h</t>
         </is>
       </c>
       <c r="E126" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 5cbe79f</t>
         </is>
       </c>
     </row>
@@ -11559,22 +11559,22 @@
       </c>
       <c r="B127" s="11" t="inlineStr">
         <is>
-          <t>复验通过</t>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C127" s="7" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>E6</t>
         </is>
       </c>
       <c r="D127" s="7" t="inlineStr">
         <is>
-          <t>桥接收核对 12-bit 复验 PASS，合主线</t>
+          <t>按名字找板 (mDNS) 完成：无串口自重启后 34 s 按名字找到并 ssh 上</t>
         </is>
       </c>
       <c r="E127" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 6a373d3</t>
+          <t>dr1v90 b0f6b5d</t>
         </is>
       </c>
     </row>
@@ -11584,22 +11584,22 @@
       </c>
       <c r="B128" s="11" t="inlineStr">
         <is>
-          <t>复验通过</t>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C128" s="7" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>E7</t>
         </is>
       </c>
       <c r="D128" s="7" t="inlineStr">
         <is>
-          <t>桥驱动 2260 1 期 6 链 24 Hz 12-bit 复验 ALL PASS，合主线</t>
+          <t>纯切片 30 Hz 位流第一次上硅 D'0–D'3，尾部 late 0.2%，暂停 netguard 后 late/miss 为 0</t>
         </is>
       </c>
       <c r="E128" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 cdf49c6</t>
+          <t>dr1v90 71d006f / 473abcf</t>
         </is>
       </c>
     </row>
@@ -11607,24 +11607,24 @@
       <c r="A129" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B129" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B129" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C129" s="7" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="D129" s="7" t="inlineStr">
         <is>
-          <t>6 链 4296 片/s 能跑但余量仅 0.40%，瓶颈是桥→2260 链路；留 10% 需 ≤3921 片/s，待用户定</t>
+          <t>主机实时推流完成：10 分钟 15.0 fps，NAK 0 / forced 0</t>
         </is>
       </c>
       <c r="E129" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 596b191</t>
         </is>
       </c>
     </row>
@@ -11639,17 +11639,17 @@
       </c>
       <c r="C130" s="7" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="D130" s="7" t="inlineStr">
         <is>
-          <t>发现 10-10 验证板 profile 寄存器在 166.67 MHz 下超规格（GCLK 667&gt;600），1 期表已改</t>
+          <t>第一次上板端到端延迟 p50 114 ms 未过（停等发送），改发送流水线后降到 84.7 ms</t>
         </is>
       </c>
       <c r="E130" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 60c619a / 596b191</t>
         </is>
       </c>
     </row>
@@ -11664,17 +11664,17 @@
       </c>
       <c r="C131" s="7" t="inlineStr">
         <is>
-          <t>D6</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="D131" s="7" t="inlineStr">
         <is>
-          <t>几何 LUT 生成器逐字节复现 2047 s3lut，verify 22 PASS，合主线</t>
+          <t>主会话新克隆独立复验离线+上板全过，合主线（延迟 p50 95 ms / p99 236.6 ms）</t>
         </is>
       </c>
       <c r="E131" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 44ed2cd</t>
+          <t>dr1v90 9bf16ad</t>
         </is>
       </c>
     </row>
@@ -11689,12 +11689,12 @@
       </c>
       <c r="C132" s="7" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="D132" s="7" t="inlineStr">
         <is>
-          <t>转子运维首次复验 T5 偶发 FAIL，退回返工</t>
+          <t>桥接收核对 12-bit 第一次复验 FAIL（新克隆无可执行位），退回</t>
         </is>
       </c>
       <c r="E132" s="7" t="inlineStr">
@@ -11714,17 +11714,17 @@
       </c>
       <c r="C133" s="7" t="inlineStr">
         <is>
-          <t>D14</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="D133" s="7" t="inlineStr">
         <is>
-          <t>10 类内容 + 手机网页遥控离线复验 ALL PASS，用户实转看过（尚未正式上板验收）</t>
+          <t>桥接收核对 12-bit 复验 PASS，合主线</t>
         </is>
       </c>
       <c r="E133" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 ffbfeeb</t>
+          <t>dr1v90 6a373d3</t>
         </is>
       </c>
     </row>
@@ -11739,17 +11739,17 @@
       </c>
       <c r="C134" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="D134" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 切片离线复验 26/0，待上板（之后 9ba9af0 测试用例过时 26/27 待修）</t>
+          <t>桥驱动 2260 1 期 6 链 24 Hz 12-bit 复验 ALL PASS，合主线</t>
         </is>
       </c>
       <c r="E134" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 cdf49c6</t>
         </is>
       </c>
     </row>
@@ -11757,19 +11757,19 @@
       <c r="A135" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B135" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B135" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C135" s="7" t="inlineStr">
         <is>
-          <t>D12</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="D135" s="7" t="inlineStr">
         <is>
-          <t>延迟降低上板复验 FAIL：B1 翻页 14.39&lt;15 fps，p99 225 ms，退回</t>
+          <t>6 链 4296 片/s 能跑但余量仅 0.40%，瓶颈是桥→2260 链路；留 10% 需 ≤3921 片/s，待用户定</t>
         </is>
       </c>
       <c r="E135" s="7" t="inlineStr">
@@ -11789,17 +11789,17 @@
       </c>
       <c r="C136" s="7" t="inlineStr">
         <is>
-          <t>D12</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="D136" s="7" t="inlineStr">
         <is>
-          <t>第二次上板仍未过，根因晚间 WiFi 尾巴（p99 334 vs 白天 48 ms）；判据改为调度问题 0 + 网络晚到 ≤1%，明早主机空闲复测</t>
+          <t>发现 10-10 验证板 profile 寄存器在 166.67 MHz 下超规格（GCLK 667&gt;600），1 期表已改</t>
         </is>
       </c>
       <c r="E136" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 764f81d</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -11807,24 +11807,24 @@
       <c r="A137" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B137" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B137" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C137" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D6</t>
         </is>
       </c>
       <c r="D137" s="7" t="inlineStr">
         <is>
-          <t>启动提速上板 FAIL 11 项，但改进已装板保留（6 次重启正常），退回继续压启动时间</t>
+          <t>几何 LUT 生成器逐字节复现 2047 s3lut，verify 22 PASS，合主线</t>
         </is>
       </c>
       <c r="E137" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 44ed2cd</t>
         </is>
       </c>
     </row>
@@ -11832,24 +11832,24 @@
       <c r="A138" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B138" s="19" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+      <c r="B138" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C138" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="D138" s="7" t="inlineStr">
         <is>
-          <t>启动提速两轮后：复位→0° 片亮起 38.7→20.1→15.8 s，找板 34→30→25.6 s</t>
+          <t>转子运维首次复验 T5 偶发 FAIL，退回返工</t>
         </is>
       </c>
       <c r="E138" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d13-boot fdbb217</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -11857,24 +11857,24 @@
       <c r="A139" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B139" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B139" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C139" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D14</t>
         </is>
       </c>
       <c r="D139" s="7" t="inlineStr">
         <is>
-          <t>第二步（bootdelay 0 / 精简 uInitrd）写启动文件被权限系统拒绝，需用户明早本人批准后执行</t>
+          <t>10 类内容 + 手机网页遥控离线复验 ALL PASS，用户实转看过（尚未正式上板验收）</t>
         </is>
       </c>
       <c r="E139" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 ffbfeeb</t>
         </is>
       </c>
     </row>
@@ -11889,17 +11889,17 @@
       </c>
       <c r="C140" s="7" t="inlineStr">
         <is>
-          <t>D15</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D140" s="7" t="inlineStr">
         <is>
-          <t>WiFi 端 32 bit 像素（X2R10G10B10）阶段 1 复验：黄金/PL 仿真一致，合主线</t>
+          <t>2047 PL 切片离线复验 26/0，待上板（之后 9ba9af0 测试用例过时 26/27 待修）</t>
         </is>
       </c>
       <c r="E140" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 1995be8</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -11907,19 +11907,19 @@
       <c r="A141" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B141" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B141" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C141" s="7" t="inlineStr">
         <is>
-          <t>D3;D4;D5</t>
+          <t>D12</t>
         </is>
       </c>
       <c r="D141" s="7" t="inlineStr">
         <is>
-          <t>下午用户：2260 相关先暂停、先做共用部分（token 不够）；15:00 又改为多开并行恢复 2260</t>
+          <t>延迟降低上板复验 FAIL：B1 翻页 14.39&lt;15 fps，p99 225 ms，退回</t>
         </is>
       </c>
       <c r="E141" s="7" t="inlineStr">
@@ -11932,20 +11932,24 @@
       <c r="A142" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B142" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
-        </is>
-      </c>
-      <c r="C142" s="7" t="inlineStr"/>
+      <c r="B142" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
+        </is>
+      </c>
+      <c r="C142" s="7" t="inlineStr">
+        <is>
+          <t>D12</t>
+        </is>
+      </c>
       <c r="D142" s="7" t="inlineStr">
         <is>
-          <t>软件三期：0 期 2047 屏（现在）/ 1 期 2260 验证板 160×180（预计 11-10 回板）/ 2 期 192×216 目标板；1 期目标 24 Hz / 358 片 / 6 链</t>
+          <t>第二次上板仍未过，根因晚间 WiFi 尾巴（p99 334 vs 白天 48 ms）；判据改为调度问题 0 + 网络晚到 ≤1%，明早主机空闲复测</t>
         </is>
       </c>
       <c r="E142" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_sw_three_phases_1013.md</t>
+          <t>dr1v90 764f81d</t>
         </is>
       </c>
     </row>
@@ -11953,20 +11957,24 @@
       <c r="A143" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B143" s="19" t="inlineStr">
-        <is>
-          <t>里程碑</t>
-        </is>
-      </c>
-      <c r="C143" s="7" t="inlineStr"/>
+      <c r="B143" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
+        </is>
+      </c>
+      <c r="C143" s="7" t="inlineStr">
+        <is>
+          <t>D13</t>
+        </is>
+      </c>
       <c r="D143" s="7" t="inlineStr">
         <is>
-          <t>硬件 1 期验证板预计 2026-11-10 回板（初步交期，可能变），回板前软件能做的都前置</t>
+          <t>启动提速上板 FAIL 11 项，但改进已装板保留（6 次重启正常），退回继续压启动时间</t>
         </is>
       </c>
       <c r="E143" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_sw_three_phases_1013.md</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -11974,20 +11982,24 @@
       <c r="A144" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B144" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
-        </is>
-      </c>
-      <c r="C144" s="7" t="inlineStr"/>
+      <c r="B144" s="19" t="inlineStr">
+        <is>
+          <t>里程碑</t>
+        </is>
+      </c>
+      <c r="C144" s="7" t="inlineStr">
+        <is>
+          <t>D13</t>
+        </is>
+      </c>
       <c r="D144" s="7" t="inlineStr">
         <is>
-          <t>架构切分：PL 切片器及之前为各期共用的公共部分，屏幕显示为可替换后端，两者之间用实时按角度片流接口</t>
+          <t>启动提速两轮后：复位→0° 片亮起 38.7→20.1→15.8 s，找板 34→30→25.6 s</t>
         </is>
       </c>
       <c r="E144" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_arch_common_front_display_backend.md</t>
+          <t>dr1v90 task/d13-boot fdbb217</t>
         </is>
       </c>
     </row>
@@ -11995,19 +12007,19 @@
       <c r="A145" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B145" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B145" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C145" s="7" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D145" s="7" t="inlineStr">
         <is>
-          <t>用户定：2 期上行 1.2G；1 期保持 24 Hz（358 片，桥链路余量 0.40%）不降档</t>
+          <t>第二步（bootdelay 0 / 精简 uInitrd）写启动文件被权限系统拒绝，需用户明早本人批准后执行</t>
         </is>
       </c>
       <c r="E145" s="7" t="inlineStr">
@@ -12020,24 +12032,24 @@
       <c r="A146" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B146" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B146" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C146" s="7" t="inlineStr">
         <is>
-          <t>D11</t>
+          <t>D15</t>
         </is>
       </c>
       <c r="D146" s="7" t="inlineStr">
         <is>
-          <t>傍晚用户：杜邦线跑不了 1.2G，1.2G 实测等 V1 回板；C1 台架只做 ≤300M 低速功能档</t>
+          <t>WiFi 端 32 bit 像素（X2R10G10B10）阶段 1 复验：黄金/PL 仿真一致，合主线</t>
         </is>
       </c>
       <c r="E146" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 1995be8</t>
         </is>
       </c>
     </row>
@@ -12052,12 +12064,12 @@
       </c>
       <c r="C147" s="7" t="inlineStr">
         <is>
-          <t>D12;D13;D14</t>
+          <t>D3;D4;D5</t>
         </is>
       </c>
       <c r="D147" s="7" t="inlineStr">
         <is>
-          <t>19:00 用户：V0 可见的先插队、V1 接着做，新派 D12 延迟降低 / D13 启动提速 / D14 内容与手机控制</t>
+          <t>下午用户：2260 相关先暂停、先做共用部分（token 不够）；15:00 又改为多开并行恢复 2260</t>
         </is>
       </c>
       <c r="E147" s="7" t="inlineStr">
@@ -12075,19 +12087,15 @@
           <t>决定</t>
         </is>
       </c>
-      <c r="C148" s="7" t="inlineStr">
-        <is>
-          <t>D13</t>
-        </is>
-      </c>
+      <c r="C148" s="7" t="inlineStr"/>
       <c r="D148" s="7" t="inlineStr">
         <is>
-          <t>21:10 用户定 D13 目标：复位到 0° 片亮起 ≤12 s，找板 ≤20 s（看板 KR8.1 已改）</t>
+          <t>软件三期：0 期 2047 屏（现在）/ 1 期 2260 验证板 160×180（预计 11-10 回板）/ 2 期 192×216 目标板；1 期目标 24 Hz / 358 片 / 6 链</t>
         </is>
       </c>
       <c r="E148" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>claude_memory/project_sw_three_phases_1013.md</t>
         </is>
       </c>
     </row>
@@ -12095,24 +12103,20 @@
       <c r="A149" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B149" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
-        </is>
-      </c>
-      <c r="C149" s="7" t="inlineStr">
-        <is>
-          <t>D15;D16</t>
-        </is>
-      </c>
+      <c r="B149" s="19" t="inlineStr">
+        <is>
+          <t>里程碑</t>
+        </is>
+      </c>
+      <c r="C149" s="7" t="inlineStr"/>
       <c r="D149" s="7" t="inlineStr">
         <is>
-          <t>用户选 12-bit 方案 A：WiFi 端传高位宽、像素位宽 16/32 bit 可配（D15）；DDR 做到极限 A 线（D16），B 线并入 T2 硬件</t>
+          <t>硬件 1 期验证板预计 2026-11-10 回板（初步交期，可能变），回板前软件能做的都前置</t>
         </is>
       </c>
       <c r="E149" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>claude_memory/project_sw_three_phases_1013.md</t>
         </is>
       </c>
     </row>
@@ -12125,19 +12129,15 @@
           <t>决定</t>
         </is>
       </c>
-      <c r="C150" s="7" t="inlineStr">
-        <is>
-          <t>KR5.2</t>
-        </is>
-      </c>
+      <c r="C150" s="7" t="inlineStr"/>
       <c r="D150" s="7" t="inlineStr">
         <is>
-          <t>用户实转核实：2047 旧表镜像，已更正为新表 0decad54</t>
+          <t>架构切分：PL 切片器及之前为各期共用的公共部分，屏幕显示为可替换后端，两者之间用实时按角度片流接口</t>
         </is>
       </c>
       <c r="E150" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 49031f6</t>
+          <t>claude_memory/project_arch_common_front_display_backend.md</t>
         </is>
       </c>
     </row>
@@ -12145,19 +12145,19 @@
       <c r="A151" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B151" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B151" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C151" s="7" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="D151" s="7" t="inlineStr">
         <is>
-          <t>D7 上板补测会装/还原 autorun，冲掉 D13 补丁，须排在 D13 定稿合并之后；夜间板子排程 D12→D13→D2→D7→8 h 长跑</t>
+          <t>用户定：2 期上行 1.2G；1 期保持 24 Hz（358 片，桥链路余量 0.40%）不降档</t>
         </is>
       </c>
       <c r="E151" s="7" t="inlineStr">
@@ -12170,18 +12170,168 @@
       <c r="A152" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B152" s="19" t="inlineStr">
+      <c r="B152" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
+        </is>
+      </c>
+      <c r="C152" s="7" t="inlineStr">
+        <is>
+          <t>D11</t>
+        </is>
+      </c>
+      <c r="D152" s="7" t="inlineStr">
+        <is>
+          <t>傍晚用户：杜邦线跑不了 1.2G，1.2G 实测等 V1 回板；C1 台架只做 ≤300M 低速功能档</t>
+        </is>
+      </c>
+      <c r="E152" s="7" t="inlineStr">
+        <is>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B153" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
+        </is>
+      </c>
+      <c r="C153" s="7" t="inlineStr">
+        <is>
+          <t>D12;D13;D14</t>
+        </is>
+      </c>
+      <c r="D153" s="7" t="inlineStr">
+        <is>
+          <t>19:00 用户：V0 可见的先插队、V1 接着做，新派 D12 延迟降低 / D13 启动提速 / D14 内容与手机控制</t>
+        </is>
+      </c>
+      <c r="E153" s="7" t="inlineStr">
+        <is>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B154" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
+        </is>
+      </c>
+      <c r="C154" s="7" t="inlineStr">
+        <is>
+          <t>D13</t>
+        </is>
+      </c>
+      <c r="D154" s="7" t="inlineStr">
+        <is>
+          <t>21:10 用户定 D13 目标：复位到 0° 片亮起 ≤12 s，找板 ≤20 s（看板 KR8.1 已改）</t>
+        </is>
+      </c>
+      <c r="E154" s="7" t="inlineStr">
+        <is>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B155" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
+        </is>
+      </c>
+      <c r="C155" s="7" t="inlineStr">
+        <is>
+          <t>D15;D16</t>
+        </is>
+      </c>
+      <c r="D155" s="7" t="inlineStr">
+        <is>
+          <t>用户选 12-bit 方案 A：WiFi 端传高位宽、像素位宽 16/32 bit 可配（D15）；DDR 做到极限 A 线（D16），B 线并入 T2 硬件</t>
+        </is>
+      </c>
+      <c r="E155" s="7" t="inlineStr">
+        <is>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B156" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
+        </is>
+      </c>
+      <c r="C156" s="7" t="inlineStr">
+        <is>
+          <t>KR5.2</t>
+        </is>
+      </c>
+      <c r="D156" s="7" t="inlineStr">
+        <is>
+          <t>用户实转核实：2047 旧表镜像，已更正为新表 0decad54</t>
+        </is>
+      </c>
+      <c r="E156" s="7" t="inlineStr">
+        <is>
+          <t>dr1v90 49031f6</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B157" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
+        </is>
+      </c>
+      <c r="C157" s="7" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="D157" s="7" t="inlineStr">
+        <is>
+          <t>D7 上板补测会装/还原 autorun，冲掉 D13 补丁，须排在 D13 定稿合并之后；夜间板子排程 D12→D13→D2→D7→8 h 长跑</t>
+        </is>
+      </c>
+      <c r="E157" s="7" t="inlineStr">
+        <is>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B158" s="19" t="inlineStr">
         <is>
           <t>里程碑</t>
         </is>
       </c>
-      <c r="C152" s="7" t="inlineStr"/>
-      <c r="D152" s="7" t="inlineStr">
+      <c r="C158" s="7" t="inlineStr"/>
+      <c r="D158" s="7" t="inlineStr">
         <is>
           <t>显性目的进度看板第一版建立：10 个显性目的 + KR 趋势 + 燃起图 + 里程碑趋势</t>
         </is>
       </c>
-      <c r="E152" s="7" t="inlineStr">
+      <c r="E158" s="7" t="inlineStr">
         <is>
           <t>claude_memory/project_progress_dashboard.md</t>
         </is>
@@ -17000,7 +17150,7 @@
         <v>20</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9">
@@ -18404,15 +18554,17 @@
       <c r="E58" s="17" t="n">
         <v>46312</v>
       </c>
-      <c r="F58" s="17" t="n"/>
-      <c r="G58" s="15" t="inlineStr">
-        <is>
-          <t>🔄</t>
+      <c r="F58" s="17" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G58" s="11" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="H58" s="7" t="inlineStr">
         <is>
-          <t>task/d20e-phaselock (agent 进行中)</t>
+          <t>合主线 c80f5fb; 上板 583 rpm 滑格 5.2%→0.19%, 900 rpm 22%→0.12%; 卡上已部署 (voxslice ba243d71), 重启验收 6/6</t>
         </is>
       </c>
     </row>
@@ -18440,15 +18592,17 @@
       <c r="E59" s="17" t="n">
         <v>46312</v>
       </c>
-      <c r="F59" s="17" t="n"/>
-      <c r="G59" s="24" t="inlineStr">
-        <is>
-          <t>⏸</t>
+      <c r="F59" s="17" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G59" s="11" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="H59" s="7" t="inlineStr">
         <is>
-          <t>待用户确认是哪版立方体动画</t>
+          <t>用户看预览后定: 保持现状 geo_loop (含线框立方体); 候选 cube_loop/cube_faces_loop 留主线 d24_bootcube (dc19477)</t>
         </is>
       </c>
     </row>
@@ -18476,15 +18630,17 @@
       <c r="E60" s="17" t="n">
         <v>46319</v>
       </c>
-      <c r="F60" s="17" t="n"/>
-      <c r="G60" s="15" t="inlineStr">
-        <is>
-          <t>🔄</t>
+      <c r="F60" s="17" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G60" s="11" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="H60" s="7" t="inlineStr">
         <is>
-          <t>task/d23-v1content (agent 进行中)</t>
+          <t>合主线 a41d63b; 离线对拍 24/0 (V1 片流 == 参考, V0 dump 不变); 回板步骤 d23_v1content/DESIGN.md §5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[看板] D12 延迟复测完成 (lead 70 ms)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/progress/显性目的进度_2026-10-16.xlsx
+++ b/docs/progress/显性目的进度_2026-10-16.xlsx
@@ -8522,7 +8522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J161"/>
+  <dimension ref="A1:J162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -10280,7 +10280,7 @@
     </row>
     <row r="76">
       <c r="A76" s="17" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B76" s="11" t="inlineStr">
         <is>
@@ -10289,17 +10289,17 @@
       </c>
       <c r="C76" s="7" t="inlineStr">
         <is>
-          <t>KR7.2</t>
+          <t>D12</t>
         </is>
       </c>
       <c r="D76" s="7" t="inlineStr">
         <is>
-          <t>8 h 无人值守长跑 9/9 通过 (重开轮 23:45-07:45; 判读 S1 行数口径误判已改为覆盖时长 fe53bde); V0 出口 ⑥ 达成 → V0 出口 8/8</t>
+          <t>延迟复测合主线: 相位锁定 auto 保持, lock-lead 150→70 ms; 583 rpm 延迟 p50/p95/p99 133/138/155 ms (锁相关 126/127/196, 滑格 2.1%→0.14%); 900 rpm 122/206/276 ms 滑格 0.37%; 帧间隔 p95 = 理想</t>
         </is>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>progress/soak_v0/report.md</t>
+          <t>dr1v90 d12_latency/RESULTS.md</t>
         </is>
       </c>
     </row>
@@ -10307,24 +10307,24 @@
       <c r="A77" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B77" s="6" t="inlineStr">
-        <is>
-          <t>测量</t>
+      <c r="B77" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C77" s="7" t="inlineStr">
         <is>
-          <t>QoS</t>
+          <t>KR7.2</t>
         </is>
       </c>
       <c r="D77" s="7" t="inlineStr">
         <is>
-          <t>QoS (XMON DDR_S2 QOS_CONFIG=0x0F) 带载对照 (纯切片 30 Hz): 体素流+TCP 迟到 4.12% → 0.000%, CPU memcpy 300 MB/s 91.5% → 0.000%; 2047 32 bit@16.15 rps 完成率无改善 (86/71% vs 无 QoS 91/82%, 带宽上限); 测后寄存器已写回 0</t>
+          <t>8 h 无人值守长跑 9/9 通过 (重开轮 23:45-07:45; 判读 S1 行数口径误判已改为覆盖时长 fe53bde); V0 出口 ⑥ 达成 → V0 出口 8/8</t>
         </is>
       </c>
       <c r="E77" s="7" t="inlineStr">
         <is>
-          <t>~/qos_runs</t>
+          <t>progress/soak_v0/report.md</t>
         </is>
       </c>
     </row>
@@ -10339,17 +10339,17 @@
       </c>
       <c r="C78" s="7" t="inlineStr">
         <is>
-          <t>D16b</t>
+          <t>QoS</t>
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr">
         <is>
-          <t>4x4 分块上板 A/B: 体素流+TCP 迟到 现布局 5.34%/4.45% (漂移 0.89 pp) vs 分块 4.79%, 收益在漂移内 = 无效; 迟到角度随相位漂移, 非几何换行主导。按约定不合主线, 分支 task/d16b-tile 保留</t>
+          <t>QoS (XMON DDR_S2 QOS_CONFIG=0x0F) 带载对照 (纯切片 30 Hz): 体素流+TCP 迟到 4.12% → 0.000%, CPU memcpy 300 MB/s 91.5% → 0.000%; 2047 32 bit@16.15 rps 完成率无改善 (86/71% vs 无 QoS 91/82%, 带宽上限); 测后寄存器已写回 0</t>
         </is>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d16b-tile 7936b7e</t>
+          <t>~/qos_runs</t>
         </is>
       </c>
     </row>
@@ -10357,24 +10357,24 @@
       <c r="A79" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B79" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B79" s="6" t="inlineStr">
+        <is>
+          <t>测量</t>
         </is>
       </c>
       <c r="C79" s="7" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>D16b</t>
         </is>
       </c>
       <c r="D79" s="7" t="inlineStr">
         <is>
-          <t>用户定 V0/V1/V2 兼容 300-1200 rpm; 实转 583 rpm PL 只 8 fps (等整圈换帧) → D19 半圈换帧开做 (RTL+voxslice+假转扫速验收)</t>
+          <t>4x4 分块上板 A/B: 体素流+TCP 迟到 现布局 5.34%/4.45% (漂移 0.89 pp) vs 分块 4.79%, 收益在漂移内 = 无效; 迟到角度随相位漂移, 非几何换行主导。按约定不合主线, 分支 task/d16b-tile 保留</t>
         </is>
       </c>
       <c r="E79" s="7" t="inlineStr">
         <is>
-          <t>用户 10-15</t>
+          <t>dr1v90 task/d16b-tile 7936b7e</t>
         </is>
       </c>
     </row>
@@ -10389,12 +10389,12 @@
       </c>
       <c r="C80" s="7" t="inlineStr">
         <is>
-          <t>D20</t>
+          <t>D19</t>
         </is>
       </c>
       <c r="D80" s="7" t="inlineStr">
         <is>
-          <t>用户定流畅显示为一等要求 (V0/V1/V2); D20 阶段 1 流畅度指标+门槛+基线开做 (与 D19 并行)</t>
+          <t>用户定 V0/V1/V2 兼容 300-1200 rpm; 实转 583 rpm PL 只 8 fps (等整圈换帧) → D19 半圈换帧开做 (RTL+voxslice+假转扫速验收)</t>
         </is>
       </c>
       <c r="E80" s="7" t="inlineStr">
@@ -10407,24 +10407,24 @@
       <c r="A81" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B81" s="6" t="inlineStr">
-        <is>
-          <t>分析</t>
+      <c r="B81" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C81" s="7" t="inlineStr">
         <is>
-          <t>V1/V2</t>
+          <t>D20</t>
         </is>
       </c>
       <c r="D81" s="7" t="inlineStr">
         <is>
-          <t>转速 300-1200 rpm 纸面预算: 300 rpm 体刷新仅 10 Hz (物理闪烁); V1 358 片只到 ~718 rpm, 1200 需降到 215 片; V2 605 片到 ~1060 rpm; 公共切片核需支持运行时换每圈片数 (见 budget/rpm_range_2026-10-15.md)</t>
+          <t>用户定流畅显示为一等要求 (V0/V1/V2); D20 阶段 1 流畅度指标+门槛+基线开做 (与 D19 并行)</t>
         </is>
       </c>
       <c r="E81" s="7" t="inlineStr">
         <is>
-          <t>budget/rpm_range_2026-10-15.md</t>
+          <t>用户 10-15</t>
         </is>
       </c>
     </row>
@@ -10432,24 +10432,24 @@
       <c r="A82" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B82" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B82" s="6" t="inlineStr">
+        <is>
+          <t>分析</t>
         </is>
       </c>
       <c r="C82" s="7" t="inlineStr">
         <is>
-          <t>KR7.3</t>
+          <t>V1/V2</t>
         </is>
       </c>
       <c r="D82" s="7" t="inlineStr">
         <is>
-          <t>实转 1 h 无故障通过 (583 rpm, QoS 开机默认已上卡 7d301a6); V0 必须项全部达成</t>
+          <t>转速 300-1200 rpm 纸面预算: 300 rpm 体刷新仅 10 Hz (物理闪烁); V1 358 片只到 ~718 rpm, 1200 需降到 215 片; V2 605 片到 ~1060 rpm; 公共切片核需支持运行时换每圈片数 (见 budget/rpm_range_2026-10-15.md)</t>
         </is>
       </c>
       <c r="E82" s="7" t="inlineStr">
         <is>
-          <t>progress/realspin_v0/</t>
+          <t>budget/rpm_range_2026-10-15.md</t>
         </is>
       </c>
     </row>
@@ -10457,19 +10457,19 @@
       <c r="A83" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B83" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B83" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C83" s="7" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>KR7.3</t>
         </is>
       </c>
       <c r="D83" s="7" t="inlineStr">
         <is>
-          <t>实转换帧仅 10.45/s (583 rpm 整圈换帧限制), 用户感觉卡; D19 半圈换帧 + D20 流畅度门槛处理</t>
+          <t>实转 1 h 无故障通过 (583 rpm, QoS 开机默认已上卡 7d301a6); V0 必须项全部达成</t>
         </is>
       </c>
       <c r="E83" s="7" t="inlineStr">
@@ -10482,24 +10482,24 @@
       <c r="A84" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B84" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+      <c r="B84" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C84" s="7" t="inlineStr">
         <is>
-          <t>D20</t>
+          <t>D19</t>
         </is>
       </c>
       <c r="D84" s="7" t="inlineStr">
         <is>
-          <t>流畅度阶段 1: host/smooth_report.py + 门槛 (软件损失≤3%, 间隔 p99≤2T0, 长停顿≤5‰, 撕裂 0 等, SPEC §12) + voxslice --flip-log; 基线: 8 h 假转软件损失 2.3% 但约每 2 min 一次 2-3 s 无新帧 (主机/链路侧, 板端 PL 无缺口) 判 FAIL; 实转 648 rpm 软件损失 3.5%, 每分钟至少一顿 0.3-1.1 s 判 FAIL。主会话复验中</t>
+          <t>实转换帧仅 10.45/s (583 rpm 整圈换帧限制), 用户感觉卡; D19 半圈换帧 + D20 流畅度门槛处理</t>
         </is>
       </c>
       <c r="E84" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20-smooth 83a5fd7</t>
+          <t>progress/realspin_v0/</t>
         </is>
       </c>
     </row>
@@ -10507,24 +10507,24 @@
       <c r="A85" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B85" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B85" s="6" t="inlineStr">
+        <is>
+          <t>交付</t>
         </is>
       </c>
       <c r="C85" s="7" t="inlineStr">
         <is>
-          <t>D14</t>
+          <t>D20</t>
         </is>
       </c>
       <c r="D85" s="7" t="inlineStr">
         <is>
-          <t>更多内容 + 手机网页控制合主线 (用户实转看过); 新克隆回归全过</t>
+          <t>流畅度阶段 1: host/smooth_report.py + 门槛 (软件损失≤3%, 间隔 p99≤2T0, 长停顿≤5‰, 撕裂 0 等, SPEC §12) + voxslice --flip-log; 基线: 8 h 假转软件损失 2.3% 但约每 2 min 一次 2-3 s 无新帧 (主机/链路侧, 板端 PL 无缺口) 判 FAIL; 实转 648 rpm 软件损失 3.5%, 每分钟至少一顿 0.3-1.1 s 判 FAIL。主会话复验中</t>
         </is>
       </c>
       <c r="E85" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 e215176</t>
+          <t>dr1v90 task/d20-smooth 83a5fd7</t>
         </is>
       </c>
     </row>
@@ -10532,24 +10532,24 @@
       <c r="A86" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B86" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+      <c r="B86" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C86" s="7" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>D14</t>
         </is>
       </c>
       <c r="D86" s="7" t="inlineStr">
         <is>
-          <t>半圈换帧: 换网格上限 1×→2×转速 (583 rpm 9.7→~19/s), 慢转均匀丢帧; 16/32 档位流时序收住 (REV 0x20471019/1A); 转速窗口 300-1200; 离线 16/16 + 仿真 21+5 + pls2047 32/32。主会话复验+上板假转扫点中</t>
+          <t>更多内容 + 手机网页控制合主线 (用户实转看过); 新克隆回归全过</t>
         </is>
       </c>
       <c r="E86" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d19-halfrev 1beafa6</t>
+          <t>dr1v90 e215176</t>
         </is>
       </c>
     </row>
@@ -10564,17 +10564,17 @@
       </c>
       <c r="C87" s="7" t="inlineStr">
         <is>
-          <t>D20b</t>
+          <t>D19</t>
         </is>
       </c>
       <c r="D87" s="7" t="inlineStr">
         <is>
-          <t>画面模拟器 host/pov_view.py (按视觉暂留合成人眼所见, 并排对比): 整圈换帧 9.8/s 跳 51 帧; 半圈 15/s 但 51/103 ms 交替 (内容 15 fps 与半圈节拍不齐 → D20 阶段 3 内容帧率跟转速); 300 rpm 闪烁; 停推冻结后跳帧。示例 gif 在 dr1v90/_work/d20b/d20_smooth/sim_out/; 复验 PASS</t>
+          <t>半圈换帧: 换网格上限 1×→2×转速 (583 rpm 9.7→~19/s), 慢转均匀丢帧; 16/32 档位流时序收住 (REV 0x20471019/1A); 转速窗口 300-1200; 离线 16/16 + 仿真 21+5 + pls2047 32/32。主会话复验+上板假转扫点中</t>
         </is>
       </c>
       <c r="E87" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20b-sim 9081f62</t>
+          <t>dr1v90 task/d19-halfrev 1beafa6</t>
         </is>
       </c>
     </row>
@@ -10584,22 +10584,22 @@
       </c>
       <c r="B88" s="6" t="inlineStr">
         <is>
-          <t>验证</t>
+          <t>交付</t>
         </is>
       </c>
       <c r="C88" s="7" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>D20b</t>
         </is>
       </c>
       <c r="D88" s="7" t="inlineStr">
         <is>
-          <t>半圈换帧上板假转扫点 PASS: 5/7.5/10/15/20 rps 换网格 9.00/13.56/15.09/15.09/15.08 每秒 (老行为 10 rps 仅 9.00), 完成率 100%, 撕裂 0, 对拍全一致, 超时 0; 卡上开机默认已是 D19 位流 0x20471019。D19+D20+D20b 合并分支全回归中</t>
+          <t>画面模拟器 host/pov_view.py (按视觉暂留合成人眼所见, 并排对比): 整圈换帧 9.8/s 跳 51 帧; 半圈 15/s 但 51/103 ms 交替 (内容 15 fps 与半圈节拍不齐 → D20 阶段 3 内容帧率跟转速); 300 rpm 闪烁; 停推冻结后跳帧。示例 gif 在 dr1v90/_work/d20b/d20_smooth/sim_out/; 复验 PASS</t>
         </is>
       </c>
       <c r="E88" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/merge-d19-d20 106364e</t>
+          <t>dr1v90 task/d20b-sim 9081f62</t>
         </is>
       </c>
     </row>
@@ -10607,24 +10607,24 @@
       <c r="A89" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B89" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B89" s="6" t="inlineStr">
+        <is>
+          <t>验证</t>
         </is>
       </c>
       <c r="C89" s="7" t="inlineStr">
         <is>
-          <t>D19/D20</t>
+          <t>D19</t>
         </is>
       </c>
       <c r="D89" s="7" t="inlineStr">
         <is>
-          <t>半圈换帧 + 流畅度检测 + 画面模拟器合主线; 全回归 10 套 (D18/D13/D19/D20/D20b/color/pls2047/rotor_ops/live_push/重连) 通过; 下一步 D20 阶段 3 (内容帧率跟转速、主机侧停顿诊断) + 实转复核</t>
+          <t>半圈换帧上板假转扫点 PASS: 5/7.5/10/15/20 rps 换网格 9.00/13.56/15.09/15.09/15.08 每秒 (老行为 10 rps 仅 9.00), 完成率 100%, 撕裂 0, 对拍全一致, 超时 0; 卡上开机默认已是 D19 位流 0x20471019。D19+D20+D20b 合并分支全回归中</t>
         </is>
       </c>
       <c r="E89" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>dr1v90 task/merge-d19-d20 106364e</t>
         </is>
       </c>
     </row>
@@ -10632,24 +10632,24 @@
       <c r="A90" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B90" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+      <c r="B90" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C90" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D19/D20</t>
         </is>
       </c>
       <c r="D90" s="7" t="inlineStr">
         <is>
-          <t>每圈片数随转速换档 (V1/V2 到 1200 rpm 的前提): N/PB/LUT 圈边界同步锁存, 回差 5%; V0 2047 人为 142/128 两档仿真逐字节一致、撕裂 0, 假转斜坡升降各 1 次不抖; 16/32 档位流时序收住 (REV 0x20471021/22)。风险: 软件写序时间窗 (可加影子寄存器)。主会话复验中, 诊断跑完后上板</t>
+          <t>半圈换帧 + 流畅度检测 + 画面模拟器合主线; 全回归 10 套 (D18/D13/D19/D20/D20b/color/pls2047/rotor_ops/live_push/重连) 通过; 下一步 D20 阶段 3 (内容帧率跟转速、主机侧停顿诊断) + 实转复核</t>
         </is>
       </c>
       <c r="E90" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d21-nband adeba44</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10659,22 +10659,22 @@
       </c>
       <c r="B91" s="6" t="inlineStr">
         <is>
-          <t>根因</t>
+          <t>交付</t>
         </is>
       </c>
       <c r="C91" s="7" t="inlineStr">
         <is>
-          <t>D20/D22</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D91" s="7" t="inlineStr">
         <is>
-          <t>推流每 124.5 s 卡 3 s 的根因 = 长跑脚本的板上对拍 (--pl-verify 1800 ≈ 每 120 s, 每次停 ~3 s), 测试工具自身, 产品默认不开; WiFi 链路同刻 ping 0 丢。WSL/Windows 各 6 min 回放对照: 无周期卡顿, 但有偶发 1-1.7 s ACK 停顿 (每 6 min 1-2 次) = 真实 WiFi 抖动 → D22 WiFi 稳定 (用户 10-15: V0 必须搞定, 不能靠串口)</t>
+          <t>每圈片数随转速换档 (V1/V2 到 1200 rpm 的前提): N/PB/LUT 圈边界同步锁存, 回差 5%; V0 2047 人为 142/128 两档仿真逐字节一致、撕裂 0, 假转斜坡升降各 1 次不抖; 16/32 档位流时序收住 (REV 0x20471021/22)。风险: 软件写序时间窗 (可加影子寄存器)。主会话复验中, 诊断跑完后上板</t>
         </is>
       </c>
       <c r="E91" s="7" t="inlineStr">
         <is>
-          <t>~/realspin/tcp</t>
+          <t>dr1v90 task/d21-nband adeba44</t>
         </is>
       </c>
     </row>
@@ -10682,24 +10682,24 @@
       <c r="A92" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B92" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B92" s="6" t="inlineStr">
+        <is>
+          <t>根因</t>
         </is>
       </c>
       <c r="C92" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D20/D22</t>
         </is>
       </c>
       <c r="D92" s="7" t="inlineStr">
         <is>
-          <t>用户: 不插串口也必须永远连得上, 彻底解决 (V0 必须) → D22 四层兜底开做: 服务监护 + 硬件看门狗 + 兜底热点 + 故障注入验收</t>
+          <t>推流每 124.5 s 卡 3 s 的根因 = 长跑脚本的板上对拍 (--pl-verify 1800 ≈ 每 120 s, 每次停 ~3 s), 测试工具自身, 产品默认不开; WiFi 链路同刻 ping 0 丢。WSL/Windows 各 6 min 回放对照: 无周期卡顿, 但有偶发 1-1.7 s ACK 停顿 (每 6 min 1-2 次) = 真实 WiFi 抖动 → D22 WiFi 稳定 (用户 10-15: V0 必须搞定, 不能靠串口)</t>
         </is>
       </c>
       <c r="E92" s="7" t="inlineStr">
         <is>
-          <t>用户 10-15</t>
+          <t>~/realspin/tcp</t>
         </is>
       </c>
     </row>
@@ -10707,9 +10707,9 @@
       <c r="A93" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B93" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+      <c r="B93" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C93" s="7" t="inlineStr">
@@ -10719,12 +10719,12 @@
       </c>
       <c r="D93" s="7" t="inlineStr">
         <is>
-          <t>不插串口永远连得上: povreach 服务监护 + 硬件看门狗 (60 s, 防风暴) + 兜底热点 POV-&lt;板名&gt; (hostapd 静编, 192.168.77.1, 状态页可填 WiFi) + 30 min 无网重启; 失效模式表 16 行; 离线 9/9。排队上板故障演练 (8 项, 含 2 次看门狗复位)</t>
+          <t>用户: 不插串口也必须永远连得上, 彻底解决 (V0 必须) → D22 四层兜底开做: 服务监护 + 硬件看门狗 + 兜底热点 + 故障注入验收</t>
         </is>
       </c>
       <c r="E93" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach ee4a55c</t>
+          <t>用户 10-15</t>
         </is>
       </c>
     </row>
@@ -10739,17 +10739,17 @@
       </c>
       <c r="C94" s="7" t="inlineStr">
         <is>
-          <t>D20c</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D94" s="7" t="inlineStr">
         <is>
-          <t>内容帧率跟转速 voxlive --fps auto: 583 rpm 换帧间隔 std 23.4→0.1-0.9 ms (离线假转)。取舍: 板端默认 (max-fps 15, margin 0.9) 下 583 rpm 均匀但仅 9.7 fps; 板端 max-fps 20 + margin 1.0 → 19.4 fps 均匀。计划 D22 后上板验证 20/1.0 后改开机默认</t>
+          <t>不插串口永远连得上: povreach 服务监护 + 硬件看门狗 (60 s, 防风暴) + 兜底热点 POV-&lt;板名&gt; (hostapd 静编, 192.168.77.1, 状态页可填 WiFi) + 30 min 无网重启; 失效模式表 16 行; 离线 9/9。排队上板故障演练 (8 项, 含 2 次看门狗复位)</t>
         </is>
       </c>
       <c r="E94" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20c-fps 338eaaf</t>
+          <t>dr1v90 task/d22-reach ee4a55c</t>
         </is>
       </c>
     </row>
@@ -10759,7 +10759,7 @@
       </c>
       <c r="B95" s="6" t="inlineStr">
         <is>
-          <t>复验</t>
+          <t>交付</t>
         </is>
       </c>
       <c r="C95" s="7" t="inlineStr">
@@ -10769,12 +10769,12 @@
       </c>
       <c r="D95" s="7" t="inlineStr">
         <is>
-          <t>复验 F3 端到端节拍均匀度在主机忙 (D8 大仿真并行) 时不达标: 583 auto std 9.0/5.2 ms (门槛 3/4), 帧率正确; 主机计时抖动敏感, 先不合主线, 待空闲复验 + 上板实测定</t>
+          <t>内容帧率跟转速 voxlive --fps auto: 583 rpm 换帧间隔 std 23.4→0.1-0.9 ms (离线假转)。取舍: 板端默认 (max-fps 15, margin 0.9) 下 583 rpm 均匀但仅 9.7 fps; 板端 max-fps 20 + margin 1.0 → 19.4 fps 均匀。计划 D22 后上板验证 20/1.0 后改开机默认</t>
         </is>
       </c>
       <c r="E95" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d20c.v.log</t>
+          <t>dr1v90 task/d20c-fps 338eaaf</t>
         </is>
       </c>
     </row>
@@ -10784,22 +10784,22 @@
       </c>
       <c r="B96" s="6" t="inlineStr">
         <is>
-          <t>交付</t>
+          <t>复验</t>
         </is>
       </c>
       <c r="C96" s="7" t="inlineStr">
         <is>
-          <t>D8</t>
+          <t>D20c</t>
         </is>
       </c>
       <c r="D96" s="7" t="inlineStr">
         <is>
-          <t>V1 主控↔桥↔2260 联合仿真 0 错 (12/8 bit, 6 链×16 片, 训练锁定, 半圈换帧); 抓出并修 2 个回板必错 bug: 12-bit 字槽格式主控两 beat vs 桥紧排不一致 (改主控 PK12, 上行 195→110 µs/片) + 1 期切片器 NXG 未传 (160 宽按 192 算); 待: 1 期 12-bit 位流重综合 (hclk 余量原 +0.001 ns)</t>
+          <t>复验 F3 端到端节拍均匀度在主机忙 (D8 大仿真并行) 时不达标: 583 auto std 9.0/5.2 ms (门槛 3/4), 帧率正确; 主机计时抖动敏感, 先不合主线, 待空闲复验 + 上板实测定</t>
         </is>
       </c>
       <c r="E96" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d8-cosim 85dfe51</t>
+          <t>~/rv_d20c.v.log</t>
         </is>
       </c>
     </row>
@@ -10807,9 +10807,9 @@
       <c r="A97" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B97" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B97" s="6" t="inlineStr">
+        <is>
+          <t>交付</t>
         </is>
       </c>
       <c r="C97" s="7" t="inlineStr">
@@ -10819,12 +10819,12 @@
       </c>
       <c r="D97" s="7" t="inlineStr">
         <is>
-          <t>V1 联合仿真合主线 (新克隆复验 5/5; 合并回归 sim_v1/pls2047/D18/D19 通过, D19 O4 一次主机忙计时抖动重跑过); V1 回板就绪清单 ⑤ 达成</t>
+          <t>V1 主控↔桥↔2260 联合仿真 0 错 (12/8 bit, 6 链×16 片, 训练锁定, 半圈换帧); 抓出并修 2 个回板必错 bug: 12-bit 字槽格式主控两 beat vs 桥紧排不一致 (改主控 PK12, 上行 195→110 µs/片) + 1 期切片器 NXG 未传 (160 宽按 192 算); 待: 1 期 12-bit 位流重综合 (hclk 余量原 +0.001 ns)</t>
         </is>
       </c>
       <c r="E97" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>dr1v90 task/d8-cosim 85dfe51</t>
         </is>
       </c>
     </row>
@@ -10832,24 +10832,24 @@
       <c r="A98" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B98" s="6" t="inlineStr">
-        <is>
-          <t>测量</t>
+      <c r="B98" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C98" s="7" t="inlineStr">
         <is>
-          <t>D22/D20</t>
+          <t>D8</t>
         </is>
       </c>
       <c r="D98" s="7" t="inlineStr">
         <is>
-          <t>1 h 产品配置 (无对拍) 推流诊断: 换帧 14.64/s 软件损失 2.4% ✅, 间隔 p99 124 ms ✅, 长停顿 3.7‰ ✅, 最长 495 ms ❌ (门槛 267); PC→板 ping 16781/0 丢; &gt;0.5 s ACK 停顿 46 min 内 4 次 (最长 0.78 s), 同刻 PC→网关 RTT 165-275 ms = PC 侧 WiFi 抖动。周期 3 s 卡顿消失 (确认系对拍)。余项: 0.5-0.8 s 偶发抖动 (播放缓冲 vs 延迟取舍 / PC 有线或专用路由)</t>
+          <t>V1 联合仿真合主线 (新克隆复验 5/5; 合并回归 sim_v1/pls2047/D18/D19 通过, D19 O4 一次主机忙计时抖动重跑过); V1 回板就绪清单 ⑤ 达成</t>
         </is>
       </c>
       <c r="E98" s="7" t="inlineStr">
         <is>
-          <t>soak_runs/netdiag_1015_1814</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10857,24 +10857,24 @@
       <c r="A99" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B99" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B99" s="6" t="inlineStr">
+        <is>
+          <t>测量</t>
         </is>
       </c>
       <c r="C99" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D22/D20</t>
         </is>
       </c>
       <c r="D99" s="7" t="inlineStr">
         <is>
-          <t>换档位流 (REV 0x20471021) 上板起步即停摆 (档 0 未换档时写完 47 片后停, 换网格全超时), 仿真全过 → 硅上与仿真不同; D21b 开查根因。另: D21 上板收尾用 m90/up.sh 会让板子没 PL, 已重启回开机默认 (0x20471019 + QoS)</t>
+          <t>1 h 产品配置 (无对拍) 推流诊断: 换帧 14.64/s 软件损失 2.4% ✅, 间隔 p99 124 ms ✅, 长停顿 3.7‰ ✅, 最长 495 ms ❌ (门槛 267); PC→板 ping 16781/0 丢; &gt;0.5 s ACK 停顿 46 min 内 4 次 (最长 0.78 s), 同刻 PC→网关 RTT 165-275 ms = PC 侧 WiFi 抖动。周期 3 s 卡顿消失 (确认系对拍)。余项: 0.5-0.8 s 偶发抖动 (播放缓冲 vs 延迟取舍 / PC 有线或专用路由)</t>
         </is>
       </c>
       <c r="E99" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d21.board.log</t>
+          <t>soak_runs/netdiag_1015_1814</t>
         </is>
       </c>
     </row>
@@ -10889,17 +10889,17 @@
       </c>
       <c r="C100" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D100" s="7" t="inlineStr">
         <is>
-          <t>新克隆离线 O6 误 FAIL: hostapd/povreach 二进制 git 模式 644, WSL 本地盘克隆不可执行, qemu 静默拒绝 (板上 autorun 有 chmod, 不受影响); 已修 (git +x, verify chmod), 重跑后自动上板演练</t>
+          <t>换档位流 (REV 0x20471021) 上板起步即停摆 (档 0 未换档时写完 47 片后停, 换网格全超时), 仿真全过 → 硅上与仿真不同; D21b 开查根因。另: D21 上板收尾用 m90/up.sh 会让板子没 PL, 已重启回开机默认 (0x20471019 + QoS)</t>
         </is>
       </c>
       <c r="E100" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach</t>
+          <t>~/rv_d21.board.log</t>
         </is>
       </c>
     </row>
@@ -10919,7 +10919,7 @@
       </c>
       <c r="D101" s="7" t="inlineStr">
         <is>
-          <t>首轮上板演练 9 项误 FAIL = 验收脚本 info() 把板上 board_d22.sh info 的非 0 退出码当失败 (内容正常), settle/wait_healthy 恒失败; 板子本身正常 (装好开机 healthy, povreach managed, 看门狗 armed)。已修, 单独重跑全套演练 (~80 min); 期间 D21 取证因同时上板被干扰, 待 D22 后单独跑</t>
+          <t>新克隆离线 O6 误 FAIL: hostapd/povreach 二进制 git 模式 644, WSL 本地盘克隆不可执行, qemu 静默拒绝 (板上 autorun 有 chmod, 不受影响); 已修 (git +x, verify chmod), 重跑后自动上板演练</t>
         </is>
       </c>
       <c r="E101" s="7" t="inlineStr">
@@ -10932,9 +10932,9 @@
       <c r="A102" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B102" s="6" t="inlineStr">
-        <is>
-          <t>验证</t>
+      <c r="B102" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C102" s="7" t="inlineStr">
@@ -10944,12 +10944,12 @@
       </c>
       <c r="D102" s="7" t="inlineStr">
         <is>
-          <t>第二轮上板演练 (单独): 杀 sshd/mdns/povnetd 27-72 s 自愈找回 ✅; 错 SSID → 兜底热点 → 自己回公司网 ✅ (但 23.5 min, 目标 ≤10); 杀 wpa/关网卡、装后重启: 板子恢复了但 mDNS 按名字 240 s 内找不回 ❌ (缓存 IP 可连); 看门狗复位发生但晚于测试判定、卡上未记非正常结束 ❌。交回 D22 agent 修 (mDNS 找回为主)</t>
+          <t>首轮上板演练 9 项误 FAIL = 验收脚本 info() 把板上 board_d22.sh info 的非 0 退出码当失败 (内容正常), settle/wait_healthy 恒失败; 板子本身正常 (装好开机 healthy, povreach managed, 看门狗 armed)。已修, 单独重跑全套演练 (~80 min); 期间 D21 取证因同时上板被干扰, 待 D22 后单独跑</t>
         </is>
       </c>
       <c r="E102" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d22.board2.log</t>
+          <t>dr1v90 task/d22-reach</t>
         </is>
       </c>
     </row>
@@ -10959,22 +10959,22 @@
       </c>
       <c r="B103" s="6" t="inlineStr">
         <is>
-          <t>根因</t>
+          <t>验证</t>
         </is>
       </c>
       <c r="C103" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D103" s="7" t="inlineStr">
         <is>
-          <t>板上取证: 显示每圈取满 142 片, 但 s3rt_sys 旁听只认片号 0..47 → PL 每圈 48 触发后停摆; 不带档位 / 补 sub10 都一样 → RTL 旁听上限 (D21 改为按 FBO) 问题。交回 D21b 修 RTL; 板子已重启回默认 0x20471019</t>
+          <t>第二轮上板演练 (单独): 杀 sshd/mdns/povnetd 27-72 s 自愈找回 ✅; 错 SSID → 兜底热点 → 自己回公司网 ✅ (但 23.5 min, 目标 ≤10); 杀 wpa/关网卡、装后重启: 板子恢复了但 mDNS 按名字 240 s 内找不回 ❌ (缓存 IP 可连); 看门狗复位发生但晚于测试判定、卡上未记非正常结束 ❌。交回 D22 agent 修 (mDNS 找回为主)</t>
         </is>
       </c>
       <c r="E103" s="7" t="inlineStr">
         <is>
-          <t>~/d21b_forensic.log</t>
+          <t>~/rv_d22.board2.log</t>
         </is>
       </c>
     </row>
@@ -10989,17 +10989,17 @@
       </c>
       <c r="C104" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D104" s="7" t="inlineStr">
         <is>
-          <t>按名字找不回的根因: povmdns 在地址回来/重关联时不重新发 IGMP 报告 (重复入组 EADDRINUSE 无报告), 企业 AP 只把组播转给报告过的站点 → mDNS 查询数分钟到不了板。修: 重关联/地址变化时退组再入组 + 宣告 (0/1/3/7/15/30 s) + 每 60 s 刷新; 看门狗读回实际超时并减半到 ≤60 s; 卡上记非正常结束。离线 10/10, 上板复验中</t>
+          <t>板上取证: 显示每圈取满 142 片, 但 s3rt_sys 旁听只认片号 0..47 → PL 每圈 48 触发后停摆; 不带档位 / 补 sub10 都一样 → RTL 旁听上限 (D21 改为按 FBO) 问题。交回 D21b 修 RTL; 板子已重启回默认 0x20471019</t>
         </is>
       </c>
       <c r="E104" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach 0d1da09</t>
+          <t>~/d21b_forensic.log</t>
         </is>
       </c>
     </row>
@@ -11009,7 +11009,7 @@
       </c>
       <c r="B105" s="6" t="inlineStr">
         <is>
-          <t>验证</t>
+          <t>根因</t>
         </is>
       </c>
       <c r="C105" s="7" t="inlineStr">
@@ -11019,12 +11019,12 @@
       </c>
       <c r="D105" s="7" t="inlineStr">
         <is>
-          <t>第三轮上板演练 9/10: 装后重启 24 s 按名字找回 ✅ (上轮找不回); sshd/mdns/povnetd 杀掉 38-72 s ✅; 关网卡 191 s ✅; 错 SSID→热点→自动回 543 s ✅ (上轮 1411); 看门狗复位 reachkill 54 s / netdstop 213 s 且记非正常结束 ✅ (实际超时 32 s); 仅 kill wpa_supplicant 240 s 内未找回 ❌ (随后恢复), 单独重跑定位中</t>
+          <t>按名字找不回的根因: povmdns 在地址回来/重关联时不重新发 IGMP 报告 (重复入组 EADDRINUSE 无报告), 企业 AP 只把组播转给报告过的站点 → mDNS 查询数分钟到不了板。修: 重关联/地址变化时退组再入组 + 宣告 (0/1/3/7/15/30 s) + 每 60 s 刷新; 看门狗读回实际超时并减半到 ≤60 s; 卡上记非正常结束。离线 10/10, 上板复验中</t>
         </is>
       </c>
       <c r="E105" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d22b.board.log</t>
+          <t>dr1v90 task/d22-reach 0d1da09</t>
         </is>
       </c>
     </row>
@@ -11034,7 +11034,7 @@
       </c>
       <c r="B106" s="6" t="inlineStr">
         <is>
-          <t>交付</t>
+          <t>验证</t>
         </is>
       </c>
       <c r="C106" s="7" t="inlineStr">
@@ -11044,12 +11044,12 @@
       </c>
       <c r="D106" s="7" t="inlineStr">
         <is>
-          <t>povnetd 1.2: wpa 进程没了/卡死/接口 down 立即重连 (原来一律等 60 s, 且 60 s 后的重连反把已自愈的连接打断 → 73-240+ s 且不稳); 只丢包仍按 60 s 防误重连; 关键事件写卡 (复位后可查); verify wpakill/ifdown 各连跑 3 次、120 s 内按名字找回。离线 11/11, 上板全套复验中</t>
+          <t>第三轮上板演练 9/10: 装后重启 24 s 按名字找回 ✅ (上轮找不回); sshd/mdns/povnetd 杀掉 38-72 s ✅; 关网卡 191 s ✅; 错 SSID→热点→自动回 543 s ✅ (上轮 1411); 看门狗复位 reachkill 54 s / netdstop 213 s 且记非正常结束 ✅ (实际超时 32 s); 仅 kill wpa_supplicant 240 s 内未找回 ❌ (随后恢复), 单独重跑定位中</t>
         </is>
       </c>
       <c r="E106" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach e438a12</t>
+          <t>~/rv_d22b.board.log</t>
         </is>
       </c>
     </row>
@@ -11059,47 +11059,47 @@
       </c>
       <c r="B107" s="6" t="inlineStr">
         <is>
-          <t>根因</t>
+          <t>交付</t>
         </is>
       </c>
       <c r="C107" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D107" s="7" t="inlineStr">
         <is>
-          <t>停摆根因不在 RTL: voxslice --pl 从不写显示 0x0C sub01 (bpp3), 重新加载位流后显示按 1-bit 片距 0x3000 取片, 旁听按 0x9000 片首只认 1/3 → 每圈 48 触发卡死。主线同有此隐患 (默认开机靠别的程序先写对)。修: pl_setup 先写 sub01; 仿真 +NOBPP3 复现与板上一致; 位流不变。离线 12/12, 排在 D22 后上板</t>
+          <t>povnetd 1.2: wpa 进程没了/卡死/接口 down 立即重连 (原来一律等 60 s, 且 60 s 后的重连反把已自愈的连接打断 → 73-240+ s 且不稳); 只丢包仍按 60 s 防误重连; 关键事件写卡 (复位后可查); verify wpakill/ifdown 各连跑 3 次、120 s 内按名字找回。离线 11/11, 上板全套复验中</t>
         </is>
       </c>
       <c r="E107" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d21-nband 084bba3</t>
+          <t>dr1v90 task/d22-reach e438a12</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="17" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B108" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+        <v>46310</v>
+      </c>
+      <c r="B108" s="6" t="inlineStr">
+        <is>
+          <t>根因</t>
         </is>
       </c>
       <c r="C108" s="7" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D108" s="7" t="inlineStr">
         <is>
-          <t>上行出口全量复验 45/0, 合主线</t>
+          <t>停摆根因不在 RTL: voxslice --pl 从不写显示 0x0C sub01 (bpp3), 重新加载位流后显示按 1-bit 片距 0x3000 取片, 旁听按 0x9000 片首只认 1/3 → 每圈 48 触发卡死。主线同有此隐患 (默认开机靠别的程序先写对)。修: pl_setup 先写 sub01; 仿真 +NOBPP3 复现与板上一致; 位流不变。离线 12/12, 排在 D22 后上板</t>
         </is>
       </c>
       <c r="E108" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 fdb4de6</t>
+          <t>dr1v90 task/d21-nband 084bba3</t>
         </is>
       </c>
     </row>
@@ -11107,24 +11107,24 @@
       <c r="A109" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B109" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B109" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C109" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="D109" s="7" t="inlineStr">
         <is>
-          <t>PL 切片上板: 与 CPU 逐字节一致、30 min 无停摆, 但内容帧率 4.2&lt;15, 退回</t>
+          <t>上行出口全量复验 45/0, 合主线</t>
         </is>
       </c>
       <c r="E109" s="7" t="inlineStr">
         <is>
-          <t>scratchpad/v_pls4_board.log</t>
+          <t>dr1v90 fdb4de6</t>
         </is>
       </c>
     </row>
@@ -11132,24 +11132,24 @@
       <c r="A110" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B110" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B110" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C110" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D110" s="7" t="inlineStr">
         <is>
-          <t>30 Hz 带载迟到+掉片 3.7% (空载 0.2% 来自旧 netguard), 归因测试中</t>
+          <t>PL 切片上板: 与 CPU 逐字节一致、30 min 无停摆, 但内容帧率 4.2&lt;15, 退回</t>
         </is>
       </c>
       <c r="E110" s="7" t="inlineStr">
         <is>
-          <t>project_ddr_budget_by_phase_1013</t>
+          <t>scratchpad/v_pls4_board.log</t>
         </is>
       </c>
     </row>
@@ -11169,7 +11169,7 @@
       </c>
       <c r="D111" s="7" t="inlineStr">
         <is>
-          <t>纯切片带载约 21 min 停摆; 无负载浸泡 2×30 min 不停摆</t>
+          <t>30 Hz 带载迟到+掉片 3.7% (空载 0.2% 来自旧 netguard), 归因测试中</t>
         </is>
       </c>
       <c r="E111" s="7" t="inlineStr">
@@ -11182,24 +11182,24 @@
       <c r="A112" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B112" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B112" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C112" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D112" s="7" t="inlineStr">
         <is>
-          <t>用户定目标: 复位到亮起 ≤12 s, 找板 ≤20 s</t>
+          <t>纯切片带载约 21 min 停摆; 无负载浸泡 2×30 min 不停摆</t>
         </is>
       </c>
       <c r="E112" s="7" t="inlineStr">
         <is>
-          <t>project_short_term_delivery_1013</t>
+          <t>project_ddr_budget_by_phase_1013</t>
         </is>
       </c>
     </row>
@@ -11207,24 +11207,24 @@
       <c r="A113" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B113" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B113" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C113" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D113" s="7" t="inlineStr">
         <is>
-          <t>找到 PL 切片器带载停摆根因: 零列描述符丢失 (公共核, 2260 也有) + pop 握手串片, 已修</t>
+          <t>用户定目标: 复位到亮起 ≤12 s, 找板 ≤20 s</t>
         </is>
       </c>
       <c r="E113" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 debd3cd</t>
+          <t>project_short_term_delivery_1013</t>
         </is>
       </c>
     </row>
@@ -11232,9 +11232,9 @@
       <c r="A114" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B114" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B114" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C114" s="7" t="inlineStr">
@@ -11244,12 +11244,12 @@
       </c>
       <c r="D114" s="7" t="inlineStr">
         <is>
-          <t>上板 60 min 带载 0 停摆、逐字节一致、late 0; 帧率 13.8 差 0.5 退回</t>
+          <t>找到 PL 切片器带载停摆根因: 零列描述符丢失 (公共核, 2260 也有) + pop 握手串片, 已修</t>
         </is>
       </c>
       <c r="E114" s="7" t="inlineStr">
         <is>
-          <t>scratchpad v_pls6_board.log</t>
+          <t>dr1v90 task/pls-2047 debd3cd</t>
         </is>
       </c>
     </row>
@@ -11257,9 +11257,9 @@
       <c r="A115" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B115" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B115" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C115" s="7" t="inlineStr">
@@ -11269,12 +11269,12 @@
       </c>
       <c r="D115" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 实时切片上板全过: 60 min 带载 0 停摆, 帧率 15.0, 与 CPU 逐字节一致</t>
+          <t>上板 60 min 带载 0 停摆、逐字节一致、late 0; 帧率 13.8 差 0.5 退回</t>
         </is>
       </c>
       <c r="E115" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 782e9e3</t>
+          <t>scratchpad v_pls6_board.log</t>
         </is>
       </c>
     </row>
@@ -11282,24 +11282,24 @@
       <c r="A116" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B116" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B116" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C116" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D116" s="7" t="inlineStr">
         <is>
-          <t>DDR 慢读根因: 每圈约 1/3 角度每取一列都换行, 两类 CPU 负载叠加越阈值 (0.002%→3%); 建议网格 4×4 分块</t>
+          <t>2047 PL 实时切片上板全过: 60 min 带载 0 停摆, 帧率 15.0, 与 CPU 逐字节一致</t>
         </is>
       </c>
       <c r="E116" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d16-ddr 539d303</t>
+          <t>dr1v90 task/pls-2047 782e9e3</t>
         </is>
       </c>
     </row>
@@ -11307,24 +11307,24 @@
       <c r="A117" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B117" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B117" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C117" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D117" s="7" t="inlineStr">
         <is>
-          <t>用户定: 子 agent 并行 ≤5 (周额度); 跑完的 agent 关掉</t>
+          <t>DDR 慢读根因: 每圈约 1/3 角度每取一列都换行, 两类 CPU 负载叠加越阈值 (0.002%→3%); 建议网格 4×4 分块</t>
         </is>
       </c>
       <c r="E117" s="7" t="inlineStr">
         <is>
-          <t>feedback_save_weekly_quota</t>
+          <t>dr1v90 task/d16-ddr 539d303</t>
         </is>
       </c>
     </row>
@@ -11332,24 +11332,24 @@
       <c r="A118" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B118" s="19" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+      <c r="B118" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C118" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D118" s="7" t="inlineStr">
         <is>
-          <t>V0 出口清单: PL 切片上板通过 (D2) 可打勾</t>
+          <t>用户定: 子 agent 并行 ≤5 (周额度); 跑完的 agent 关掉</t>
         </is>
       </c>
       <c r="E118" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 782e9e3</t>
+          <t>feedback_save_weekly_quota</t>
         </is>
       </c>
     </row>
@@ -11357,24 +11357,24 @@
       <c r="A119" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B119" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B119" s="19" t="inlineStr">
+        <is>
+          <t>里程碑</t>
         </is>
       </c>
       <c r="C119" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D119" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 实时切片合进主线 (含公共核两处 bug 修复); D3 上行档位流需按新核重综合</t>
+          <t>V0 出口清单: PL 切片上板通过 (D2) 可打勾</t>
         </is>
       </c>
       <c r="E119" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 2364e5c</t>
+          <t>dr1v90 task/pls-2047 782e9e3</t>
         </is>
       </c>
     </row>
@@ -11382,9 +11382,9 @@
       <c r="A120" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B120" s="19" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+      <c r="B120" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C120" s="7" t="inlineStr">
@@ -11394,12 +11394,12 @@
       </c>
       <c r="D120" s="7" t="inlineStr">
         <is>
-          <t>PL 硬件切片首次实转上屏 (650 rpm, 完成率 100%, CPU 82% 空闲), 用户确认与 CPU 切片无区别</t>
+          <t>2047 PL 实时切片合进主线 (含公共核两处 bug 修复); D3 上行档位流需按新核重综合</t>
         </is>
       </c>
       <c r="E120" s="7" t="inlineStr">
         <is>
-          <t>用户在场实转</t>
+          <t>dr1v90 2364e5c</t>
         </is>
       </c>
     </row>
@@ -11407,24 +11407,24 @@
       <c r="A121" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B121" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B121" s="19" t="inlineStr">
+        <is>
+          <t>里程碑</t>
         </is>
       </c>
       <c r="C121" s="7" t="inlineStr">
         <is>
-          <t>D18</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D121" s="7" t="inlineStr">
         <is>
-          <t>用户定: 只保留 PL 切片, 固化开机流程, CPU 切片只留应急退路</t>
+          <t>PL 硬件切片首次实转上屏 (650 rpm, 完成率 100%, CPU 82% 空闲), 用户确认与 CPU 切片无区别</t>
         </is>
       </c>
       <c r="E121" s="7" t="inlineStr">
         <is>
-          <t>用户 10-14</t>
+          <t>用户在场实转</t>
         </is>
       </c>
     </row>
@@ -11432,9 +11432,9 @@
       <c r="A122" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B122" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B122" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C122" s="7" t="inlineStr">
@@ -11444,12 +11444,12 @@
       </c>
       <c r="D122" s="7" t="inlineStr">
         <is>
-          <t>开机默认 PL 切片合主线: 上电基础显示 → 推流显示推流 → 停推 5 min 回基础演示; CPU 只留应急退路</t>
+          <t>用户定: 只保留 PL 切片, 固化开机流程, CPU 切片只留应急退路</t>
         </is>
       </c>
       <c r="E122" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d18-pl-default d35c6d4</t>
+          <t>用户 10-14</t>
         </is>
       </c>
     </row>
@@ -11457,24 +11457,24 @@
       <c r="A123" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B123" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B123" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C123" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D18</t>
         </is>
       </c>
       <c r="D123" s="7" t="inlineStr">
         <is>
-          <t>用户定目标放宽: 亮起 ≤12.5 s / 找板 ≤21 s; V0 出口 ④ 达成</t>
+          <t>开机默认 PL 切片合主线: 上电基础显示 → 推流显示推流 → 停推 5 min 回基础演示; CPU 只留应急退路</t>
         </is>
       </c>
       <c r="E123" s="7" t="inlineStr">
         <is>
-          <t>用户 10-14</t>
+          <t>dr1v90 task/d18-pl-default d35c6d4</t>
         </is>
       </c>
     </row>
@@ -11482,24 +11482,24 @@
       <c r="A124" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B124" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B124" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C124" s="7" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D124" s="7" t="inlineStr">
         <is>
-          <t>无串口远程运维合主线: 升级坏包 (含断网包) 自动回滚后板子能按名字找回; 网络守护不再造成切片迟到 (旧版每分钟 2061 次 → 0); V0 出口 ⑤ 达成</t>
+          <t>用户定目标放宽: 亮起 ≤12.5 s / 找板 ≤21 s; V0 出口 ④ 达成</t>
         </is>
       </c>
       <c r="E124" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 dee9be6</t>
+          <t>用户 10-14</t>
         </is>
       </c>
     </row>
@@ -11507,24 +11507,24 @@
       <c r="A125" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B125" s="6" t="inlineStr">
-        <is>
-          <t>根因</t>
+      <c r="B125" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C125" s="7" t="inlineStr">
         <is>
-          <t>D15b</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="D125" s="7" t="inlineStr">
         <is>
-          <t>32 bit PL 全黑: 板端写 LUT 基址仍用 16 bit 布局偏移, PL 把网格当角度表读; 已修 308d1bb, 待上板</t>
+          <t>无串口远程运维合主线: 升级坏包 (含断网包) 自动回滚后板子能按名字找回; 网络守护不再造成切片迟到 (旧版每分钟 2061 次 → 0); V0 出口 ⑤ 达成</t>
         </is>
       </c>
       <c r="E125" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d15b-color-p2</t>
+          <t>dr1v90 dee9be6</t>
         </is>
       </c>
     </row>
@@ -11532,24 +11532,24 @@
       <c r="A126" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B126" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B126" s="6" t="inlineStr">
+        <is>
+          <t>根因</t>
         </is>
       </c>
       <c r="C126" s="7" t="inlineStr">
         <is>
-          <t>D15</t>
+          <t>D15b</t>
         </is>
       </c>
       <c r="D126" s="7" t="inlineStr">
         <is>
-          <t>WiFi 端 12-bit 通路合主线: 32 bit 像素 PL/CPU 与 CPU 逐字节一致, 2047 上跑通; V0 出口 ⑦ 达成 (7/8)。已知限制: 32 bit 只到 10.83 rps (16.15 rps 时完成率 82-91%)</t>
+          <t>32 bit PL 全黑: 板端写 LUT 基址仍用 16 bit 布局偏移, PL 把网格当角度表读; 已修 308d1bb, 待上板</t>
         </is>
       </c>
       <c r="E126" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 3a41eb7</t>
+          <t>dr1v90 task/d15b-color-p2</t>
         </is>
       </c>
     </row>
@@ -11557,24 +11557,24 @@
       <c r="A127" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B127" s="6" t="inlineStr">
-        <is>
-          <t>开始</t>
+      <c r="B127" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C127" s="7" t="inlineStr">
         <is>
-          <t>KR7.2</t>
+          <t>D15</t>
         </is>
       </c>
       <c r="D127" s="7" t="inlineStr">
         <is>
-          <t>8 h 无人值守长跑开跑 19:20 (假转黑屏, 主线 voxslice 0.6 + 卡上 PL 默认; 推 40 min/停 7 min 循环; 判据 S1-S9; 15 min 试跑 9/9)</t>
+          <t>WiFi 端 12-bit 通路合主线: 32 bit 像素 PL/CPU 与 CPU 逐字节一致, 2047 上跑通; V0 出口 ⑦ 达成 (7/8)。已知限制: 32 bit 只到 10.83 rps (16.15 rps 时完成率 82-91%)</t>
         </is>
       </c>
       <c r="E127" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 26e69ec soak8h</t>
+          <t>dr1v90 3a41eb7</t>
         </is>
       </c>
     </row>
@@ -11582,24 +11582,24 @@
       <c r="A128" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B128" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B128" s="6" t="inlineStr">
+        <is>
+          <t>开始</t>
         </is>
       </c>
       <c r="C128" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>KR7.2</t>
         </is>
       </c>
       <c r="D128" s="7" t="inlineStr">
         <is>
-          <t>用户批准 QoS 寄存器写入 + 网格 4×4 分块 (D16b 开做, 离线); 长跑后在 2047 做对照</t>
+          <t>8 h 无人值守长跑开跑 19:20 (假转黑屏, 主线 voxslice 0.6 + 卡上 PL 默认; 推 40 min/停 7 min 循环; 判据 S1-S9; 15 min 试跑 9/9)</t>
         </is>
       </c>
       <c r="E128" s="7" t="inlineStr">
         <is>
-          <t>用户 10-14</t>
+          <t>dr1v90 26e69ec soak8h</t>
         </is>
       </c>
     </row>
@@ -11607,49 +11607,49 @@
       <c r="A129" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B129" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B129" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C129" s="7" t="inlineStr">
         <is>
-          <t>KR7.2</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D129" s="7" t="inlineStr">
         <is>
-          <t>长跑第 6 段企业 WiFi 踢线 ~5 s, 推流端 voxlive 不重连直接退出 (板端处理正确); 修: voxlive 断线自动重连 5cbe79f; 23:45 重开 8 h</t>
+          <t>用户批准 QoS 寄存器写入 + 网格 4×4 分块 (D16b 开做, 离线); 长跑后在 2047 做对照</t>
         </is>
       </c>
       <c r="E129" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 5cbe79f</t>
+          <t>用户 10-14</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="17" t="n">
-        <v>46308</v>
-      </c>
-      <c r="B130" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46309</v>
+      </c>
+      <c r="B130" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C130" s="7" t="inlineStr">
         <is>
-          <t>E6</t>
+          <t>KR7.2</t>
         </is>
       </c>
       <c r="D130" s="7" t="inlineStr">
         <is>
-          <t>按名字找板 (mDNS) 完成：无串口自重启后 34 s 按名字找到并 ssh 上</t>
+          <t>长跑第 6 段企业 WiFi 踢线 ~5 s, 推流端 voxlive 不重连直接退出 (板端处理正确); 修: voxlive 断线自动重连 5cbe79f; 23:45 重开 8 h</t>
         </is>
       </c>
       <c r="E130" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 b0f6b5d</t>
+          <t>dr1v90 5cbe79f</t>
         </is>
       </c>
     </row>
@@ -11664,17 +11664,17 @@
       </c>
       <c r="C131" s="7" t="inlineStr">
         <is>
-          <t>E7</t>
+          <t>E6</t>
         </is>
       </c>
       <c r="D131" s="7" t="inlineStr">
         <is>
-          <t>纯切片 30 Hz 位流第一次上硅 D'0–D'3，尾部 late 0.2%，暂停 netguard 后 late/miss 为 0</t>
+          <t>按名字找板 (mDNS) 完成：无串口自重启后 34 s 按名字找到并 ssh 上</t>
         </is>
       </c>
       <c r="E131" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 71d006f / 473abcf</t>
+          <t>dr1v90 b0f6b5d</t>
         </is>
       </c>
     </row>
@@ -11689,17 +11689,17 @@
       </c>
       <c r="C132" s="7" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>E7</t>
         </is>
       </c>
       <c r="D132" s="7" t="inlineStr">
         <is>
-          <t>主机实时推流完成：10 分钟 15.0 fps，NAK 0 / forced 0</t>
+          <t>纯切片 30 Hz 位流第一次上硅 D'0–D'3，尾部 late 0.2%，暂停 netguard 后 late/miss 为 0</t>
         </is>
       </c>
       <c r="E132" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 596b191</t>
+          <t>dr1v90 71d006f / 473abcf</t>
         </is>
       </c>
     </row>
@@ -11707,9 +11707,9 @@
       <c r="A133" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B133" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B133" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C133" s="7" t="inlineStr">
@@ -11719,12 +11719,12 @@
       </c>
       <c r="D133" s="7" t="inlineStr">
         <is>
-          <t>第一次上板端到端延迟 p50 114 ms 未过（停等发送），改发送流水线后降到 84.7 ms</t>
+          <t>主机实时推流完成：10 分钟 15.0 fps，NAK 0 / forced 0</t>
         </is>
       </c>
       <c r="E133" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 60c619a / 596b191</t>
+          <t>dr1v90 596b191</t>
         </is>
       </c>
     </row>
@@ -11732,9 +11732,9 @@
       <c r="A134" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B134" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B134" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C134" s="7" t="inlineStr">
@@ -11744,12 +11744,12 @@
       </c>
       <c r="D134" s="7" t="inlineStr">
         <is>
-          <t>主会话新克隆独立复验离线+上板全过，合主线（延迟 p50 95 ms / p99 236.6 ms）</t>
+          <t>第一次上板端到端延迟 p50 114 ms 未过（停等发送），改发送流水线后降到 84.7 ms</t>
         </is>
       </c>
       <c r="E134" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 9bf16ad</t>
+          <t>dr1v90 60c619a / 596b191</t>
         </is>
       </c>
     </row>
@@ -11757,24 +11757,24 @@
       <c r="A135" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B135" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B135" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C135" s="7" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="D135" s="7" t="inlineStr">
         <is>
-          <t>桥接收核对 12-bit 第一次复验 FAIL（新克隆无可执行位），退回</t>
+          <t>主会话新克隆独立复验离线+上板全过，合主线（延迟 p50 95 ms / p99 236.6 ms）</t>
         </is>
       </c>
       <c r="E135" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 9bf16ad</t>
         </is>
       </c>
     </row>
@@ -11782,9 +11782,9 @@
       <c r="A136" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B136" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B136" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C136" s="7" t="inlineStr">
@@ -11794,12 +11794,12 @@
       </c>
       <c r="D136" s="7" t="inlineStr">
         <is>
-          <t>桥接收核对 12-bit 复验 PASS，合主线</t>
+          <t>桥接收核对 12-bit 第一次复验 FAIL（新克隆无可执行位），退回</t>
         </is>
       </c>
       <c r="E136" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 6a373d3</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -11814,17 +11814,17 @@
       </c>
       <c r="C137" s="7" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="D137" s="7" t="inlineStr">
         <is>
-          <t>桥驱动 2260 1 期 6 链 24 Hz 12-bit 复验 ALL PASS，合主线</t>
+          <t>桥接收核对 12-bit 复验 PASS，合主线</t>
         </is>
       </c>
       <c r="E137" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 cdf49c6</t>
+          <t>dr1v90 6a373d3</t>
         </is>
       </c>
     </row>
@@ -11832,9 +11832,9 @@
       <c r="A138" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B138" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B138" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C138" s="7" t="inlineStr">
@@ -11844,12 +11844,12 @@
       </c>
       <c r="D138" s="7" t="inlineStr">
         <is>
-          <t>6 链 4296 片/s 能跑但余量仅 0.40%，瓶颈是桥→2260 链路；留 10% 需 ≤3921 片/s，待用户定</t>
+          <t>桥驱动 2260 1 期 6 链 24 Hz 12-bit 复验 ALL PASS，合主线</t>
         </is>
       </c>
       <c r="E138" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 cdf49c6</t>
         </is>
       </c>
     </row>
@@ -11869,7 +11869,7 @@
       </c>
       <c r="D139" s="7" t="inlineStr">
         <is>
-          <t>发现 10-10 验证板 profile 寄存器在 166.67 MHz 下超规格（GCLK 667&gt;600），1 期表已改</t>
+          <t>6 链 4296 片/s 能跑但余量仅 0.40%，瓶颈是桥→2260 链路；留 10% 需 ≤3921 片/s，待用户定</t>
         </is>
       </c>
       <c r="E139" s="7" t="inlineStr">
@@ -11882,24 +11882,24 @@
       <c r="A140" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B140" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B140" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C140" s="7" t="inlineStr">
         <is>
-          <t>D6</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="D140" s="7" t="inlineStr">
         <is>
-          <t>几何 LUT 生成器逐字节复现 2047 s3lut，verify 22 PASS，合主线</t>
+          <t>发现 10-10 验证板 profile 寄存器在 166.67 MHz 下超规格（GCLK 667&gt;600），1 期表已改</t>
         </is>
       </c>
       <c r="E140" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 44ed2cd</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -11907,24 +11907,24 @@
       <c r="A141" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B141" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B141" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C141" s="7" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>D6</t>
         </is>
       </c>
       <c r="D141" s="7" t="inlineStr">
         <is>
-          <t>转子运维首次复验 T5 偶发 FAIL，退回返工</t>
+          <t>几何 LUT 生成器逐字节复现 2047 s3lut，verify 22 PASS，合主线</t>
         </is>
       </c>
       <c r="E141" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 44ed2cd</t>
         </is>
       </c>
     </row>
@@ -11932,24 +11932,24 @@
       <c r="A142" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B142" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B142" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C142" s="7" t="inlineStr">
         <is>
-          <t>D14</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="D142" s="7" t="inlineStr">
         <is>
-          <t>10 类内容 + 手机网页遥控离线复验 ALL PASS，用户实转看过（尚未正式上板验收）</t>
+          <t>转子运维首次复验 T5 偶发 FAIL，退回返工</t>
         </is>
       </c>
       <c r="E142" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 ffbfeeb</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -11964,17 +11964,17 @@
       </c>
       <c r="C143" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D14</t>
         </is>
       </c>
       <c r="D143" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 切片离线复验 26/0，待上板（之后 9ba9af0 测试用例过时 26/27 待修）</t>
+          <t>10 类内容 + 手机网页遥控离线复验 ALL PASS，用户实转看过（尚未正式上板验收）</t>
         </is>
       </c>
       <c r="E143" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 ffbfeeb</t>
         </is>
       </c>
     </row>
@@ -11982,19 +11982,19 @@
       <c r="A144" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B144" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B144" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C144" s="7" t="inlineStr">
         <is>
-          <t>D12</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D144" s="7" t="inlineStr">
         <is>
-          <t>延迟降低上板复验 FAIL：B1 翻页 14.39&lt;15 fps，p99 225 ms，退回</t>
+          <t>2047 PL 切片离线复验 26/0，待上板（之后 9ba9af0 测试用例过时 26/27 待修）</t>
         </is>
       </c>
       <c r="E144" s="7" t="inlineStr">
@@ -12007,9 +12007,9 @@
       <c r="A145" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B145" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B145" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C145" s="7" t="inlineStr">
@@ -12019,12 +12019,12 @@
       </c>
       <c r="D145" s="7" t="inlineStr">
         <is>
-          <t>第二次上板仍未过，根因晚间 WiFi 尾巴（p99 334 vs 白天 48 ms）；判据改为调度问题 0 + 网络晚到 ≤1%，明早主机空闲复测</t>
+          <t>延迟降低上板复验 FAIL：B1 翻页 14.39&lt;15 fps，p99 225 ms，退回</t>
         </is>
       </c>
       <c r="E145" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 764f81d</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12032,24 +12032,24 @@
       <c r="A146" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B146" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B146" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C146" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D12</t>
         </is>
       </c>
       <c r="D146" s="7" t="inlineStr">
         <is>
-          <t>启动提速上板 FAIL 11 项，但改进已装板保留（6 次重启正常），退回继续压启动时间</t>
+          <t>第二次上板仍未过，根因晚间 WiFi 尾巴（p99 334 vs 白天 48 ms）；判据改为调度问题 0 + 网络晚到 ≤1%，明早主机空闲复测</t>
         </is>
       </c>
       <c r="E146" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 764f81d</t>
         </is>
       </c>
     </row>
@@ -12057,9 +12057,9 @@
       <c r="A147" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B147" s="19" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+      <c r="B147" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C147" s="7" t="inlineStr">
@@ -12069,12 +12069,12 @@
       </c>
       <c r="D147" s="7" t="inlineStr">
         <is>
-          <t>启动提速两轮后：复位→0° 片亮起 38.7→20.1→15.8 s，找板 34→30→25.6 s</t>
+          <t>启动提速上板 FAIL 11 项，但改进已装板保留（6 次重启正常），退回继续压启动时间</t>
         </is>
       </c>
       <c r="E147" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d13-boot fdbb217</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12082,9 +12082,9 @@
       <c r="A148" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B148" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B148" s="19" t="inlineStr">
+        <is>
+          <t>里程碑</t>
         </is>
       </c>
       <c r="C148" s="7" t="inlineStr">
@@ -12094,12 +12094,12 @@
       </c>
       <c r="D148" s="7" t="inlineStr">
         <is>
-          <t>第二步（bootdelay 0 / 精简 uInitrd）写启动文件被权限系统拒绝，需用户明早本人批准后执行</t>
+          <t>启动提速两轮后：复位→0° 片亮起 38.7→20.1→15.8 s，找板 34→30→25.6 s</t>
         </is>
       </c>
       <c r="E148" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 task/d13-boot fdbb217</t>
         </is>
       </c>
     </row>
@@ -12107,24 +12107,24 @@
       <c r="A149" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B149" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B149" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C149" s="7" t="inlineStr">
         <is>
-          <t>D15</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D149" s="7" t="inlineStr">
         <is>
-          <t>WiFi 端 32 bit 像素（X2R10G10B10）阶段 1 复验：黄金/PL 仿真一致，合主线</t>
+          <t>第二步（bootdelay 0 / 精简 uInitrd）写启动文件被权限系统拒绝，需用户明早本人批准后执行</t>
         </is>
       </c>
       <c r="E149" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 1995be8</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12132,24 +12132,24 @@
       <c r="A150" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B150" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B150" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C150" s="7" t="inlineStr">
         <is>
-          <t>D3;D4;D5</t>
+          <t>D15</t>
         </is>
       </c>
       <c r="D150" s="7" t="inlineStr">
         <is>
-          <t>下午用户：2260 相关先暂停、先做共用部分（token 不够）；15:00 又改为多开并行恢复 2260</t>
+          <t>WiFi 端 32 bit 像素（X2R10G10B10）阶段 1 复验：黄金/PL 仿真一致，合主线</t>
         </is>
       </c>
       <c r="E150" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 1995be8</t>
         </is>
       </c>
     </row>
@@ -12162,15 +12162,19 @@
           <t>决定</t>
         </is>
       </c>
-      <c r="C151" s="7" t="inlineStr"/>
+      <c r="C151" s="7" t="inlineStr">
+        <is>
+          <t>D3;D4;D5</t>
+        </is>
+      </c>
       <c r="D151" s="7" t="inlineStr">
         <is>
-          <t>软件三期：0 期 2047 屏（现在）/ 1 期 2260 验证板 160×180（预计 11-10 回板）/ 2 期 192×216 目标板；1 期目标 24 Hz / 358 片 / 6 链</t>
+          <t>下午用户：2260 相关先暂停、先做共用部分（token 不够）；15:00 又改为多开并行恢复 2260</t>
         </is>
       </c>
       <c r="E151" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_sw_three_phases_1013.md</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12178,15 +12182,15 @@
       <c r="A152" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B152" s="19" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+      <c r="B152" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C152" s="7" t="inlineStr"/>
       <c r="D152" s="7" t="inlineStr">
         <is>
-          <t>硬件 1 期验证板预计 2026-11-10 回板（初步交期，可能变），回板前软件能做的都前置</t>
+          <t>软件三期：0 期 2047 屏（现在）/ 1 期 2260 验证板 160×180（预计 11-10 回板）/ 2 期 192×216 目标板；1 期目标 24 Hz / 358 片 / 6 链</t>
         </is>
       </c>
       <c r="E152" s="7" t="inlineStr">
@@ -12199,20 +12203,20 @@
       <c r="A153" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B153" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B153" s="19" t="inlineStr">
+        <is>
+          <t>里程碑</t>
         </is>
       </c>
       <c r="C153" s="7" t="inlineStr"/>
       <c r="D153" s="7" t="inlineStr">
         <is>
-          <t>架构切分：PL 切片器及之前为各期共用的公共部分，屏幕显示为可替换后端，两者之间用实时按角度片流接口</t>
+          <t>硬件 1 期验证板预计 2026-11-10 回板（初步交期，可能变），回板前软件能做的都前置</t>
         </is>
       </c>
       <c r="E153" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_arch_common_front_display_backend.md</t>
+          <t>claude_memory/project_sw_three_phases_1013.md</t>
         </is>
       </c>
     </row>
@@ -12225,19 +12229,15 @@
           <t>决定</t>
         </is>
       </c>
-      <c r="C154" s="7" t="inlineStr">
-        <is>
-          <t>D3</t>
-        </is>
-      </c>
+      <c r="C154" s="7" t="inlineStr"/>
       <c r="D154" s="7" t="inlineStr">
         <is>
-          <t>用户定：2 期上行 1.2G；1 期保持 24 Hz（358 片，桥链路余量 0.40%）不降档</t>
+          <t>架构切分：PL 切片器及之前为各期共用的公共部分，屏幕显示为可替换后端，两者之间用实时按角度片流接口</t>
         </is>
       </c>
       <c r="E154" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>claude_memory/project_arch_common_front_display_backend.md</t>
         </is>
       </c>
     </row>
@@ -12252,12 +12252,12 @@
       </c>
       <c r="C155" s="7" t="inlineStr">
         <is>
-          <t>D11</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="D155" s="7" t="inlineStr">
         <is>
-          <t>傍晚用户：杜邦线跑不了 1.2G，1.2G 实测等 V1 回板；C1 台架只做 ≤300M 低速功能档</t>
+          <t>用户定：2 期上行 1.2G；1 期保持 24 Hz（358 片，桥链路余量 0.40%）不降档</t>
         </is>
       </c>
       <c r="E155" s="7" t="inlineStr">
@@ -12277,12 +12277,12 @@
       </c>
       <c r="C156" s="7" t="inlineStr">
         <is>
-          <t>D12;D13;D14</t>
+          <t>D11</t>
         </is>
       </c>
       <c r="D156" s="7" t="inlineStr">
         <is>
-          <t>19:00 用户：V0 可见的先插队、V1 接着做，新派 D12 延迟降低 / D13 启动提速 / D14 内容与手机控制</t>
+          <t>傍晚用户：杜邦线跑不了 1.2G，1.2G 实测等 V1 回板；C1 台架只做 ≤300M 低速功能档</t>
         </is>
       </c>
       <c r="E156" s="7" t="inlineStr">
@@ -12302,12 +12302,12 @@
       </c>
       <c r="C157" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D12;D13;D14</t>
         </is>
       </c>
       <c r="D157" s="7" t="inlineStr">
         <is>
-          <t>21:10 用户定 D13 目标：复位到 0° 片亮起 ≤12 s，找板 ≤20 s（看板 KR8.1 已改）</t>
+          <t>19:00 用户：V0 可见的先插队、V1 接着做，新派 D12 延迟降低 / D13 启动提速 / D14 内容与手机控制</t>
         </is>
       </c>
       <c r="E157" s="7" t="inlineStr">
@@ -12327,12 +12327,12 @@
       </c>
       <c r="C158" s="7" t="inlineStr">
         <is>
-          <t>D15;D16</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D158" s="7" t="inlineStr">
         <is>
-          <t>用户选 12-bit 方案 A：WiFi 端传高位宽、像素位宽 16/32 bit 可配（D15）；DDR 做到极限 A 线（D16），B 线并入 T2 硬件</t>
+          <t>21:10 用户定 D13 目标：复位到 0° 片亮起 ≤12 s，找板 ≤20 s（看板 KR8.1 已改）</t>
         </is>
       </c>
       <c r="E158" s="7" t="inlineStr">
@@ -12352,17 +12352,17 @@
       </c>
       <c r="C159" s="7" t="inlineStr">
         <is>
-          <t>KR5.2</t>
+          <t>D15;D16</t>
         </is>
       </c>
       <c r="D159" s="7" t="inlineStr">
         <is>
-          <t>用户实转核实：2047 旧表镜像，已更正为新表 0decad54</t>
+          <t>用户选 12-bit 方案 A：WiFi 端传高位宽、像素位宽 16/32 bit 可配（D15）；DDR 做到极限 A 线（D16），B 线并入 T2 硬件</t>
         </is>
       </c>
       <c r="E159" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 49031f6</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12370,24 +12370,24 @@
       <c r="A160" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B160" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B160" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C160" s="7" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>KR5.2</t>
         </is>
       </c>
       <c r="D160" s="7" t="inlineStr">
         <is>
-          <t>D7 上板补测会装/还原 autorun，冲掉 D13 补丁，须排在 D13 定稿合并之后；夜间板子排程 D12→D13→D2→D7→8 h 长跑</t>
+          <t>用户实转核实：2047 旧表镜像，已更正为新表 0decad54</t>
         </is>
       </c>
       <c r="E160" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 49031f6</t>
         </is>
       </c>
     </row>
@@ -12395,18 +12395,43 @@
       <c r="A161" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B161" s="19" t="inlineStr">
+      <c r="B161" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
+        </is>
+      </c>
+      <c r="C161" s="7" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="D161" s="7" t="inlineStr">
+        <is>
+          <t>D7 上板补测会装/还原 autorun，冲掉 D13 补丁，须排在 D13 定稿合并之后；夜间板子排程 D12→D13→D2→D7→8 h 长跑</t>
+        </is>
+      </c>
+      <c r="E161" s="7" t="inlineStr">
+        <is>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B162" s="19" t="inlineStr">
         <is>
           <t>里程碑</t>
         </is>
       </c>
-      <c r="C161" s="7" t="inlineStr"/>
-      <c r="D161" s="7" t="inlineStr">
+      <c r="C162" s="7" t="inlineStr"/>
+      <c r="D162" s="7" t="inlineStr">
         <is>
           <t>显性目的进度看板第一版建立：10 个显性目的 + KR 趋势 + 燃起图 + 里程碑趋势</t>
         </is>
       </c>
-      <c r="E161" s="7" t="inlineStr">
+      <c r="E162" s="7" t="inlineStr">
         <is>
           <t>claude_memory/project_progress_dashboard.md</t>
         </is>
@@ -17225,7 +17250,7 @@
         <v>20</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9">
@@ -18077,10 +18102,12 @@
       <c r="E43" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="F43" s="17" t="n"/>
-      <c r="G43" s="15" t="inlineStr">
-        <is>
-          <t>🔄</t>
+      <c r="F43" s="17" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G43" s="11" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="H43" s="7" t="inlineStr">

</xml_diff>

<commit_message>
[看板] 03 起来+验收 6/6; D26 完成; 周末 D27/D28/D29 + 24h 长跑
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/progress/显性目的进度_2026-10-16.xlsx
+++ b/docs/progress/显性目的进度_2026-10-16.xlsx
@@ -8522,7 +8522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J163"/>
+  <dimension ref="A1:J166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -8593,16 +8593,16 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>0.9767441860465116</v>
+        <v>0.9545454545454546</v>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>42/43</t>
+          <t>42/44</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>KR 24/25 + 交付 18/18 — 统一口径：达成率_P = (P 目标已达标的 KR 数 + P 需要的交付里已完成数) ÷ (有 P 目标的 KR 数 + P 需要的交付总数)，P = V0 / V1 / V2。</t>
+          <t>KR 24/25 + 交付 18/19 — 统一口径：达成率_P = (P 目标已达标的 KR 数 + P 需要的交付里已完成数) ÷ (有 P 目标的 KR 数 + P 需要的交付总数)，P = V0 / V1 / V2。</t>
         </is>
       </c>
       <c r="G4" s="8" t="n">
@@ -8625,16 +8625,16 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.7894736842105263</v>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>45/54</t>
+          <t>45/57</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>KR 16/24 + 交付 29/30 — 只按「必须」项计：KR 全算必须；交付看 deliverables.csv 的「级别」列 (必须/加分)，加分项不进分子分母。</t>
+          <t>KR 16/24 + 交付 29/33 — 只按「必须」项计：KR 全算必须；交付看 deliverables.csv 的「级别」列 (必须/加分)，加分项不进分子分母。</t>
         </is>
       </c>
       <c r="G5" s="8" t="n">
@@ -8657,16 +8657,16 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.7413793103448276</v>
+        <v>0.7096774193548387</v>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>43/58</t>
+          <t>44/62</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>KR 14/24 + 交付 29/34 — 交付的"需要"是嵌套的：V0 需要 = 阶段 V0；V1 需要 = V0 + V1准备；V2 需要 = V1 需要 + V2 (阶段列见 deliverables.csv，没填阶段的交付不计)。</t>
+          <t>KR 14/24 + 交付 30/38 — 交付的"需要"是嵌套的：V0 需要 = 阶段 V0；V1 需要 = V0 + V1准备；V2 需要 = V1 需要 + V2 (阶段列见 deliverables.csv，没填阶段的交付不计)。</t>
         </is>
       </c>
       <c r="G6" s="8" t="n">
@@ -8706,13 +8706,13 @@
         <v>46311</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>0.9767</v>
+        <v>0.9545</v>
       </c>
       <c r="I8" s="9" t="n">
-        <v>0.8333</v>
+        <v>0.7895</v>
       </c>
       <c r="J8" s="9" t="n">
-        <v>0.7413999999999999</v>
+        <v>0.7097</v>
       </c>
     </row>
     <row r="9">
@@ -10330,76 +10330,76 @@
     </row>
     <row r="78">
       <c r="A78" s="17" t="n">
-        <v>46310</v>
-      </c>
-      <c r="B78" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46311</v>
+      </c>
+      <c r="B78" s="6" t="inlineStr">
+        <is>
+          <t>硬件</t>
         </is>
       </c>
       <c r="C78" s="7" t="inlineStr">
         <is>
-          <t>KR7.2</t>
+          <t>DR1M90-03</t>
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr">
         <is>
-          <t>8 h 无人值守长跑 9/9 通过 (重开轮 23:45-07:45; 判读 S1 行数口径误判已改为覆盖时长 fe53bde); V0 出口 ⑥ 达成 → V0 出口 8/8</t>
+          <t>03 起来了: 控制台 COM30 (CH342-A); 冷上电 u-boot 报 Card did not respond to voltage select -110 停在 =&gt;, mmc rescan + boot 后正常; 登记 dr1m90-03 (10.10.21.10), V0 验收 6/6 PASS (WiFi -45 dBm, 推流 1351 帧/90 s) → D29 查根因</t>
         </is>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
-          <t>progress/soak_v0/report.md</t>
+          <t>D:\card03\boot03.log</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="17" t="n">
-        <v>46310</v>
-      </c>
-      <c r="B79" s="6" t="inlineStr">
-        <is>
-          <t>测量</t>
+        <v>46311</v>
+      </c>
+      <c r="B79" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C79" s="7" t="inlineStr">
         <is>
-          <t>QoS</t>
+          <t>D26</t>
         </is>
       </c>
       <c r="D79" s="7" t="inlineStr">
         <is>
-          <t>QoS (XMON DDR_S2 QOS_CONFIG=0x0F) 带载对照 (纯切片 30 Hz): 体素流+TCP 迟到 4.12% → 0.000%, CPU memcpy 300 MB/s 91.5% → 0.000%; 2047 32 bit@16.15 rps 完成率无改善 (86/71% vs 无 QoS 91/82%, 带宽上限); 测后寄存器已写回 0</t>
+          <t>V2 位流按主线重出合主线 c8e8294: 0 违例但余量 0.000 ns (旧 +0.001), 资源略降; D26 agent 遗留的卡死构建进程 (嵌套 flock) 占锁 2.5 h, 已按 PID 清掉</t>
         </is>
       </c>
       <c r="E79" s="7" t="inlineStr">
         <is>
-          <t>~/qos_runs</t>
+          <t>dr1v90 td_pov/pure_ul/results/p2_ul1200_b12_v3</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="17" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>测量</t>
+          <t>开工</t>
         </is>
       </c>
       <c r="C80" s="7" t="inlineStr">
         <is>
-          <t>D16b</t>
+          <t>周末</t>
         </is>
       </c>
       <c r="D80" s="7" t="inlineStr">
         <is>
-          <t>4x4 分块上板 A/B: 体素流+TCP 迟到 现布局 5.34%/4.45% (漂移 0.89 pp) vs 分块 4.79%, 收益在漂移内 = 无效; 迟到角度随相位漂移, 非几何换行主导。按约定不合主线, 分支 task/d16b-tile 保留</t>
+          <t>用户: SoC↔桥通信全功能开工, 软件能做的都做, 周一看结果。开 D27 (SoC↔桥全功能, Opus) / D28 (V1 回板一键脚本) / D29 (冷启动认卡); 02 跑 24 h 产品配置长跑 (PLV=0 max-fps 20 margin 1.0, 主线 8eced5a)</t>
         </is>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d16b-tile 7936b7e</t>
+          <t>dr1v90 soak8h/runs/1016_wkend_24h</t>
         </is>
       </c>
     </row>
@@ -10407,24 +10407,24 @@
       <c r="A81" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B81" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B81" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C81" s="7" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>KR7.2</t>
         </is>
       </c>
       <c r="D81" s="7" t="inlineStr">
         <is>
-          <t>用户定 V0/V1/V2 兼容 300-1200 rpm; 实转 583 rpm PL 只 8 fps (等整圈换帧) → D19 半圈换帧开做 (RTL+voxslice+假转扫速验收)</t>
+          <t>8 h 无人值守长跑 9/9 通过 (重开轮 23:45-07:45; 判读 S1 行数口径误判已改为覆盖时长 fe53bde); V0 出口 ⑥ 达成 → V0 出口 8/8</t>
         </is>
       </c>
       <c r="E81" s="7" t="inlineStr">
         <is>
-          <t>用户 10-15</t>
+          <t>progress/soak_v0/report.md</t>
         </is>
       </c>
     </row>
@@ -10432,24 +10432,24 @@
       <c r="A82" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B82" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B82" s="6" t="inlineStr">
+        <is>
+          <t>测量</t>
         </is>
       </c>
       <c r="C82" s="7" t="inlineStr">
         <is>
-          <t>D20</t>
+          <t>QoS</t>
         </is>
       </c>
       <c r="D82" s="7" t="inlineStr">
         <is>
-          <t>用户定流畅显示为一等要求 (V0/V1/V2); D20 阶段 1 流畅度指标+门槛+基线开做 (与 D19 并行)</t>
+          <t>QoS (XMON DDR_S2 QOS_CONFIG=0x0F) 带载对照 (纯切片 30 Hz): 体素流+TCP 迟到 4.12% → 0.000%, CPU memcpy 300 MB/s 91.5% → 0.000%; 2047 32 bit@16.15 rps 完成率无改善 (86/71% vs 无 QoS 91/82%, 带宽上限); 测后寄存器已写回 0</t>
         </is>
       </c>
       <c r="E82" s="7" t="inlineStr">
         <is>
-          <t>用户 10-15</t>
+          <t>~/qos_runs</t>
         </is>
       </c>
     </row>
@@ -10459,22 +10459,22 @@
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>分析</t>
+          <t>测量</t>
         </is>
       </c>
       <c r="C83" s="7" t="inlineStr">
         <is>
-          <t>V1/V2</t>
+          <t>D16b</t>
         </is>
       </c>
       <c r="D83" s="7" t="inlineStr">
         <is>
-          <t>转速 300-1200 rpm 纸面预算: 300 rpm 体刷新仅 10 Hz (物理闪烁); V1 358 片只到 ~718 rpm, 1200 需降到 215 片; V2 605 片到 ~1060 rpm; 公共切片核需支持运行时换每圈片数 (见 budget/rpm_range_2026-10-15.md)</t>
+          <t>4x4 分块上板 A/B: 体素流+TCP 迟到 现布局 5.34%/4.45% (漂移 0.89 pp) vs 分块 4.79%, 收益在漂移内 = 无效; 迟到角度随相位漂移, 非几何换行主导。按约定不合主线, 分支 task/d16b-tile 保留</t>
         </is>
       </c>
       <c r="E83" s="7" t="inlineStr">
         <is>
-          <t>budget/rpm_range_2026-10-15.md</t>
+          <t>dr1v90 task/d16b-tile 7936b7e</t>
         </is>
       </c>
     </row>
@@ -10482,24 +10482,24 @@
       <c r="A84" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B84" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B84" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C84" s="7" t="inlineStr">
         <is>
-          <t>KR7.3</t>
+          <t>D19</t>
         </is>
       </c>
       <c r="D84" s="7" t="inlineStr">
         <is>
-          <t>实转 1 h 无故障通过 (583 rpm, QoS 开机默认已上卡 7d301a6); V0 必须项全部达成</t>
+          <t>用户定 V0/V1/V2 兼容 300-1200 rpm; 实转 583 rpm PL 只 8 fps (等整圈换帧) → D19 半圈换帧开做 (RTL+voxslice+假转扫速验收)</t>
         </is>
       </c>
       <c r="E84" s="7" t="inlineStr">
         <is>
-          <t>progress/realspin_v0/</t>
+          <t>用户 10-15</t>
         </is>
       </c>
     </row>
@@ -10507,24 +10507,24 @@
       <c r="A85" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B85" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B85" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C85" s="7" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>D20</t>
         </is>
       </c>
       <c r="D85" s="7" t="inlineStr">
         <is>
-          <t>实转换帧仅 10.45/s (583 rpm 整圈换帧限制), 用户感觉卡; D19 半圈换帧 + D20 流畅度门槛处理</t>
+          <t>用户定流畅显示为一等要求 (V0/V1/V2); D20 阶段 1 流畅度指标+门槛+基线开做 (与 D19 并行)</t>
         </is>
       </c>
       <c r="E85" s="7" t="inlineStr">
         <is>
-          <t>progress/realspin_v0/</t>
+          <t>用户 10-15</t>
         </is>
       </c>
     </row>
@@ -10534,22 +10534,22 @@
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>交付</t>
+          <t>分析</t>
         </is>
       </c>
       <c r="C86" s="7" t="inlineStr">
         <is>
-          <t>D20</t>
+          <t>V1/V2</t>
         </is>
       </c>
       <c r="D86" s="7" t="inlineStr">
         <is>
-          <t>流畅度阶段 1: host/smooth_report.py + 门槛 (软件损失≤3%, 间隔 p99≤2T0, 长停顿≤5‰, 撕裂 0 等, SPEC §12) + voxslice --flip-log; 基线: 8 h 假转软件损失 2.3% 但约每 2 min 一次 2-3 s 无新帧 (主机/链路侧, 板端 PL 无缺口) 判 FAIL; 实转 648 rpm 软件损失 3.5%, 每分钟至少一顿 0.3-1.1 s 判 FAIL。主会话复验中</t>
+          <t>转速 300-1200 rpm 纸面预算: 300 rpm 体刷新仅 10 Hz (物理闪烁); V1 358 片只到 ~718 rpm, 1200 需降到 215 片; V2 605 片到 ~1060 rpm; 公共切片核需支持运行时换每圈片数 (见 budget/rpm_range_2026-10-15.md)</t>
         </is>
       </c>
       <c r="E86" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20-smooth 83a5fd7</t>
+          <t>budget/rpm_range_2026-10-15.md</t>
         </is>
       </c>
     </row>
@@ -10564,17 +10564,17 @@
       </c>
       <c r="C87" s="7" t="inlineStr">
         <is>
-          <t>D14</t>
+          <t>KR7.3</t>
         </is>
       </c>
       <c r="D87" s="7" t="inlineStr">
         <is>
-          <t>更多内容 + 手机网页控制合主线 (用户实转看过); 新克隆回归全过</t>
+          <t>实转 1 h 无故障通过 (583 rpm, QoS 开机默认已上卡 7d301a6); V0 必须项全部达成</t>
         </is>
       </c>
       <c r="E87" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 e215176</t>
+          <t>progress/realspin_v0/</t>
         </is>
       </c>
     </row>
@@ -10582,9 +10582,9 @@
       <c r="A88" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B88" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+      <c r="B88" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C88" s="7" t="inlineStr">
@@ -10594,12 +10594,12 @@
       </c>
       <c r="D88" s="7" t="inlineStr">
         <is>
-          <t>半圈换帧: 换网格上限 1×→2×转速 (583 rpm 9.7→~19/s), 慢转均匀丢帧; 16/32 档位流时序收住 (REV 0x20471019/1A); 转速窗口 300-1200; 离线 16/16 + 仿真 21+5 + pls2047 32/32。主会话复验+上板假转扫点中</t>
+          <t>实转换帧仅 10.45/s (583 rpm 整圈换帧限制), 用户感觉卡; D19 半圈换帧 + D20 流畅度门槛处理</t>
         </is>
       </c>
       <c r="E88" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d19-halfrev 1beafa6</t>
+          <t>progress/realspin_v0/</t>
         </is>
       </c>
     </row>
@@ -10614,17 +10614,17 @@
       </c>
       <c r="C89" s="7" t="inlineStr">
         <is>
-          <t>D20b</t>
+          <t>D20</t>
         </is>
       </c>
       <c r="D89" s="7" t="inlineStr">
         <is>
-          <t>画面模拟器 host/pov_view.py (按视觉暂留合成人眼所见, 并排对比): 整圈换帧 9.8/s 跳 51 帧; 半圈 15/s 但 51/103 ms 交替 (内容 15 fps 与半圈节拍不齐 → D20 阶段 3 内容帧率跟转速); 300 rpm 闪烁; 停推冻结后跳帧。示例 gif 在 dr1v90/_work/d20b/d20_smooth/sim_out/; 复验 PASS</t>
+          <t>流畅度阶段 1: host/smooth_report.py + 门槛 (软件损失≤3%, 间隔 p99≤2T0, 长停顿≤5‰, 撕裂 0 等, SPEC §12) + voxslice --flip-log; 基线: 8 h 假转软件损失 2.3% 但约每 2 min 一次 2-3 s 无新帧 (主机/链路侧, 板端 PL 无缺口) 判 FAIL; 实转 648 rpm 软件损失 3.5%, 每分钟至少一顿 0.3-1.1 s 判 FAIL。主会话复验中</t>
         </is>
       </c>
       <c r="E89" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20b-sim 9081f62</t>
+          <t>dr1v90 task/d20-smooth 83a5fd7</t>
         </is>
       </c>
     </row>
@@ -10632,24 +10632,24 @@
       <c r="A90" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B90" s="6" t="inlineStr">
-        <is>
-          <t>验证</t>
+      <c r="B90" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C90" s="7" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>D14</t>
         </is>
       </c>
       <c r="D90" s="7" t="inlineStr">
         <is>
-          <t>半圈换帧上板假转扫点 PASS: 5/7.5/10/15/20 rps 换网格 9.00/13.56/15.09/15.09/15.08 每秒 (老行为 10 rps 仅 9.00), 完成率 100%, 撕裂 0, 对拍全一致, 超时 0; 卡上开机默认已是 D19 位流 0x20471019。D19+D20+D20b 合并分支全回归中</t>
+          <t>更多内容 + 手机网页控制合主线 (用户实转看过); 新克隆回归全过</t>
         </is>
       </c>
       <c r="E90" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/merge-d19-d20 106364e</t>
+          <t>dr1v90 e215176</t>
         </is>
       </c>
     </row>
@@ -10657,24 +10657,24 @@
       <c r="A91" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B91" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B91" s="6" t="inlineStr">
+        <is>
+          <t>交付</t>
         </is>
       </c>
       <c r="C91" s="7" t="inlineStr">
         <is>
-          <t>D19/D20</t>
+          <t>D19</t>
         </is>
       </c>
       <c r="D91" s="7" t="inlineStr">
         <is>
-          <t>半圈换帧 + 流畅度检测 + 画面模拟器合主线; 全回归 10 套 (D18/D13/D19/D20/D20b/color/pls2047/rotor_ops/live_push/重连) 通过; 下一步 D20 阶段 3 (内容帧率跟转速、主机侧停顿诊断) + 实转复核</t>
+          <t>半圈换帧: 换网格上限 1×→2×转速 (583 rpm 9.7→~19/s), 慢转均匀丢帧; 16/32 档位流时序收住 (REV 0x20471019/1A); 转速窗口 300-1200; 离线 16/16 + 仿真 21+5 + pls2047 32/32。主会话复验+上板假转扫点中</t>
         </is>
       </c>
       <c r="E91" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>dr1v90 task/d19-halfrev 1beafa6</t>
         </is>
       </c>
     </row>
@@ -10689,17 +10689,17 @@
       </c>
       <c r="C92" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D20b</t>
         </is>
       </c>
       <c r="D92" s="7" t="inlineStr">
         <is>
-          <t>每圈片数随转速换档 (V1/V2 到 1200 rpm 的前提): N/PB/LUT 圈边界同步锁存, 回差 5%; V0 2047 人为 142/128 两档仿真逐字节一致、撕裂 0, 假转斜坡升降各 1 次不抖; 16/32 档位流时序收住 (REV 0x20471021/22)。风险: 软件写序时间窗 (可加影子寄存器)。主会话复验中, 诊断跑完后上板</t>
+          <t>画面模拟器 host/pov_view.py (按视觉暂留合成人眼所见, 并排对比): 整圈换帧 9.8/s 跳 51 帧; 半圈 15/s 但 51/103 ms 交替 (内容 15 fps 与半圈节拍不齐 → D20 阶段 3 内容帧率跟转速); 300 rpm 闪烁; 停推冻结后跳帧。示例 gif 在 dr1v90/_work/d20b/d20_smooth/sim_out/; 复验 PASS</t>
         </is>
       </c>
       <c r="E92" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d21-nband adeba44</t>
+          <t>dr1v90 task/d20b-sim 9081f62</t>
         </is>
       </c>
     </row>
@@ -10709,22 +10709,22 @@
       </c>
       <c r="B93" s="6" t="inlineStr">
         <is>
-          <t>根因</t>
+          <t>验证</t>
         </is>
       </c>
       <c r="C93" s="7" t="inlineStr">
         <is>
-          <t>D20/D22</t>
+          <t>D19</t>
         </is>
       </c>
       <c r="D93" s="7" t="inlineStr">
         <is>
-          <t>推流每 124.5 s 卡 3 s 的根因 = 长跑脚本的板上对拍 (--pl-verify 1800 ≈ 每 120 s, 每次停 ~3 s), 测试工具自身, 产品默认不开; WiFi 链路同刻 ping 0 丢。WSL/Windows 各 6 min 回放对照: 无周期卡顿, 但有偶发 1-1.7 s ACK 停顿 (每 6 min 1-2 次) = 真实 WiFi 抖动 → D22 WiFi 稳定 (用户 10-15: V0 必须搞定, 不能靠串口)</t>
+          <t>半圈换帧上板假转扫点 PASS: 5/7.5/10/15/20 rps 换网格 9.00/13.56/15.09/15.09/15.08 每秒 (老行为 10 rps 仅 9.00), 完成率 100%, 撕裂 0, 对拍全一致, 超时 0; 卡上开机默认已是 D19 位流 0x20471019。D19+D20+D20b 合并分支全回归中</t>
         </is>
       </c>
       <c r="E93" s="7" t="inlineStr">
         <is>
-          <t>~/realspin/tcp</t>
+          <t>dr1v90 task/merge-d19-d20 106364e</t>
         </is>
       </c>
     </row>
@@ -10732,24 +10732,24 @@
       <c r="A94" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B94" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B94" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C94" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D19/D20</t>
         </is>
       </c>
       <c r="D94" s="7" t="inlineStr">
         <is>
-          <t>用户: 不插串口也必须永远连得上, 彻底解决 (V0 必须) → D22 四层兜底开做: 服务监护 + 硬件看门狗 + 兜底热点 + 故障注入验收</t>
+          <t>半圈换帧 + 流畅度检测 + 画面模拟器合主线; 全回归 10 套 (D18/D13/D19/D20/D20b/color/pls2047/rotor_ops/live_push/重连) 通过; 下一步 D20 阶段 3 (内容帧率跟转速、主机侧停顿诊断) + 实转复核</t>
         </is>
       </c>
       <c r="E94" s="7" t="inlineStr">
         <is>
-          <t>用户 10-15</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10764,17 +10764,17 @@
       </c>
       <c r="C95" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D95" s="7" t="inlineStr">
         <is>
-          <t>不插串口永远连得上: povreach 服务监护 + 硬件看门狗 (60 s, 防风暴) + 兜底热点 POV-&lt;板名&gt; (hostapd 静编, 192.168.77.1, 状态页可填 WiFi) + 30 min 无网重启; 失效模式表 16 行; 离线 9/9。排队上板故障演练 (8 项, 含 2 次看门狗复位)</t>
+          <t>每圈片数随转速换档 (V1/V2 到 1200 rpm 的前提): N/PB/LUT 圈边界同步锁存, 回差 5%; V0 2047 人为 142/128 两档仿真逐字节一致、撕裂 0, 假转斜坡升降各 1 次不抖; 16/32 档位流时序收住 (REV 0x20471021/22)。风险: 软件写序时间窗 (可加影子寄存器)。主会话复验中, 诊断跑完后上板</t>
         </is>
       </c>
       <c r="E95" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach ee4a55c</t>
+          <t>dr1v90 task/d21-nband adeba44</t>
         </is>
       </c>
     </row>
@@ -10784,22 +10784,22 @@
       </c>
       <c r="B96" s="6" t="inlineStr">
         <is>
-          <t>交付</t>
+          <t>根因</t>
         </is>
       </c>
       <c r="C96" s="7" t="inlineStr">
         <is>
-          <t>D20c</t>
+          <t>D20/D22</t>
         </is>
       </c>
       <c r="D96" s="7" t="inlineStr">
         <is>
-          <t>内容帧率跟转速 voxlive --fps auto: 583 rpm 换帧间隔 std 23.4→0.1-0.9 ms (离线假转)。取舍: 板端默认 (max-fps 15, margin 0.9) 下 583 rpm 均匀但仅 9.7 fps; 板端 max-fps 20 + margin 1.0 → 19.4 fps 均匀。计划 D22 后上板验证 20/1.0 后改开机默认</t>
+          <t>推流每 124.5 s 卡 3 s 的根因 = 长跑脚本的板上对拍 (--pl-verify 1800 ≈ 每 120 s, 每次停 ~3 s), 测试工具自身, 产品默认不开; WiFi 链路同刻 ping 0 丢。WSL/Windows 各 6 min 回放对照: 无周期卡顿, 但有偶发 1-1.7 s ACK 停顿 (每 6 min 1-2 次) = 真实 WiFi 抖动 → D22 WiFi 稳定 (用户 10-15: V0 必须搞定, 不能靠串口)</t>
         </is>
       </c>
       <c r="E96" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20c-fps 338eaaf</t>
+          <t>~/realspin/tcp</t>
         </is>
       </c>
     </row>
@@ -10807,24 +10807,24 @@
       <c r="A97" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B97" s="6" t="inlineStr">
-        <is>
-          <t>复验</t>
+      <c r="B97" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C97" s="7" t="inlineStr">
         <is>
-          <t>D20c</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D97" s="7" t="inlineStr">
         <is>
-          <t>复验 F3 端到端节拍均匀度在主机忙 (D8 大仿真并行) 时不达标: 583 auto std 9.0/5.2 ms (门槛 3/4), 帧率正确; 主机计时抖动敏感, 先不合主线, 待空闲复验 + 上板实测定</t>
+          <t>用户: 不插串口也必须永远连得上, 彻底解决 (V0 必须) → D22 四层兜底开做: 服务监护 + 硬件看门狗 + 兜底热点 + 故障注入验收</t>
         </is>
       </c>
       <c r="E97" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d20c.v.log</t>
+          <t>用户 10-15</t>
         </is>
       </c>
     </row>
@@ -10839,17 +10839,17 @@
       </c>
       <c r="C98" s="7" t="inlineStr">
         <is>
-          <t>D8</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D98" s="7" t="inlineStr">
         <is>
-          <t>V1 主控↔桥↔2260 联合仿真 0 错 (12/8 bit, 6 链×16 片, 训练锁定, 半圈换帧); 抓出并修 2 个回板必错 bug: 12-bit 字槽格式主控两 beat vs 桥紧排不一致 (改主控 PK12, 上行 195→110 µs/片) + 1 期切片器 NXG 未传 (160 宽按 192 算); 待: 1 期 12-bit 位流重综合 (hclk 余量原 +0.001 ns)</t>
+          <t>不插串口永远连得上: povreach 服务监护 + 硬件看门狗 (60 s, 防风暴) + 兜底热点 POV-&lt;板名&gt; (hostapd 静编, 192.168.77.1, 状态页可填 WiFi) + 30 min 无网重启; 失效模式表 16 行; 离线 9/9。排队上板故障演练 (8 项, 含 2 次看门狗复位)</t>
         </is>
       </c>
       <c r="E98" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d8-cosim 85dfe51</t>
+          <t>dr1v90 task/d22-reach ee4a55c</t>
         </is>
       </c>
     </row>
@@ -10857,24 +10857,24 @@
       <c r="A99" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B99" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B99" s="6" t="inlineStr">
+        <is>
+          <t>交付</t>
         </is>
       </c>
       <c r="C99" s="7" t="inlineStr">
         <is>
-          <t>D8</t>
+          <t>D20c</t>
         </is>
       </c>
       <c r="D99" s="7" t="inlineStr">
         <is>
-          <t>V1 联合仿真合主线 (新克隆复验 5/5; 合并回归 sim_v1/pls2047/D18/D19 通过, D19 O4 一次主机忙计时抖动重跑过); V1 回板就绪清单 ⑤ 达成</t>
+          <t>内容帧率跟转速 voxlive --fps auto: 583 rpm 换帧间隔 std 23.4→0.1-0.9 ms (离线假转)。取舍: 板端默认 (max-fps 15, margin 0.9) 下 583 rpm 均匀但仅 9.7 fps; 板端 max-fps 20 + margin 1.0 → 19.4 fps 均匀。计划 D22 后上板验证 20/1.0 后改开机默认</t>
         </is>
       </c>
       <c r="E99" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>dr1v90 task/d20c-fps 338eaaf</t>
         </is>
       </c>
     </row>
@@ -10884,22 +10884,22 @@
       </c>
       <c r="B100" s="6" t="inlineStr">
         <is>
-          <t>测量</t>
+          <t>复验</t>
         </is>
       </c>
       <c r="C100" s="7" t="inlineStr">
         <is>
-          <t>D22/D20</t>
+          <t>D20c</t>
         </is>
       </c>
       <c r="D100" s="7" t="inlineStr">
         <is>
-          <t>1 h 产品配置 (无对拍) 推流诊断: 换帧 14.64/s 软件损失 2.4% ✅, 间隔 p99 124 ms ✅, 长停顿 3.7‰ ✅, 最长 495 ms ❌ (门槛 267); PC→板 ping 16781/0 丢; &gt;0.5 s ACK 停顿 46 min 内 4 次 (最长 0.78 s), 同刻 PC→网关 RTT 165-275 ms = PC 侧 WiFi 抖动。周期 3 s 卡顿消失 (确认系对拍)。余项: 0.5-0.8 s 偶发抖动 (播放缓冲 vs 延迟取舍 / PC 有线或专用路由)</t>
+          <t>复验 F3 端到端节拍均匀度在主机忙 (D8 大仿真并行) 时不达标: 583 auto std 9.0/5.2 ms (门槛 3/4), 帧率正确; 主机计时抖动敏感, 先不合主线, 待空闲复验 + 上板实测定</t>
         </is>
       </c>
       <c r="E100" s="7" t="inlineStr">
         <is>
-          <t>soak_runs/netdiag_1015_1814</t>
+          <t>~/rv_d20c.v.log</t>
         </is>
       </c>
     </row>
@@ -10907,24 +10907,24 @@
       <c r="A101" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B101" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B101" s="6" t="inlineStr">
+        <is>
+          <t>交付</t>
         </is>
       </c>
       <c r="C101" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D8</t>
         </is>
       </c>
       <c r="D101" s="7" t="inlineStr">
         <is>
-          <t>换档位流 (REV 0x20471021) 上板起步即停摆 (档 0 未换档时写完 47 片后停, 换网格全超时), 仿真全过 → 硅上与仿真不同; D21b 开查根因。另: D21 上板收尾用 m90/up.sh 会让板子没 PL, 已重启回开机默认 (0x20471019 + QoS)</t>
+          <t>V1 主控↔桥↔2260 联合仿真 0 错 (12/8 bit, 6 链×16 片, 训练锁定, 半圈换帧); 抓出并修 2 个回板必错 bug: 12-bit 字槽格式主控两 beat vs 桥紧排不一致 (改主控 PK12, 上行 195→110 µs/片) + 1 期切片器 NXG 未传 (160 宽按 192 算); 待: 1 期 12-bit 位流重综合 (hclk 余量原 +0.001 ns)</t>
         </is>
       </c>
       <c r="E101" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d21.board.log</t>
+          <t>dr1v90 task/d8-cosim 85dfe51</t>
         </is>
       </c>
     </row>
@@ -10932,24 +10932,24 @@
       <c r="A102" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B102" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B102" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C102" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D8</t>
         </is>
       </c>
       <c r="D102" s="7" t="inlineStr">
         <is>
-          <t>新克隆离线 O6 误 FAIL: hostapd/povreach 二进制 git 模式 644, WSL 本地盘克隆不可执行, qemu 静默拒绝 (板上 autorun 有 chmod, 不受影响); 已修 (git +x, verify chmod), 重跑后自动上板演练</t>
+          <t>V1 联合仿真合主线 (新克隆复验 5/5; 合并回归 sim_v1/pls2047/D18/D19 通过, D19 O4 一次主机忙计时抖动重跑过); V1 回板就绪清单 ⑤ 达成</t>
         </is>
       </c>
       <c r="E102" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10957,24 +10957,24 @@
       <c r="A103" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B103" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B103" s="6" t="inlineStr">
+        <is>
+          <t>测量</t>
         </is>
       </c>
       <c r="C103" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D22/D20</t>
         </is>
       </c>
       <c r="D103" s="7" t="inlineStr">
         <is>
-          <t>首轮上板演练 9 项误 FAIL = 验收脚本 info() 把板上 board_d22.sh info 的非 0 退出码当失败 (内容正常), settle/wait_healthy 恒失败; 板子本身正常 (装好开机 healthy, povreach managed, 看门狗 armed)。已修, 单独重跑全套演练 (~80 min); 期间 D21 取证因同时上板被干扰, 待 D22 后单独跑</t>
+          <t>1 h 产品配置 (无对拍) 推流诊断: 换帧 14.64/s 软件损失 2.4% ✅, 间隔 p99 124 ms ✅, 长停顿 3.7‰ ✅, 最长 495 ms ❌ (门槛 267); PC→板 ping 16781/0 丢; &gt;0.5 s ACK 停顿 46 min 内 4 次 (最长 0.78 s), 同刻 PC→网关 RTT 165-275 ms = PC 侧 WiFi 抖动。周期 3 s 卡顿消失 (确认系对拍)。余项: 0.5-0.8 s 偶发抖动 (播放缓冲 vs 延迟取舍 / PC 有线或专用路由)</t>
         </is>
       </c>
       <c r="E103" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach</t>
+          <t>soak_runs/netdiag_1015_1814</t>
         </is>
       </c>
     </row>
@@ -10982,24 +10982,24 @@
       <c r="A104" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B104" s="6" t="inlineStr">
-        <is>
-          <t>验证</t>
+      <c r="B104" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C104" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D104" s="7" t="inlineStr">
         <is>
-          <t>第二轮上板演练 (单独): 杀 sshd/mdns/povnetd 27-72 s 自愈找回 ✅; 错 SSID → 兜底热点 → 自己回公司网 ✅ (但 23.5 min, 目标 ≤10); 杀 wpa/关网卡、装后重启: 板子恢复了但 mDNS 按名字 240 s 内找不回 ❌ (缓存 IP 可连); 看门狗复位发生但晚于测试判定、卡上未记非正常结束 ❌。交回 D22 agent 修 (mDNS 找回为主)</t>
+          <t>换档位流 (REV 0x20471021) 上板起步即停摆 (档 0 未换档时写完 47 片后停, 换网格全超时), 仿真全过 → 硅上与仿真不同; D21b 开查根因。另: D21 上板收尾用 m90/up.sh 会让板子没 PL, 已重启回开机默认 (0x20471019 + QoS)</t>
         </is>
       </c>
       <c r="E104" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d22.board2.log</t>
+          <t>~/rv_d21.board.log</t>
         </is>
       </c>
     </row>
@@ -11007,24 +11007,24 @@
       <c r="A105" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B105" s="6" t="inlineStr">
-        <is>
-          <t>根因</t>
+      <c r="B105" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C105" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D105" s="7" t="inlineStr">
         <is>
-          <t>板上取证: 显示每圈取满 142 片, 但 s3rt_sys 旁听只认片号 0..47 → PL 每圈 48 触发后停摆; 不带档位 / 补 sub10 都一样 → RTL 旁听上限 (D21 改为按 FBO) 问题。交回 D21b 修 RTL; 板子已重启回默认 0x20471019</t>
+          <t>新克隆离线 O6 误 FAIL: hostapd/povreach 二进制 git 模式 644, WSL 本地盘克隆不可执行, qemu 静默拒绝 (板上 autorun 有 chmod, 不受影响); 已修 (git +x, verify chmod), 重跑后自动上板演练</t>
         </is>
       </c>
       <c r="E105" s="7" t="inlineStr">
         <is>
-          <t>~/d21b_forensic.log</t>
+          <t>dr1v90 task/d22-reach</t>
         </is>
       </c>
     </row>
@@ -11032,9 +11032,9 @@
       <c r="A106" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B106" s="6" t="inlineStr">
-        <is>
-          <t>根因</t>
+      <c r="B106" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C106" s="7" t="inlineStr">
@@ -11044,12 +11044,12 @@
       </c>
       <c r="D106" s="7" t="inlineStr">
         <is>
-          <t>按名字找不回的根因: povmdns 在地址回来/重关联时不重新发 IGMP 报告 (重复入组 EADDRINUSE 无报告), 企业 AP 只把组播转给报告过的站点 → mDNS 查询数分钟到不了板。修: 重关联/地址变化时退组再入组 + 宣告 (0/1/3/7/15/30 s) + 每 60 s 刷新; 看门狗读回实际超时并减半到 ≤60 s; 卡上记非正常结束。离线 10/10, 上板复验中</t>
+          <t>首轮上板演练 9 项误 FAIL = 验收脚本 info() 把板上 board_d22.sh info 的非 0 退出码当失败 (内容正常), settle/wait_healthy 恒失败; 板子本身正常 (装好开机 healthy, povreach managed, 看门狗 armed)。已修, 单独重跑全套演练 (~80 min); 期间 D21 取证因同时上板被干扰, 待 D22 后单独跑</t>
         </is>
       </c>
       <c r="E106" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach 0d1da09</t>
+          <t>dr1v90 task/d22-reach</t>
         </is>
       </c>
     </row>
@@ -11069,12 +11069,12 @@
       </c>
       <c r="D107" s="7" t="inlineStr">
         <is>
-          <t>第三轮上板演练 9/10: 装后重启 24 s 按名字找回 ✅ (上轮找不回); sshd/mdns/povnetd 杀掉 38-72 s ✅; 关网卡 191 s ✅; 错 SSID→热点→自动回 543 s ✅ (上轮 1411); 看门狗复位 reachkill 54 s / netdstop 213 s 且记非正常结束 ✅ (实际超时 32 s); 仅 kill wpa_supplicant 240 s 内未找回 ❌ (随后恢复), 单独重跑定位中</t>
+          <t>第二轮上板演练 (单独): 杀 sshd/mdns/povnetd 27-72 s 自愈找回 ✅; 错 SSID → 兜底热点 → 自己回公司网 ✅ (但 23.5 min, 目标 ≤10); 杀 wpa/关网卡、装后重启: 板子恢复了但 mDNS 按名字 240 s 内找不回 ❌ (缓存 IP 可连); 看门狗复位发生但晚于测试判定、卡上未记非正常结束 ❌。交回 D22 agent 修 (mDNS 找回为主)</t>
         </is>
       </c>
       <c r="E107" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d22b.board.log</t>
+          <t>~/rv_d22.board2.log</t>
         </is>
       </c>
     </row>
@@ -11084,22 +11084,22 @@
       </c>
       <c r="B108" s="6" t="inlineStr">
         <is>
-          <t>交付</t>
+          <t>根因</t>
         </is>
       </c>
       <c r="C108" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D108" s="7" t="inlineStr">
         <is>
-          <t>povnetd 1.2: wpa 进程没了/卡死/接口 down 立即重连 (原来一律等 60 s, 且 60 s 后的重连反把已自愈的连接打断 → 73-240+ s 且不稳); 只丢包仍按 60 s 防误重连; 关键事件写卡 (复位后可查); verify wpakill/ifdown 各连跑 3 次、120 s 内按名字找回。离线 11/11, 上板全套复验中</t>
+          <t>板上取证: 显示每圈取满 142 片, 但 s3rt_sys 旁听只认片号 0..47 → PL 每圈 48 触发后停摆; 不带档位 / 补 sub10 都一样 → RTL 旁听上限 (D21 改为按 FBO) 问题。交回 D21b 修 RTL; 板子已重启回默认 0x20471019</t>
         </is>
       </c>
       <c r="E108" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach e438a12</t>
+          <t>~/d21b_forensic.log</t>
         </is>
       </c>
     </row>
@@ -11114,92 +11114,92 @@
       </c>
       <c r="C109" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D109" s="7" t="inlineStr">
         <is>
-          <t>停摆根因不在 RTL: voxslice --pl 从不写显示 0x0C sub01 (bpp3), 重新加载位流后显示按 1-bit 片距 0x3000 取片, 旁听按 0x9000 片首只认 1/3 → 每圈 48 触发卡死。主线同有此隐患 (默认开机靠别的程序先写对)。修: pl_setup 先写 sub01; 仿真 +NOBPP3 复现与板上一致; 位流不变。离线 12/12, 排在 D22 后上板</t>
+          <t>按名字找不回的根因: povmdns 在地址回来/重关联时不重新发 IGMP 报告 (重复入组 EADDRINUSE 无报告), 企业 AP 只把组播转给报告过的站点 → mDNS 查询数分钟到不了板。修: 重关联/地址变化时退组再入组 + 宣告 (0/1/3/7/15/30 s) + 每 60 s 刷新; 看门狗读回实际超时并减半到 ≤60 s; 卡上记非正常结束。离线 10/10, 上板复验中</t>
         </is>
       </c>
       <c r="E109" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d21-nband 084bba3</t>
+          <t>dr1v90 task/d22-reach 0d1da09</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="17" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B110" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+        <v>46310</v>
+      </c>
+      <c r="B110" s="6" t="inlineStr">
+        <is>
+          <t>验证</t>
         </is>
       </c>
       <c r="C110" s="7" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D110" s="7" t="inlineStr">
         <is>
-          <t>上行出口全量复验 45/0, 合主线</t>
+          <t>第三轮上板演练 9/10: 装后重启 24 s 按名字找回 ✅ (上轮找不回); sshd/mdns/povnetd 杀掉 38-72 s ✅; 关网卡 191 s ✅; 错 SSID→热点→自动回 543 s ✅ (上轮 1411); 看门狗复位 reachkill 54 s / netdstop 213 s 且记非正常结束 ✅ (实际超时 32 s); 仅 kill wpa_supplicant 240 s 内未找回 ❌ (随后恢复), 单独重跑定位中</t>
         </is>
       </c>
       <c r="E110" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 fdb4de6</t>
+          <t>~/rv_d22b.board.log</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="17" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B111" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+        <v>46310</v>
+      </c>
+      <c r="B111" s="6" t="inlineStr">
+        <is>
+          <t>交付</t>
         </is>
       </c>
       <c r="C111" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D111" s="7" t="inlineStr">
         <is>
-          <t>PL 切片上板: 与 CPU 逐字节一致、30 min 无停摆, 但内容帧率 4.2&lt;15, 退回</t>
+          <t>povnetd 1.2: wpa 进程没了/卡死/接口 down 立即重连 (原来一律等 60 s, 且 60 s 后的重连反把已自愈的连接打断 → 73-240+ s 且不稳); 只丢包仍按 60 s 防误重连; 关键事件写卡 (复位后可查); verify wpakill/ifdown 各连跑 3 次、120 s 内按名字找回。离线 11/11, 上板全套复验中</t>
         </is>
       </c>
       <c r="E111" s="7" t="inlineStr">
         <is>
-          <t>scratchpad/v_pls4_board.log</t>
+          <t>dr1v90 task/d22-reach e438a12</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="17" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B112" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+        <v>46310</v>
+      </c>
+      <c r="B112" s="6" t="inlineStr">
+        <is>
+          <t>根因</t>
         </is>
       </c>
       <c r="C112" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D112" s="7" t="inlineStr">
         <is>
-          <t>30 Hz 带载迟到+掉片 3.7% (空载 0.2% 来自旧 netguard), 归因测试中</t>
+          <t>停摆根因不在 RTL: voxslice --pl 从不写显示 0x0C sub01 (bpp3), 重新加载位流后显示按 1-bit 片距 0x3000 取片, 旁听按 0x9000 片首只认 1/3 → 每圈 48 触发卡死。主线同有此隐患 (默认开机靠别的程序先写对)。修: pl_setup 先写 sub01; 仿真 +NOBPP3 复现与板上一致; 位流不变。离线 12/12, 排在 D22 后上板</t>
         </is>
       </c>
       <c r="E112" s="7" t="inlineStr">
         <is>
-          <t>project_ddr_budget_by_phase_1013</t>
+          <t>dr1v90 task/d21-nband 084bba3</t>
         </is>
       </c>
     </row>
@@ -11207,24 +11207,24 @@
       <c r="A113" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B113" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B113" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C113" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="D113" s="7" t="inlineStr">
         <is>
-          <t>纯切片带载约 21 min 停摆; 无负载浸泡 2×30 min 不停摆</t>
+          <t>上行出口全量复验 45/0, 合主线</t>
         </is>
       </c>
       <c r="E113" s="7" t="inlineStr">
         <is>
-          <t>project_ddr_budget_by_phase_1013</t>
+          <t>dr1v90 fdb4de6</t>
         </is>
       </c>
     </row>
@@ -11232,24 +11232,24 @@
       <c r="A114" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B114" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B114" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C114" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D114" s="7" t="inlineStr">
         <is>
-          <t>用户定目标: 复位到亮起 ≤12 s, 找板 ≤20 s</t>
+          <t>PL 切片上板: 与 CPU 逐字节一致、30 min 无停摆, 但内容帧率 4.2&lt;15, 退回</t>
         </is>
       </c>
       <c r="E114" s="7" t="inlineStr">
         <is>
-          <t>project_short_term_delivery_1013</t>
+          <t>scratchpad/v_pls4_board.log</t>
         </is>
       </c>
     </row>
@@ -11264,17 +11264,17 @@
       </c>
       <c r="C115" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D115" s="7" t="inlineStr">
         <is>
-          <t>找到 PL 切片器带载停摆根因: 零列描述符丢失 (公共核, 2260 也有) + pop 握手串片, 已修</t>
+          <t>30 Hz 带载迟到+掉片 3.7% (空载 0.2% 来自旧 netguard), 归因测试中</t>
         </is>
       </c>
       <c r="E115" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 debd3cd</t>
+          <t>project_ddr_budget_by_phase_1013</t>
         </is>
       </c>
     </row>
@@ -11282,24 +11282,24 @@
       <c r="A116" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B116" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B116" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C116" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D116" s="7" t="inlineStr">
         <is>
-          <t>上板 60 min 带载 0 停摆、逐字节一致、late 0; 帧率 13.8 差 0.5 退回</t>
+          <t>纯切片带载约 21 min 停摆; 无负载浸泡 2×30 min 不停摆</t>
         </is>
       </c>
       <c r="E116" s="7" t="inlineStr">
         <is>
-          <t>scratchpad v_pls6_board.log</t>
+          <t>project_ddr_budget_by_phase_1013</t>
         </is>
       </c>
     </row>
@@ -11307,24 +11307,24 @@
       <c r="A117" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B117" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B117" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C117" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D117" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 实时切片上板全过: 60 min 带载 0 停摆, 帧率 15.0, 与 CPU 逐字节一致</t>
+          <t>用户定目标: 复位到亮起 ≤12 s, 找板 ≤20 s</t>
         </is>
       </c>
       <c r="E117" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 782e9e3</t>
+          <t>project_short_term_delivery_1013</t>
         </is>
       </c>
     </row>
@@ -11339,17 +11339,17 @@
       </c>
       <c r="C118" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D118" s="7" t="inlineStr">
         <is>
-          <t>DDR 慢读根因: 每圈约 1/3 角度每取一列都换行, 两类 CPU 负载叠加越阈值 (0.002%→3%); 建议网格 4×4 分块</t>
+          <t>找到 PL 切片器带载停摆根因: 零列描述符丢失 (公共核, 2260 也有) + pop 握手串片, 已修</t>
         </is>
       </c>
       <c r="E118" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d16-ddr 539d303</t>
+          <t>dr1v90 task/pls-2047 debd3cd</t>
         </is>
       </c>
     </row>
@@ -11357,24 +11357,24 @@
       <c r="A119" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B119" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B119" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C119" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D119" s="7" t="inlineStr">
         <is>
-          <t>用户定: 子 agent 并行 ≤5 (周额度); 跑完的 agent 关掉</t>
+          <t>上板 60 min 带载 0 停摆、逐字节一致、late 0; 帧率 13.8 差 0.5 退回</t>
         </is>
       </c>
       <c r="E119" s="7" t="inlineStr">
         <is>
-          <t>feedback_save_weekly_quota</t>
+          <t>scratchpad v_pls6_board.log</t>
         </is>
       </c>
     </row>
@@ -11382,19 +11382,19 @@
       <c r="A120" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B120" s="19" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+      <c r="B120" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C120" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D120" s="7" t="inlineStr">
         <is>
-          <t>V0 出口清单: PL 切片上板通过 (D2) 可打勾</t>
+          <t>2047 PL 实时切片上板全过: 60 min 带载 0 停摆, 帧率 15.0, 与 CPU 逐字节一致</t>
         </is>
       </c>
       <c r="E120" s="7" t="inlineStr">
@@ -11407,24 +11407,24 @@
       <c r="A121" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B121" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B121" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C121" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D121" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 实时切片合进主线 (含公共核两处 bug 修复); D3 上行档位流需按新核重综合</t>
+          <t>DDR 慢读根因: 每圈约 1/3 角度每取一列都换行, 两类 CPU 负载叠加越阈值 (0.002%→3%); 建议网格 4×4 分块</t>
         </is>
       </c>
       <c r="E121" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 2364e5c</t>
+          <t>dr1v90 task/d16-ddr 539d303</t>
         </is>
       </c>
     </row>
@@ -11432,24 +11432,24 @@
       <c r="A122" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B122" s="19" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+      <c r="B122" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C122" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D122" s="7" t="inlineStr">
         <is>
-          <t>PL 硬件切片首次实转上屏 (650 rpm, 完成率 100%, CPU 82% 空闲), 用户确认与 CPU 切片无区别</t>
+          <t>用户定: 子 agent 并行 ≤5 (周额度); 跑完的 agent 关掉</t>
         </is>
       </c>
       <c r="E122" s="7" t="inlineStr">
         <is>
-          <t>用户在场实转</t>
+          <t>feedback_save_weekly_quota</t>
         </is>
       </c>
     </row>
@@ -11457,24 +11457,24 @@
       <c r="A123" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B123" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B123" s="19" t="inlineStr">
+        <is>
+          <t>里程碑</t>
         </is>
       </c>
       <c r="C123" s="7" t="inlineStr">
         <is>
-          <t>D18</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D123" s="7" t="inlineStr">
         <is>
-          <t>用户定: 只保留 PL 切片, 固化开机流程, CPU 切片只留应急退路</t>
+          <t>V0 出口清单: PL 切片上板通过 (D2) 可打勾</t>
         </is>
       </c>
       <c r="E123" s="7" t="inlineStr">
         <is>
-          <t>用户 10-14</t>
+          <t>dr1v90 task/pls-2047 782e9e3</t>
         </is>
       </c>
     </row>
@@ -11489,17 +11489,17 @@
       </c>
       <c r="C124" s="7" t="inlineStr">
         <is>
-          <t>D18</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D124" s="7" t="inlineStr">
         <is>
-          <t>开机默认 PL 切片合主线: 上电基础显示 → 推流显示推流 → 停推 5 min 回基础演示; CPU 只留应急退路</t>
+          <t>2047 PL 实时切片合进主线 (含公共核两处 bug 修复); D3 上行档位流需按新核重综合</t>
         </is>
       </c>
       <c r="E124" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d18-pl-default d35c6d4</t>
+          <t>dr1v90 2364e5c</t>
         </is>
       </c>
     </row>
@@ -11507,24 +11507,24 @@
       <c r="A125" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B125" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B125" s="19" t="inlineStr">
+        <is>
+          <t>里程碑</t>
         </is>
       </c>
       <c r="C125" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D125" s="7" t="inlineStr">
         <is>
-          <t>用户定目标放宽: 亮起 ≤12.5 s / 找板 ≤21 s; V0 出口 ④ 达成</t>
+          <t>PL 硬件切片首次实转上屏 (650 rpm, 完成率 100%, CPU 82% 空闲), 用户确认与 CPU 切片无区别</t>
         </is>
       </c>
       <c r="E125" s="7" t="inlineStr">
         <is>
-          <t>用户 10-14</t>
+          <t>用户在场实转</t>
         </is>
       </c>
     </row>
@@ -11532,24 +11532,24 @@
       <c r="A126" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B126" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B126" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C126" s="7" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>D18</t>
         </is>
       </c>
       <c r="D126" s="7" t="inlineStr">
         <is>
-          <t>无串口远程运维合主线: 升级坏包 (含断网包) 自动回滚后板子能按名字找回; 网络守护不再造成切片迟到 (旧版每分钟 2061 次 → 0); V0 出口 ⑤ 达成</t>
+          <t>用户定: 只保留 PL 切片, 固化开机流程, CPU 切片只留应急退路</t>
         </is>
       </c>
       <c r="E126" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 dee9be6</t>
+          <t>用户 10-14</t>
         </is>
       </c>
     </row>
@@ -11557,24 +11557,24 @@
       <c r="A127" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B127" s="6" t="inlineStr">
-        <is>
-          <t>根因</t>
+      <c r="B127" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C127" s="7" t="inlineStr">
         <is>
-          <t>D15b</t>
+          <t>D18</t>
         </is>
       </c>
       <c r="D127" s="7" t="inlineStr">
         <is>
-          <t>32 bit PL 全黑: 板端写 LUT 基址仍用 16 bit 布局偏移, PL 把网格当角度表读; 已修 308d1bb, 待上板</t>
+          <t>开机默认 PL 切片合主线: 上电基础显示 → 推流显示推流 → 停推 5 min 回基础演示; CPU 只留应急退路</t>
         </is>
       </c>
       <c r="E127" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d15b-color-p2</t>
+          <t>dr1v90 task/d18-pl-default d35c6d4</t>
         </is>
       </c>
     </row>
@@ -11582,24 +11582,24 @@
       <c r="A128" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B128" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B128" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C128" s="7" t="inlineStr">
         <is>
-          <t>D15</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D128" s="7" t="inlineStr">
         <is>
-          <t>WiFi 端 12-bit 通路合主线: 32 bit 像素 PL/CPU 与 CPU 逐字节一致, 2047 上跑通; V0 出口 ⑦ 达成 (7/8)。已知限制: 32 bit 只到 10.83 rps (16.15 rps 时完成率 82-91%)</t>
+          <t>用户定目标放宽: 亮起 ≤12.5 s / 找板 ≤21 s; V0 出口 ④ 达成</t>
         </is>
       </c>
       <c r="E128" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 3a41eb7</t>
+          <t>用户 10-14</t>
         </is>
       </c>
     </row>
@@ -11607,24 +11607,24 @@
       <c r="A129" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B129" s="6" t="inlineStr">
-        <is>
-          <t>开始</t>
+      <c r="B129" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C129" s="7" t="inlineStr">
         <is>
-          <t>KR7.2</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="D129" s="7" t="inlineStr">
         <is>
-          <t>8 h 无人值守长跑开跑 19:20 (假转黑屏, 主线 voxslice 0.6 + 卡上 PL 默认; 推 40 min/停 7 min 循环; 判据 S1-S9; 15 min 试跑 9/9)</t>
+          <t>无串口远程运维合主线: 升级坏包 (含断网包) 自动回滚后板子能按名字找回; 网络守护不再造成切片迟到 (旧版每分钟 2061 次 → 0); V0 出口 ⑤ 达成</t>
         </is>
       </c>
       <c r="E129" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 26e69ec soak8h</t>
+          <t>dr1v90 dee9be6</t>
         </is>
       </c>
     </row>
@@ -11632,24 +11632,24 @@
       <c r="A130" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B130" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B130" s="6" t="inlineStr">
+        <is>
+          <t>根因</t>
         </is>
       </c>
       <c r="C130" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D15b</t>
         </is>
       </c>
       <c r="D130" s="7" t="inlineStr">
         <is>
-          <t>用户批准 QoS 寄存器写入 + 网格 4×4 分块 (D16b 开做, 离线); 长跑后在 2047 做对照</t>
+          <t>32 bit PL 全黑: 板端写 LUT 基址仍用 16 bit 布局偏移, PL 把网格当角度表读; 已修 308d1bb, 待上板</t>
         </is>
       </c>
       <c r="E130" s="7" t="inlineStr">
         <is>
-          <t>用户 10-14</t>
+          <t>dr1v90 task/d15b-color-p2</t>
         </is>
       </c>
     </row>
@@ -11657,99 +11657,99 @@
       <c r="A131" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B131" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B131" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C131" s="7" t="inlineStr">
         <is>
-          <t>KR7.2</t>
+          <t>D15</t>
         </is>
       </c>
       <c r="D131" s="7" t="inlineStr">
         <is>
-          <t>长跑第 6 段企业 WiFi 踢线 ~5 s, 推流端 voxlive 不重连直接退出 (板端处理正确); 修: voxlive 断线自动重连 5cbe79f; 23:45 重开 8 h</t>
+          <t>WiFi 端 12-bit 通路合主线: 32 bit 像素 PL/CPU 与 CPU 逐字节一致, 2047 上跑通; V0 出口 ⑦ 达成 (7/8)。已知限制: 32 bit 只到 10.83 rps (16.15 rps 时完成率 82-91%)</t>
         </is>
       </c>
       <c r="E131" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 5cbe79f</t>
+          <t>dr1v90 3a41eb7</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="17" t="n">
-        <v>46308</v>
-      </c>
-      <c r="B132" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46309</v>
+      </c>
+      <c r="B132" s="6" t="inlineStr">
+        <is>
+          <t>开始</t>
         </is>
       </c>
       <c r="C132" s="7" t="inlineStr">
         <is>
-          <t>E6</t>
+          <t>KR7.2</t>
         </is>
       </c>
       <c r="D132" s="7" t="inlineStr">
         <is>
-          <t>按名字找板 (mDNS) 完成：无串口自重启后 34 s 按名字找到并 ssh 上</t>
+          <t>8 h 无人值守长跑开跑 19:20 (假转黑屏, 主线 voxslice 0.6 + 卡上 PL 默认; 推 40 min/停 7 min 循环; 判据 S1-S9; 15 min 试跑 9/9)</t>
         </is>
       </c>
       <c r="E132" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 b0f6b5d</t>
+          <t>dr1v90 26e69ec soak8h</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="17" t="n">
-        <v>46308</v>
-      </c>
-      <c r="B133" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46309</v>
+      </c>
+      <c r="B133" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C133" s="7" t="inlineStr">
         <is>
-          <t>E7</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D133" s="7" t="inlineStr">
         <is>
-          <t>纯切片 30 Hz 位流第一次上硅 D'0–D'3，尾部 late 0.2%，暂停 netguard 后 late/miss 为 0</t>
+          <t>用户批准 QoS 寄存器写入 + 网格 4×4 分块 (D16b 开做, 离线); 长跑后在 2047 做对照</t>
         </is>
       </c>
       <c r="E133" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 71d006f / 473abcf</t>
+          <t>用户 10-14</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="17" t="n">
-        <v>46308</v>
-      </c>
-      <c r="B134" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46309</v>
+      </c>
+      <c r="B134" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C134" s="7" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>KR7.2</t>
         </is>
       </c>
       <c r="D134" s="7" t="inlineStr">
         <is>
-          <t>主机实时推流完成：10 分钟 15.0 fps，NAK 0 / forced 0</t>
+          <t>长跑第 6 段企业 WiFi 踢线 ~5 s, 推流端 voxlive 不重连直接退出 (板端处理正确); 修: voxlive 断线自动重连 5cbe79f; 23:45 重开 8 h</t>
         </is>
       </c>
       <c r="E134" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 596b191</t>
+          <t>dr1v90 5cbe79f</t>
         </is>
       </c>
     </row>
@@ -11757,24 +11757,24 @@
       <c r="A135" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B135" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B135" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C135" s="7" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>E6</t>
         </is>
       </c>
       <c r="D135" s="7" t="inlineStr">
         <is>
-          <t>第一次上板端到端延迟 p50 114 ms 未过（停等发送），改发送流水线后降到 84.7 ms</t>
+          <t>按名字找板 (mDNS) 完成：无串口自重启后 34 s 按名字找到并 ssh 上</t>
         </is>
       </c>
       <c r="E135" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 60c619a / 596b191</t>
+          <t>dr1v90 b0f6b5d</t>
         </is>
       </c>
     </row>
@@ -11784,22 +11784,22 @@
       </c>
       <c r="B136" s="11" t="inlineStr">
         <is>
-          <t>复验通过</t>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C136" s="7" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>E7</t>
         </is>
       </c>
       <c r="D136" s="7" t="inlineStr">
         <is>
-          <t>主会话新克隆独立复验离线+上板全过，合主线（延迟 p50 95 ms / p99 236.6 ms）</t>
+          <t>纯切片 30 Hz 位流第一次上硅 D'0–D'3，尾部 late 0.2%，暂停 netguard 后 late/miss 为 0</t>
         </is>
       </c>
       <c r="E136" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 9bf16ad</t>
+          <t>dr1v90 71d006f / 473abcf</t>
         </is>
       </c>
     </row>
@@ -11807,24 +11807,24 @@
       <c r="A137" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B137" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B137" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C137" s="7" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="D137" s="7" t="inlineStr">
         <is>
-          <t>桥接收核对 12-bit 第一次复验 FAIL（新克隆无可执行位），退回</t>
+          <t>主机实时推流完成：10 分钟 15.0 fps，NAK 0 / forced 0</t>
         </is>
       </c>
       <c r="E137" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 596b191</t>
         </is>
       </c>
     </row>
@@ -11832,24 +11832,24 @@
       <c r="A138" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B138" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B138" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C138" s="7" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="D138" s="7" t="inlineStr">
         <is>
-          <t>桥接收核对 12-bit 复验 PASS，合主线</t>
+          <t>第一次上板端到端延迟 p50 114 ms 未过（停等发送），改发送流水线后降到 84.7 ms</t>
         </is>
       </c>
       <c r="E138" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 6a373d3</t>
+          <t>dr1v90 60c619a / 596b191</t>
         </is>
       </c>
     </row>
@@ -11864,17 +11864,17 @@
       </c>
       <c r="C139" s="7" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="D139" s="7" t="inlineStr">
         <is>
-          <t>桥驱动 2260 1 期 6 链 24 Hz 12-bit 复验 ALL PASS，合主线</t>
+          <t>主会话新克隆独立复验离线+上板全过，合主线（延迟 p50 95 ms / p99 236.6 ms）</t>
         </is>
       </c>
       <c r="E139" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 cdf49c6</t>
+          <t>dr1v90 9bf16ad</t>
         </is>
       </c>
     </row>
@@ -11882,19 +11882,19 @@
       <c r="A140" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B140" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B140" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C140" s="7" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="D140" s="7" t="inlineStr">
         <is>
-          <t>6 链 4296 片/s 能跑但余量仅 0.40%，瓶颈是桥→2260 链路；留 10% 需 ≤3921 片/s，待用户定</t>
+          <t>桥接收核对 12-bit 第一次复验 FAIL（新克隆无可执行位），退回</t>
         </is>
       </c>
       <c r="E140" s="7" t="inlineStr">
@@ -11907,24 +11907,24 @@
       <c r="A141" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B141" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B141" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C141" s="7" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="D141" s="7" t="inlineStr">
         <is>
-          <t>发现 10-10 验证板 profile 寄存器在 166.67 MHz 下超规格（GCLK 667&gt;600），1 期表已改</t>
+          <t>桥接收核对 12-bit 复验 PASS，合主线</t>
         </is>
       </c>
       <c r="E141" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 6a373d3</t>
         </is>
       </c>
     </row>
@@ -11939,17 +11939,17 @@
       </c>
       <c r="C142" s="7" t="inlineStr">
         <is>
-          <t>D6</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="D142" s="7" t="inlineStr">
         <is>
-          <t>几何 LUT 生成器逐字节复现 2047 s3lut，verify 22 PASS，合主线</t>
+          <t>桥驱动 2260 1 期 6 链 24 Hz 12-bit 复验 ALL PASS，合主线</t>
         </is>
       </c>
       <c r="E142" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 44ed2cd</t>
+          <t>dr1v90 cdf49c6</t>
         </is>
       </c>
     </row>
@@ -11957,19 +11957,19 @@
       <c r="A143" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B143" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B143" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C143" s="7" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="D143" s="7" t="inlineStr">
         <is>
-          <t>转子运维首次复验 T5 偶发 FAIL，退回返工</t>
+          <t>6 链 4296 片/s 能跑但余量仅 0.40%，瓶颈是桥→2260 链路；留 10% 需 ≤3921 片/s，待用户定</t>
         </is>
       </c>
       <c r="E143" s="7" t="inlineStr">
@@ -11982,24 +11982,24 @@
       <c r="A144" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B144" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B144" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C144" s="7" t="inlineStr">
         <is>
-          <t>D14</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="D144" s="7" t="inlineStr">
         <is>
-          <t>10 类内容 + 手机网页遥控离线复验 ALL PASS，用户实转看过（尚未正式上板验收）</t>
+          <t>发现 10-10 验证板 profile 寄存器在 166.67 MHz 下超规格（GCLK 667&gt;600），1 期表已改</t>
         </is>
       </c>
       <c r="E144" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 ffbfeeb</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12014,17 +12014,17 @@
       </c>
       <c r="C145" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D6</t>
         </is>
       </c>
       <c r="D145" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 切片离线复验 26/0，待上板（之后 9ba9af0 测试用例过时 26/27 待修）</t>
+          <t>几何 LUT 生成器逐字节复现 2047 s3lut，verify 22 PASS，合主线</t>
         </is>
       </c>
       <c r="E145" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 44ed2cd</t>
         </is>
       </c>
     </row>
@@ -12039,12 +12039,12 @@
       </c>
       <c r="C146" s="7" t="inlineStr">
         <is>
-          <t>D12</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="D146" s="7" t="inlineStr">
         <is>
-          <t>延迟降低上板复验 FAIL：B1 翻页 14.39&lt;15 fps，p99 225 ms，退回</t>
+          <t>转子运维首次复验 T5 偶发 FAIL，退回返工</t>
         </is>
       </c>
       <c r="E146" s="7" t="inlineStr">
@@ -12057,24 +12057,24 @@
       <c r="A147" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B147" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B147" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C147" s="7" t="inlineStr">
         <is>
-          <t>D12</t>
+          <t>D14</t>
         </is>
       </c>
       <c r="D147" s="7" t="inlineStr">
         <is>
-          <t>第二次上板仍未过，根因晚间 WiFi 尾巴（p99 334 vs 白天 48 ms）；判据改为调度问题 0 + 网络晚到 ≤1%，明早主机空闲复测</t>
+          <t>10 类内容 + 手机网页遥控离线复验 ALL PASS，用户实转看过（尚未正式上板验收）</t>
         </is>
       </c>
       <c r="E147" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 764f81d</t>
+          <t>dr1v90 ffbfeeb</t>
         </is>
       </c>
     </row>
@@ -12082,19 +12082,19 @@
       <c r="A148" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B148" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B148" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C148" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D148" s="7" t="inlineStr">
         <is>
-          <t>启动提速上板 FAIL 11 项，但改进已装板保留（6 次重启正常），退回继续压启动时间</t>
+          <t>2047 PL 切片离线复验 26/0，待上板（之后 9ba9af0 测试用例过时 26/27 待修）</t>
         </is>
       </c>
       <c r="E148" s="7" t="inlineStr">
@@ -12107,24 +12107,24 @@
       <c r="A149" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B149" s="19" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+      <c r="B149" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C149" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D12</t>
         </is>
       </c>
       <c r="D149" s="7" t="inlineStr">
         <is>
-          <t>启动提速两轮后：复位→0° 片亮起 38.7→20.1→15.8 s，找板 34→30→25.6 s</t>
+          <t>延迟降低上板复验 FAIL：B1 翻页 14.39&lt;15 fps，p99 225 ms，退回</t>
         </is>
       </c>
       <c r="E149" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d13-boot fdbb217</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12139,17 +12139,17 @@
       </c>
       <c r="C150" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D12</t>
         </is>
       </c>
       <c r="D150" s="7" t="inlineStr">
         <is>
-          <t>第二步（bootdelay 0 / 精简 uInitrd）写启动文件被权限系统拒绝，需用户明早本人批准后执行</t>
+          <t>第二次上板仍未过，根因晚间 WiFi 尾巴（p99 334 vs 白天 48 ms）；判据改为调度问题 0 + 网络晚到 ≤1%，明早主机空闲复测</t>
         </is>
       </c>
       <c r="E150" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 764f81d</t>
         </is>
       </c>
     </row>
@@ -12157,24 +12157,24 @@
       <c r="A151" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B151" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B151" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C151" s="7" t="inlineStr">
         <is>
-          <t>D15</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D151" s="7" t="inlineStr">
         <is>
-          <t>WiFi 端 32 bit 像素（X2R10G10B10）阶段 1 复验：黄金/PL 仿真一致，合主线</t>
+          <t>启动提速上板 FAIL 11 项，但改进已装板保留（6 次重启正常），退回继续压启动时间</t>
         </is>
       </c>
       <c r="E151" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 1995be8</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12182,24 +12182,24 @@
       <c r="A152" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B152" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B152" s="19" t="inlineStr">
+        <is>
+          <t>里程碑</t>
         </is>
       </c>
       <c r="C152" s="7" t="inlineStr">
         <is>
-          <t>D3;D4;D5</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D152" s="7" t="inlineStr">
         <is>
-          <t>下午用户：2260 相关先暂停、先做共用部分（token 不够）；15:00 又改为多开并行恢复 2260</t>
+          <t>启动提速两轮后：复位→0° 片亮起 38.7→20.1→15.8 s，找板 34→30→25.6 s</t>
         </is>
       </c>
       <c r="E152" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 task/d13-boot fdbb217</t>
         </is>
       </c>
     </row>
@@ -12207,20 +12207,24 @@
       <c r="A153" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B153" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
-        </is>
-      </c>
-      <c r="C153" s="7" t="inlineStr"/>
+      <c r="B153" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
+        </is>
+      </c>
+      <c r="C153" s="7" t="inlineStr">
+        <is>
+          <t>D13</t>
+        </is>
+      </c>
       <c r="D153" s="7" t="inlineStr">
         <is>
-          <t>软件三期：0 期 2047 屏（现在）/ 1 期 2260 验证板 160×180（预计 11-10 回板）/ 2 期 192×216 目标板；1 期目标 24 Hz / 358 片 / 6 链</t>
+          <t>第二步（bootdelay 0 / 精简 uInitrd）写启动文件被权限系统拒绝，需用户明早本人批准后执行</t>
         </is>
       </c>
       <c r="E153" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_sw_three_phases_1013.md</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12228,20 +12232,24 @@
       <c r="A154" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B154" s="19" t="inlineStr">
-        <is>
-          <t>里程碑</t>
-        </is>
-      </c>
-      <c r="C154" s="7" t="inlineStr"/>
+      <c r="B154" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
+        </is>
+      </c>
+      <c r="C154" s="7" t="inlineStr">
+        <is>
+          <t>D15</t>
+        </is>
+      </c>
       <c r="D154" s="7" t="inlineStr">
         <is>
-          <t>硬件 1 期验证板预计 2026-11-10 回板（初步交期，可能变），回板前软件能做的都前置</t>
+          <t>WiFi 端 32 bit 像素（X2R10G10B10）阶段 1 复验：黄金/PL 仿真一致，合主线</t>
         </is>
       </c>
       <c r="E154" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_sw_three_phases_1013.md</t>
+          <t>dr1v90 1995be8</t>
         </is>
       </c>
     </row>
@@ -12254,15 +12262,19 @@
           <t>决定</t>
         </is>
       </c>
-      <c r="C155" s="7" t="inlineStr"/>
+      <c r="C155" s="7" t="inlineStr">
+        <is>
+          <t>D3;D4;D5</t>
+        </is>
+      </c>
       <c r="D155" s="7" t="inlineStr">
         <is>
-          <t>架构切分：PL 切片器及之前为各期共用的公共部分，屏幕显示为可替换后端，两者之间用实时按角度片流接口</t>
+          <t>下午用户：2260 相关先暂停、先做共用部分（token 不够）；15:00 又改为多开并行恢复 2260</t>
         </is>
       </c>
       <c r="E155" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_arch_common_front_display_backend.md</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12275,19 +12287,15 @@
           <t>决定</t>
         </is>
       </c>
-      <c r="C156" s="7" t="inlineStr">
-        <is>
-          <t>D3</t>
-        </is>
-      </c>
+      <c r="C156" s="7" t="inlineStr"/>
       <c r="D156" s="7" t="inlineStr">
         <is>
-          <t>用户定：2 期上行 1.2G；1 期保持 24 Hz（358 片，桥链路余量 0.40%）不降档</t>
+          <t>软件三期：0 期 2047 屏（现在）/ 1 期 2260 验证板 160×180（预计 11-10 回板）/ 2 期 192×216 目标板；1 期目标 24 Hz / 358 片 / 6 链</t>
         </is>
       </c>
       <c r="E156" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>claude_memory/project_sw_three_phases_1013.md</t>
         </is>
       </c>
     </row>
@@ -12295,24 +12303,20 @@
       <c r="A157" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B157" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
-        </is>
-      </c>
-      <c r="C157" s="7" t="inlineStr">
-        <is>
-          <t>D11</t>
-        </is>
-      </c>
+      <c r="B157" s="19" t="inlineStr">
+        <is>
+          <t>里程碑</t>
+        </is>
+      </c>
+      <c r="C157" s="7" t="inlineStr"/>
       <c r="D157" s="7" t="inlineStr">
         <is>
-          <t>傍晚用户：杜邦线跑不了 1.2G，1.2G 实测等 V1 回板；C1 台架只做 ≤300M 低速功能档</t>
+          <t>硬件 1 期验证板预计 2026-11-10 回板（初步交期，可能变），回板前软件能做的都前置</t>
         </is>
       </c>
       <c r="E157" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>claude_memory/project_sw_three_phases_1013.md</t>
         </is>
       </c>
     </row>
@@ -12325,19 +12329,15 @@
           <t>决定</t>
         </is>
       </c>
-      <c r="C158" s="7" t="inlineStr">
-        <is>
-          <t>D12;D13;D14</t>
-        </is>
-      </c>
+      <c r="C158" s="7" t="inlineStr"/>
       <c r="D158" s="7" t="inlineStr">
         <is>
-          <t>19:00 用户：V0 可见的先插队、V1 接着做，新派 D12 延迟降低 / D13 启动提速 / D14 内容与手机控制</t>
+          <t>架构切分：PL 切片器及之前为各期共用的公共部分，屏幕显示为可替换后端，两者之间用实时按角度片流接口</t>
         </is>
       </c>
       <c r="E158" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>claude_memory/project_arch_common_front_display_backend.md</t>
         </is>
       </c>
     </row>
@@ -12352,12 +12352,12 @@
       </c>
       <c r="C159" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="D159" s="7" t="inlineStr">
         <is>
-          <t>21:10 用户定 D13 目标：复位到 0° 片亮起 ≤12 s，找板 ≤20 s（看板 KR8.1 已改）</t>
+          <t>用户定：2 期上行 1.2G；1 期保持 24 Hz（358 片，桥链路余量 0.40%）不降档</t>
         </is>
       </c>
       <c r="E159" s="7" t="inlineStr">
@@ -12377,12 +12377,12 @@
       </c>
       <c r="C160" s="7" t="inlineStr">
         <is>
-          <t>D15;D16</t>
+          <t>D11</t>
         </is>
       </c>
       <c r="D160" s="7" t="inlineStr">
         <is>
-          <t>用户选 12-bit 方案 A：WiFi 端传高位宽、像素位宽 16/32 bit 可配（D15）；DDR 做到极限 A 线（D16），B 线并入 T2 硬件</t>
+          <t>傍晚用户：杜邦线跑不了 1.2G，1.2G 实测等 V1 回板；C1 台架只做 ≤300M 低速功能档</t>
         </is>
       </c>
       <c r="E160" s="7" t="inlineStr">
@@ -12402,17 +12402,17 @@
       </c>
       <c r="C161" s="7" t="inlineStr">
         <is>
-          <t>KR5.2</t>
+          <t>D12;D13;D14</t>
         </is>
       </c>
       <c r="D161" s="7" t="inlineStr">
         <is>
-          <t>用户实转核实：2047 旧表镜像，已更正为新表 0decad54</t>
+          <t>19:00 用户：V0 可见的先插队、V1 接着做，新派 D12 延迟降低 / D13 启动提速 / D14 内容与手机控制</t>
         </is>
       </c>
       <c r="E161" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 49031f6</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12420,19 +12420,19 @@
       <c r="A162" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B162" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B162" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C162" s="7" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D162" s="7" t="inlineStr">
         <is>
-          <t>D7 上板补测会装/还原 autorun，冲掉 D13 补丁，须排在 D13 定稿合并之后；夜间板子排程 D12→D13→D2→D7→8 h 长跑</t>
+          <t>21:10 用户定 D13 目标：复位到 0° 片亮起 ≤12 s，找板 ≤20 s（看板 KR8.1 已改）</t>
         </is>
       </c>
       <c r="E162" s="7" t="inlineStr">
@@ -12445,18 +12445,93 @@
       <c r="A163" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B163" s="19" t="inlineStr">
+      <c r="B163" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
+        </is>
+      </c>
+      <c r="C163" s="7" t="inlineStr">
+        <is>
+          <t>D15;D16</t>
+        </is>
+      </c>
+      <c r="D163" s="7" t="inlineStr">
+        <is>
+          <t>用户选 12-bit 方案 A：WiFi 端传高位宽、像素位宽 16/32 bit 可配（D15）；DDR 做到极限 A 线（D16），B 线并入 T2 硬件</t>
+        </is>
+      </c>
+      <c r="E163" s="7" t="inlineStr">
+        <is>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B164" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
+        </is>
+      </c>
+      <c r="C164" s="7" t="inlineStr">
+        <is>
+          <t>KR5.2</t>
+        </is>
+      </c>
+      <c r="D164" s="7" t="inlineStr">
+        <is>
+          <t>用户实转核实：2047 旧表镜像，已更正为新表 0decad54</t>
+        </is>
+      </c>
+      <c r="E164" s="7" t="inlineStr">
+        <is>
+          <t>dr1v90 49031f6</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B165" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
+        </is>
+      </c>
+      <c r="C165" s="7" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="D165" s="7" t="inlineStr">
+        <is>
+          <t>D7 上板补测会装/还原 autorun，冲掉 D13 补丁，须排在 D13 定稿合并之后；夜间板子排程 D12→D13→D2→D7→8 h 长跑</t>
+        </is>
+      </c>
+      <c r="E165" s="7" t="inlineStr">
+        <is>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B166" s="19" t="inlineStr">
         <is>
           <t>里程碑</t>
         </is>
       </c>
-      <c r="C163" s="7" t="inlineStr"/>
-      <c r="D163" s="7" t="inlineStr">
+      <c r="C166" s="7" t="inlineStr"/>
+      <c r="D166" s="7" t="inlineStr">
         <is>
           <t>显性目的进度看板第一版建立：10 个显性目的 + KR 趋势 + 燃起图 + 里程碑趋势</t>
         </is>
       </c>
-      <c r="E163" s="7" t="inlineStr">
+      <c r="E166" s="7" t="inlineStr">
         <is>
           <t>claude_memory/project_progress_dashboard.md</t>
         </is>
@@ -17169,7 +17244,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H61"/>
+  <dimension ref="A1:H65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -17213,7 +17288,7 @@
         <v>46307</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C4" s="6" t="n">
         <v>5</v>
@@ -17227,7 +17302,7 @@
         <v>46308</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C5" s="6" t="n">
         <v>7</v>
@@ -17241,7 +17316,7 @@
         <v>46309</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C6" s="6" t="n">
         <v>8</v>
@@ -17255,7 +17330,7 @@
         <v>46310</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>12</v>
@@ -17269,13 +17344,13 @@
         <v>46311</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C8" s="6" t="n">
         <v>20</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="9">
@@ -17283,10 +17358,10 @@
         <v>46312</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D9" s="6" t="n"/>
     </row>
@@ -17295,10 +17370,10 @@
         <v>46313</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D10" s="6" t="n"/>
     </row>
@@ -17307,10 +17382,10 @@
         <v>46314</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D11" s="6" t="n"/>
     </row>
@@ -17319,10 +17394,10 @@
         <v>46315</v>
       </c>
       <c r="B12" s="6" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="D12" s="6" t="n"/>
     </row>
@@ -17331,10 +17406,10 @@
         <v>46316</v>
       </c>
       <c r="B13" s="6" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C13" s="6" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="D13" s="6" t="n"/>
     </row>
@@ -17343,10 +17418,10 @@
         <v>46317</v>
       </c>
       <c r="B14" s="6" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C14" s="6" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="D14" s="6" t="n"/>
     </row>
@@ -17355,10 +17430,10 @@
         <v>46318</v>
       </c>
       <c r="B15" s="6" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="D15" s="6" t="n"/>
     </row>
@@ -17367,10 +17442,10 @@
         <v>46319</v>
       </c>
       <c r="B16" s="6" t="n">
+        <v>41</v>
+      </c>
+      <c r="C16" s="6" t="n">
         <v>37</v>
-      </c>
-      <c r="C16" s="6" t="n">
-        <v>33</v>
       </c>
       <c r="D16" s="6" t="n"/>
     </row>
@@ -18808,6 +18883,152 @@
       <c r="H61" s="7" t="inlineStr">
         <is>
           <t>合主线 90b1d79; 不改 RTL; 桥余量各档 ≥2.7%; 离线+RTL 仿真 24/0</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>D26</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>V2 主控位流跟上主线 (p2_ul1200_b12_v3)</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D62" s="6" t="inlineStr">
+        <is>
+          <t>公共</t>
+        </is>
+      </c>
+      <c r="E62" s="17" t="n">
+        <v>46312</v>
+      </c>
+      <c r="F62" s="17" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G62" s="11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H62" s="7" t="inlineStr">
+        <is>
+          <t>合主线 c8e8294; SWNS 0.000 HWNS 0.001 (无裕量); bin a333a82d</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="inlineStr">
+        <is>
+          <t>D27</t>
+        </is>
+      </c>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>SoC↔桥通信全功能 (配置/状态/错误恢复/升级)</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="D63" s="6" t="inlineStr">
+        <is>
+          <t>公共</t>
+        </is>
+      </c>
+      <c r="E63" s="17" t="n">
+        <v>46315</v>
+      </c>
+      <c r="F63" s="17" t="n"/>
+      <c r="G63" s="15" t="inlineStr">
+        <is>
+          <t>🔄</t>
+        </is>
+      </c>
+      <c r="H63" s="7" t="inlineStr">
+        <is>
+          <t>task/d27-link (agent 进行中)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="inlineStr">
+        <is>
+          <t>D28</t>
+        </is>
+      </c>
+      <c r="B64" s="7" t="inlineStr">
+        <is>
+          <t>V1 回板当天一键 bring-up 脚本</t>
+        </is>
+      </c>
+      <c r="C64" s="6" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D64" s="6" t="inlineStr">
+        <is>
+          <t>公共</t>
+        </is>
+      </c>
+      <c r="E64" s="17" t="n">
+        <v>46315</v>
+      </c>
+      <c r="F64" s="17" t="n"/>
+      <c r="G64" s="15" t="inlineStr">
+        <is>
+          <t>🔄</t>
+        </is>
+      </c>
+      <c r="H64" s="7" t="inlineStr">
+        <is>
+          <t>task/d28-bringup (agent 进行中)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="inlineStr">
+        <is>
+          <t>D29</t>
+        </is>
+      </c>
+      <c r="B65" s="7" t="inlineStr">
+        <is>
+          <t>冷启动认不到 TF 卡 (03 停在 u-boot)</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D65" s="6" t="inlineStr">
+        <is>
+          <t>公共</t>
+        </is>
+      </c>
+      <c r="E65" s="17" t="n">
+        <v>46315</v>
+      </c>
+      <c r="F65" s="17" t="n"/>
+      <c r="G65" s="15" t="inlineStr">
+        <is>
+          <t>🔄</t>
+        </is>
+      </c>
+      <c r="H65" s="7" t="inlineStr">
+        <is>
+          <t>task/d29-sdboot (agent 进行中); 改 u-boot 读的文件需用户批准</t>
         </is>
       </c>
     </row>

</xml_diff>